<commit_message>
SPC-700 instructions up to 09.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4979F2C-0057-418F-A13C-26F8577DC452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FD401A-EC92-4F3E-AA71-882231C08B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11235" yWindow="630" windowWidth="16575" windowHeight="14745" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
+    <workbookView xWindow="11235" yWindow="0" windowWidth="16575" windowHeight="15600" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$177</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$590</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="71">
   <si>
     <t>Implied</t>
   </si>
@@ -50,6 +50,9 @@
     <t>R/W</t>
   </si>
   <si>
+    <t>Cycles: 6</t>
+  </si>
+  <si>
     <t>Size: 2</t>
   </si>
   <si>
@@ -68,12 +71,27 @@
     <t>Cycles: 8</t>
   </si>
   <si>
+    <t>Cycles: 3</t>
+  </si>
+  <si>
     <t>Cycles: 2</t>
   </si>
   <si>
     <t>Cycles: 4</t>
   </si>
   <si>
+    <t>Store as Address.L.</t>
+  </si>
+  <si>
+    <t>Absolute (Read)</t>
+  </si>
+  <si>
+    <t>Size: 3</t>
+  </si>
+  <si>
+    <t>Immediate</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Push </t>
     </r>
@@ -126,6 +144,9 @@
     </r>
   </si>
   <si>
+    <t>Store as Pointer.H.</t>
+  </si>
+  <si>
     <t xml:space="preserve"> +X.1</t>
   </si>
   <si>
@@ -164,6 +185,12 @@
     </r>
   </si>
   <si>
+    <t>Store as Address.H.</t>
+  </si>
+  <si>
+    <t>Read Pointer</t>
+  </si>
+  <si>
     <t>NOP (00)</t>
   </si>
   <si>
@@ -400,6 +427,631 @@
   </si>
   <si>
     <t>Direct Page Bit (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <t>BBS (03)</t>
+  </si>
+  <si>
+    <t>Direct Page Bit Relative</t>
+  </si>
+  <si>
+    <t>Set Jump to (Operand &amp; (1 &lt;&lt; 0)) == (1 &lt;&lt; 0).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. If !Jump, end instruction (next half-cycle is 7.2).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Address = (Operand | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SPW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Address = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + int8( Operand ).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L = Address.L.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.H = Address.H.</t>
+    </r>
+  </si>
+  <si>
+    <t>Cycles: 5-7</t>
+  </si>
+  <si>
+    <t>OR (04)</t>
+  </si>
+  <si>
+    <t>Direct Page (Read)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> |= Operand.  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (05)</t>
+  </si>
+  <si>
+    <t>OR (06)</t>
+  </si>
+  <si>
+    <t>Indirect X (Read)</t>
+  </si>
+  <si>
+    <r>
+      <t>Read (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SPW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3))</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (07)</t>
+  </si>
+  <si>
+    <t>X-Indexed Indirect (Read)</t>
+  </si>
+  <si>
+    <t>Store as Pointer.L.</t>
+  </si>
+  <si>
+    <r>
+      <t>Read ((Address + 1) &amp; $FF) | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SPW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag) &lt;&lt; 3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Address = ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + Operand) &amp; $FF) | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SPW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3).</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (08)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> |= Operand.  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (09)</t>
+  </si>
+  <si>
+    <t>Store as Operand0.</t>
+  </si>
+  <si>
+    <t>Store as Operand1.</t>
+  </si>
+  <si>
+    <t>Write Operand0.</t>
+  </si>
+  <si>
+    <t>Direct Page to Direct Page (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Operand0 |= Operand1.  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand0 &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !Operand0.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -565,7 +1217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -615,6 +1267,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -622,6 +1280,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -958,25 +1619,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C548"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="17" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" style="17" customWidth="1"/>
-    <col min="3" max="3" width="92.28515625" style="17" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" style="19" customWidth="1"/>
+    <col min="3" max="3" width="92.28515625" style="19" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
     <col min="6" max="7" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -994,18 +1655,18 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1014,7 +1675,7 @@
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1036,28 +1697,28 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="8"/>
     </row>
     <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B60" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="12" t="s">
         <v>8</v>
-      </c>
-      <c r="C60" s="12" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1075,18 +1736,18 @@
         <v>2</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1095,7 +1756,7 @@
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1103,10 +1764,10 @@
         <v>1.2</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1135,10 +1796,10 @@
         <v>3.2</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1153,10 +1814,10 @@
         <v>4.2</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1165,7 +1826,7 @@
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="2" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1187,10 +1848,10 @@
         <v>6.2</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1205,10 +1866,10 @@
         <v>7.2</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1223,36 +1884,36 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B80" s="9"/>
       <c r="C80" s="8"/>
     </row>
     <row r="119" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C119" s="12" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
-      <c r="B120" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C120" s="19"/>
+      <c r="B120" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C120" s="21"/>
     </row>
     <row r="121" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
@@ -1262,18 +1923,18 @@
         <v>2</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C122" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1282,7 +1943,7 @@
       </c>
       <c r="B123" s="7"/>
       <c r="C123" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1290,10 +1951,10 @@
         <v>1.2</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1302,7 +1963,7 @@
       </c>
       <c r="B125" s="7"/>
       <c r="C125" s="2" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1310,30 +1971,30 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B126" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
         <v>3.1</v>
       </c>
-      <c r="B127" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C127" s="2"/>
+      <c r="B127" s="7"/>
+      <c r="C127" s="7" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="128" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
         <v>3.2</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1348,22 +2009,954 @@
         <v>4.2</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B131" s="9"/>
       <c r="C131" s="8"/>
     </row>
+    <row r="178" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B178" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C178" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="13"/>
+      <c r="B179" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C179" s="21"/>
+    </row>
+    <row r="180" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B180" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C180" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C181" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B182" s="7"/>
+      <c r="C182" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B183" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C183" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B184" s="7"/>
+      <c r="C184" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B185" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C185" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B186" s="7"/>
+      <c r="C186" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B187" s="7"/>
+      <c r="C187" s="2"/>
+    </row>
+    <row r="188" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B188" s="7"/>
+      <c r="C188" s="2"/>
+    </row>
+    <row r="189" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B189" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C189" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B190" s="7"/>
+      <c r="C190" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B191" s="7"/>
+      <c r="C191" s="2"/>
+    </row>
+    <row r="192" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B192" s="7"/>
+      <c r="C192" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="3"/>
+      <c r="B193" s="7"/>
+      <c r="C193" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B194" s="7"/>
+      <c r="C194" s="2"/>
+    </row>
+    <row r="195" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B195" s="7"/>
+      <c r="C195" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B196" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C196" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B197" s="9"/>
+      <c r="C197" s="8"/>
+    </row>
+    <row r="237" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A237" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B237" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C237" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A238" s="13"/>
+      <c r="B238" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C238" s="18"/>
+    </row>
+    <row r="239" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A239" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C239" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A240" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B240" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C240" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A241" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B241" s="7"/>
+      <c r="C241" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A242" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B242" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C242" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A243" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B243" s="7"/>
+      <c r="C243" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A244" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B244" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C244" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A245" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B245" s="7"/>
+      <c r="C245" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A246" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B246" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C246" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A247" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B247" s="9"/>
+      <c r="C247" s="8"/>
+    </row>
+    <row r="296" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A296" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B296" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C296" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A297" s="13"/>
+      <c r="B297" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C297" s="18"/>
+    </row>
+    <row r="298" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A298" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C298" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A299" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B299" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C299" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A300" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B300" s="7"/>
+      <c r="C300" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A301" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B301" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C301" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A302" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B302" s="7"/>
+      <c r="C302" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A303" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B303" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C303" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A304" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B304" s="7"/>
+      <c r="C304" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A305" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B305" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C305" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A306" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B306" s="7"/>
+      <c r="C306" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A307" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B307" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C307" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A308" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B308" s="9"/>
+      <c r="C308" s="8"/>
+    </row>
+    <row r="355" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A355" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B355" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C355" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A356" s="13"/>
+      <c r="B356" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C356" s="18"/>
+    </row>
+    <row r="357" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A357" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B357" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C357" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A358" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B358" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C358" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A359" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B359" s="7"/>
+      <c r="C359" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A360" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B360" s="7"/>
+      <c r="C360" s="2"/>
+    </row>
+    <row r="361" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A361" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B361" s="7"/>
+      <c r="C361" s="2"/>
+    </row>
+    <row r="362" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A362" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B362" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C362" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A363" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B363" s="7"/>
+      <c r="C363" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A364" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B364" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C364" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A365" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B365" s="9"/>
+      <c r="C365" s="8"/>
+    </row>
+    <row r="414" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A414" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B414" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C414" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A415" s="13"/>
+      <c r="B415" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C415" s="18"/>
+    </row>
+    <row r="416" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A416" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B416" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C416" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="417" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A417" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B417" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C417" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="418" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A418" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B418" s="7"/>
+      <c r="C418" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="419" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A419" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B419" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C419" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A420" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B420" s="7"/>
+      <c r="C420" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A421" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B421" s="7"/>
+      <c r="C421" s="2"/>
+    </row>
+    <row r="422" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A422" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B422" s="7"/>
+      <c r="C422" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="423" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A423" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B423" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C423" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A424" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B424" s="7"/>
+      <c r="C424" s="2"/>
+    </row>
+    <row r="425" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A425" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B425" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C425" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A426" s="3"/>
+      <c r="B426" s="22"/>
+      <c r="C426" s="2"/>
+    </row>
+    <row r="427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A427" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B427" s="7"/>
+      <c r="C427" s="2"/>
+    </row>
+    <row r="428" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A428" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B428" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C428" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="429" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A429" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B429" s="7"/>
+      <c r="C429" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A430" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B430" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C430" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="431" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A431" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B431" s="9"/>
+      <c r="C431" s="8"/>
+    </row>
+    <row r="473" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A473" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B473" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C473" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="474" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A474" s="13"/>
+      <c r="B474" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C474" s="18"/>
+    </row>
+    <row r="475" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A475" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B475" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C475" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="476" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A476" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B476" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C476" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="477" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A477" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B477" s="7"/>
+      <c r="C477" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="478" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A478" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B478" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C478" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="479" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A479" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B479" s="7"/>
+      <c r="C479" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A480" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B480" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C480" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="481" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A481" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B481" s="9"/>
+      <c r="C481" s="8"/>
+    </row>
+    <row r="532" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A532" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B532" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C532" s="12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A533" s="13"/>
+      <c r="B533" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C533" s="21"/>
+    </row>
+    <row r="534" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A534" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B534" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C534" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="535" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A535" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B535" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C535" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="536" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A536" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B536" s="7"/>
+      <c r="C536" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="537" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A537" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B537" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C537" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="538" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A538" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B538" s="7"/>
+      <c r="C538" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A539" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B539" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C539" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A540" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B540" s="7"/>
+      <c r="C540" s="2"/>
+    </row>
+    <row r="541" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A541" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B541" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C541" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="542" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A542" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B542" s="7"/>
+      <c r="C542" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="543" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A543" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B543" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C543" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A544" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B544" s="7"/>
+      <c r="C544" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A545" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B545" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C545" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A546" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B546" s="7"/>
+      <c r="C546" s="2"/>
+    </row>
+    <row r="547" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A547" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B547" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C547" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A548" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B548" s="9"/>
+      <c r="C548" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="B120:C120"/>
+    <mergeCell ref="B179:C179"/>
+    <mergeCell ref="B425:B426"/>
+    <mergeCell ref="B533:C533"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup scale="79" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
SPC-700 instructions up to 0B.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FD401A-EC92-4F3E-AA71-882231C08B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF57CCB6-E034-4B07-8030-87F4F3897370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11235" yWindow="0" windowWidth="16575" windowHeight="15600" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$590</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$687</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="80">
   <si>
     <t>Implied</t>
   </si>
@@ -74,6 +74,9 @@
     <t>Cycles: 3</t>
   </si>
   <si>
+    <t>Cycles: 5</t>
+  </si>
+  <si>
     <t>Cycles: 2</t>
   </si>
   <si>
@@ -592,6 +595,218 @@
     <t>Direct Page (Read)</t>
   </si>
   <si>
+    <t>OR (05)</t>
+  </si>
+  <si>
+    <t>OR (06)</t>
+  </si>
+  <si>
+    <t>Indirect X (Read)</t>
+  </si>
+  <si>
+    <r>
+      <t>Read (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SPW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3))</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (07)</t>
+  </si>
+  <si>
+    <t>X-Indexed Indirect (Read)</t>
+  </si>
+  <si>
+    <t>Store as Pointer.L.</t>
+  </si>
+  <si>
+    <r>
+      <t>Read ((Address + 1) &amp; $FF) | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SPW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag) &lt;&lt; 3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Address = ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + Operand) &amp; $FF) | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SPW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3).</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (08)</t>
+  </si>
+  <si>
+    <t>OR (09)</t>
+  </si>
+  <si>
+    <t>Store as Operand0.</t>
+  </si>
+  <si>
+    <t>Store as Operand1.</t>
+  </si>
+  <si>
+    <t>Write Operand0.</t>
+  </si>
+  <si>
+    <t>Direct Page to Direct Page (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <t>OR1 (0A)</t>
+  </si>
+  <si>
+    <t>Absolute Boolean Bit</t>
+  </si>
+  <si>
+    <t>Read (Address &amp; $1FFF)</t>
+  </si>
+  <si>
+    <t>Bit = Address &gt;&gt; 13.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag |= ((Operand &amp; (1 &lt;&lt; Bit)) != 0).</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -611,7 +826,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> |= Operand.  </t>
+      <t xml:space="preserve"> |= Operand. </t>
     </r>
     <r>
       <rPr>
@@ -699,168 +914,6 @@
     </r>
   </si>
   <si>
-    <t>OR (05)</t>
-  </si>
-  <si>
-    <t>OR (06)</t>
-  </si>
-  <si>
-    <t>Indirect X (Read)</t>
-  </si>
-  <si>
-    <r>
-      <t>Read (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>X</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> | ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SPW</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3))</t>
-    </r>
-  </si>
-  <si>
-    <t>OR (07)</t>
-  </si>
-  <si>
-    <t>X-Indexed Indirect (Read)</t>
-  </si>
-  <si>
-    <t>Store as Pointer.L.</t>
-  </si>
-  <si>
-    <r>
-      <t>Read ((Address + 1) &amp; $FF) | ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SPW</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>P</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag) &lt;&lt; 3)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Address = ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>X</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> + Operand) &amp; $FF) | ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SPW</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3).</t>
-    </r>
-  </si>
-  <si>
-    <t>OR (08)</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Inc. </t>
     </r>
@@ -904,7 +957,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> |= Operand.  </t>
+      <t xml:space="preserve"> |= Operand. </t>
     </r>
     <r>
       <rPr>
@@ -992,23 +1045,8 @@
     </r>
   </si>
   <si>
-    <t>OR (09)</t>
-  </si>
-  <si>
-    <t>Store as Operand0.</t>
-  </si>
-  <si>
-    <t>Store as Operand1.</t>
-  </si>
-  <si>
-    <t>Write Operand0.</t>
-  </si>
-  <si>
-    <t>Direct Page to Direct Page (Read/Modify/Write)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Operand0 |= Operand1.  </t>
+    <r>
+      <t xml:space="preserve">Operand0 |= Operand1. </t>
     </r>
     <r>
       <rPr>
@@ -1051,6 +1089,77 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> flag = !Operand0.</t>
+    </r>
+  </si>
+  <si>
+    <t>ASL (0B)</t>
+  </si>
+  <si>
+    <t>Direct Page (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand &amp; $80). Operand &lt;&lt;= 1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !Operand.</t>
     </r>
   </si>
 </sst>
@@ -1619,7 +1728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C548"/>
+  <dimension ref="A1:C662"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -1631,10 +1740,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>8</v>
@@ -1655,15 +1764,15 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -1675,7 +1784,7 @@
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1697,7 +1806,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>5</v>
@@ -1705,14 +1814,14 @@
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="8"/>
     </row>
     <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>9</v>
@@ -1736,15 +1845,15 @@
         <v>2</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>5</v>
@@ -1756,7 +1865,7 @@
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1764,7 +1873,7 @@
         <v>1.2</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>6</v>
@@ -1796,10 +1905,10 @@
         <v>3.2</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1814,10 +1923,10 @@
         <v>4.2</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1826,7 +1935,7 @@
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1848,10 +1957,10 @@
         <v>6.2</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1866,10 +1975,10 @@
         <v>7.2</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1884,7 +1993,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>5</v>
@@ -1892,17 +2001,17 @@
     </row>
     <row r="80" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B80" s="9"/>
       <c r="C80" s="8"/>
     </row>
     <row r="119" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C119" s="12" t="s">
         <v>4</v>
@@ -1911,7 +2020,7 @@
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
       <c r="B120" s="20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C120" s="21"/>
     </row>
@@ -1923,15 +2032,15 @@
         <v>2</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C122" t="s">
         <v>5</v>
@@ -1943,7 +2052,7 @@
       </c>
       <c r="B123" s="7"/>
       <c r="C123" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1951,7 +2060,7 @@
         <v>1.2</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>6</v>
@@ -1963,7 +2072,7 @@
       </c>
       <c r="B125" s="7"/>
       <c r="C125" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1983,7 +2092,7 @@
       </c>
       <c r="B127" s="7"/>
       <c r="C127" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1991,10 +2100,10 @@
         <v>3.2</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2009,7 +2118,7 @@
         <v>4.2</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>5</v>
@@ -2017,26 +2126,26 @@
     </row>
     <row r="131" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B131" s="9"/>
       <c r="C131" s="8"/>
     </row>
     <row r="178" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B178" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C178" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="13"/>
       <c r="B179" s="20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C179" s="21"/>
     </row>
@@ -2048,15 +2157,15 @@
         <v>2</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="181" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C181" t="s">
         <v>5</v>
@@ -2068,7 +2177,7 @@
       </c>
       <c r="B182" s="7"/>
       <c r="C182" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2076,7 +2185,7 @@
         <v>1.2</v>
       </c>
       <c r="B183" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C183" s="2" t="s">
         <v>6</v>
@@ -2088,7 +2197,7 @@
       </c>
       <c r="B184" s="7"/>
       <c r="C184" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2108,7 +2217,7 @@
       </c>
       <c r="B186" s="7"/>
       <c r="C186" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="187" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2130,7 +2239,7 @@
         <v>4.2</v>
       </c>
       <c r="B189" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>6</v>
@@ -2142,7 +2251,7 @@
       </c>
       <c r="B190" s="7"/>
       <c r="C190" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2158,14 +2267,14 @@
       </c>
       <c r="B192" s="7"/>
       <c r="C192" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="3"/>
       <c r="B193" s="7"/>
       <c r="C193" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2181,7 +2290,7 @@
       </c>
       <c r="B195" s="7"/>
       <c r="C195" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2189,7 +2298,7 @@
         <v>7.2</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>5</v>
@@ -2197,14 +2306,14 @@
     </row>
     <row r="197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B197" s="9"/>
       <c r="C197" s="8"/>
     </row>
     <row r="237" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B237" s="11" t="s">
         <v>10</v>
@@ -2216,7 +2325,7 @@
     <row r="238" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="13"/>
       <c r="B238" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C238" s="18"/>
     </row>
@@ -2228,15 +2337,15 @@
         <v>2</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="240" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C240" t="s">
         <v>5</v>
@@ -2248,7 +2357,7 @@
       </c>
       <c r="B241" s="7"/>
       <c r="C241" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="242" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2256,7 +2365,7 @@
         <v>1.2</v>
       </c>
       <c r="B242" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>6</v>
@@ -2268,7 +2377,7 @@
       </c>
       <c r="B243" s="7"/>
       <c r="C243" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2288,7 +2397,7 @@
       </c>
       <c r="B245" s="7"/>
       <c r="C245" s="2" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2296,7 +2405,7 @@
         <v>3.2</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>5</v>
@@ -2304,7 +2413,7 @@
     </row>
     <row r="247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A247" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B247" s="9"/>
       <c r="C247" s="8"/>
@@ -2314,16 +2423,16 @@
         <v>54</v>
       </c>
       <c r="B296" s="11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C296" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="297" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A297" s="13"/>
       <c r="B297" s="17" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C297" s="18"/>
     </row>
@@ -2335,15 +2444,15 @@
         <v>2</v>
       </c>
       <c r="C298" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="299" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A299" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C299" t="s">
         <v>5</v>
@@ -2355,7 +2464,7 @@
       </c>
       <c r="B300" s="7"/>
       <c r="C300" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2363,10 +2472,10 @@
         <v>1.2</v>
       </c>
       <c r="B301" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C301" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="302" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2375,7 +2484,7 @@
       </c>
       <c r="B302" s="7"/>
       <c r="C302" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2383,10 +2492,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B303" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="304" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2395,7 +2504,7 @@
       </c>
       <c r="B304" s="7"/>
       <c r="C304" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="305" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2415,7 +2524,7 @@
       </c>
       <c r="B306" s="7"/>
       <c r="C306" s="2" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2423,7 +2532,7 @@
         <v>4.2</v>
       </c>
       <c r="B307" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C307" s="2" t="s">
         <v>5</v>
@@ -2431,7 +2540,7 @@
     </row>
     <row r="308" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A308" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B308" s="9"/>
       <c r="C308" s="8"/>
@@ -2462,15 +2571,15 @@
         <v>2</v>
       </c>
       <c r="C357" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="358" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A358" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B358" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C358" t="s">
         <v>5</v>
@@ -2482,7 +2591,7 @@
       </c>
       <c r="B359" s="7"/>
       <c r="C359" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2516,7 +2625,7 @@
       </c>
       <c r="B363" s="7"/>
       <c r="C363" s="2" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2524,7 +2633,7 @@
         <v>3.2</v>
       </c>
       <c r="B364" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C364" s="2" t="s">
         <v>5</v>
@@ -2532,7 +2641,7 @@
     </row>
     <row r="365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A365" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B365" s="9"/>
       <c r="C365" s="8"/>
@@ -2563,15 +2672,15 @@
         <v>2</v>
       </c>
       <c r="C416" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="417" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A417" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B417" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C417" t="s">
         <v>5</v>
@@ -2583,7 +2692,7 @@
       </c>
       <c r="B418" s="7"/>
       <c r="C418" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="419" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2591,7 +2700,7 @@
         <v>1.2</v>
       </c>
       <c r="B419" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C419" s="2" t="s">
         <v>6</v>
@@ -2603,7 +2712,7 @@
       </c>
       <c r="B420" s="7"/>
       <c r="C420" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2648,7 +2757,7 @@
         <v>61</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2668,7 +2777,7 @@
         <v>5.2</v>
       </c>
       <c r="B428" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C428" s="2" t="s">
         <v>6</v>
@@ -2680,7 +2789,7 @@
       </c>
       <c r="B429" s="7"/>
       <c r="C429" s="2" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2688,7 +2797,7 @@
         <v>6.2</v>
       </c>
       <c r="B430" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C430" s="2" t="s">
         <v>5</v>
@@ -2696,7 +2805,7 @@
     </row>
     <row r="431" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A431" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B431" s="9"/>
       <c r="C431" s="8"/>
@@ -2706,7 +2815,7 @@
         <v>63</v>
       </c>
       <c r="B473" s="11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C473" s="12" t="s">
         <v>4</v>
@@ -2715,7 +2824,7 @@
     <row r="474" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A474" s="13"/>
       <c r="B474" s="17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C474" s="18"/>
     </row>
@@ -2727,15 +2836,15 @@
         <v>2</v>
       </c>
       <c r="C475" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="476" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A476" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B476" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C476" t="s">
         <v>5</v>
@@ -2747,7 +2856,7 @@
       </c>
       <c r="B477" s="7"/>
       <c r="C477" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="478" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2755,7 +2864,7 @@
         <v>1.2</v>
       </c>
       <c r="B478" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C478" s="2" t="s">
         <v>6</v>
@@ -2767,7 +2876,7 @@
       </c>
       <c r="B479" s="7"/>
       <c r="C479" s="2" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2775,7 +2884,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B480" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C480" s="2" t="s">
         <v>5</v>
@@ -2783,26 +2892,26 @@
     </row>
     <row r="481" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A481" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B481" s="9"/>
       <c r="C481" s="8"/>
     </row>
     <row r="532" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A532" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B532" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C532" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A533" s="13"/>
       <c r="B533" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C533" s="21"/>
     </row>
@@ -2814,15 +2923,15 @@
         <v>2</v>
       </c>
       <c r="C534" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="535" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A535" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B535" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C535" t="s">
         <v>5</v>
@@ -2834,7 +2943,7 @@
       </c>
       <c r="B536" s="7"/>
       <c r="C536" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="537" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2842,7 +2951,7 @@
         <v>1.2</v>
       </c>
       <c r="B537" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C537" s="2" t="s">
         <v>6</v>
@@ -2854,7 +2963,7 @@
       </c>
       <c r="B538" s="7"/>
       <c r="C538" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2865,7 +2974,7 @@
         <v>7</v>
       </c>
       <c r="C539" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2880,7 +2989,7 @@
         <v>3.2</v>
       </c>
       <c r="B541" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C541" s="2" t="s">
         <v>6</v>
@@ -2892,7 +3001,7 @@
       </c>
       <c r="B542" s="7"/>
       <c r="C542" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="543" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2903,7 +3012,7 @@
         <v>7</v>
       </c>
       <c r="C543" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2912,7 +3021,7 @@
       </c>
       <c r="B544" s="7"/>
       <c r="C544" s="2" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2920,10 +3029,10 @@
         <v>5.2</v>
       </c>
       <c r="B545" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C545" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2938,7 +3047,7 @@
         <v>6.2</v>
       </c>
       <c r="B547" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C547" s="2" t="s">
         <v>5</v>
@@ -2946,17 +3055,291 @@
     </row>
     <row r="548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A548" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B548" s="9"/>
       <c r="C548" s="8"/>
     </row>
+    <row r="591" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A591" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B591" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C591" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="592" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A592" s="13"/>
+      <c r="B592" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C592" s="18"/>
+    </row>
+    <row r="593" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A593" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B593" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C593" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="594" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A594" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B594" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C594" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="595" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A595" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B595" s="7"/>
+      <c r="C595" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="596" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A596" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B596" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C596" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="597" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A597" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B597" s="7"/>
+      <c r="C597" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="598" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A598" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B598" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C598" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="599" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A599" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B599" s="7"/>
+      <c r="C599" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="600" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A600" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B600" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C600" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="601" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A601" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B601" s="7"/>
+      <c r="C601" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="602" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A602" s="3"/>
+      <c r="B602" s="7"/>
+      <c r="C602" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A603" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B603" s="7"/>
+      <c r="C603" s="2"/>
+    </row>
+    <row r="604" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A604" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B604" s="7"/>
+      <c r="C604" s="2"/>
+    </row>
+    <row r="605" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A605" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B605" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C605" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="606" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A606" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B606" s="9"/>
+      <c r="C606" s="8"/>
+    </row>
+    <row r="650" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A650" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B650" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C650" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="651" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A651" s="13"/>
+      <c r="B651" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C651" s="21"/>
+    </row>
+    <row r="652" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A652" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B652" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C652" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="653" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A653" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B653" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C653" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="654" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A654" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B654" s="7"/>
+      <c r="C654" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="655" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A655" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B655" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C655" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="656" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A656" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B656" s="7"/>
+      <c r="C656" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="657" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A657" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B657" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C657" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="658" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A658" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B658" s="7"/>
+      <c r="C658" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="659" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A659" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B659" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C659" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="660" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A660" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B660" s="7"/>
+      <c r="C660" s="2"/>
+    </row>
+    <row r="661" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A661" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B661" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C661" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="662" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A662" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B662" s="9"/>
+      <c r="C662" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B120:C120"/>
     <mergeCell ref="B179:C179"/>
     <mergeCell ref="B425:B426"/>
     <mergeCell ref="B533:C533"/>
+    <mergeCell ref="B651:C651"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup scale="79" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Every SPC-700 instruction up to 0E.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF57CCB6-E034-4B07-8030-87F4F3897370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66FFF95-91CD-43C0-81E9-524877467981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11235" yWindow="0" windowWidth="16575" windowHeight="15600" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$687</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$883</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="90">
   <si>
     <t>Implied</t>
   </si>
@@ -86,6 +86,9 @@
     <t>Store as Address.L.</t>
   </si>
   <si>
+    <t>Absolute (Read/Modify/Write)</t>
+  </si>
+  <si>
     <t>Absolute (Read)</t>
   </si>
   <si>
@@ -188,6 +191,9 @@
     </r>
   </si>
   <si>
+    <t>Discard.</t>
+  </si>
+  <si>
     <t>Store as Address.H.</t>
   </si>
   <si>
@@ -300,6 +306,567 @@
     </r>
   </si>
   <si>
+    <t>SET1 (02)</t>
+  </si>
+  <si>
+    <t>Operand = (Operand &amp; ~1) | 1.</t>
+  </si>
+  <si>
+    <t>Write Operand.</t>
+  </si>
+  <si>
+    <t>Direct Page Bit (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <t>BBS (03)</t>
+  </si>
+  <si>
+    <t>Direct Page Bit Relative</t>
+  </si>
+  <si>
+    <t>Set Jump to (Operand &amp; (1 &lt;&lt; 0)) == (1 &lt;&lt; 0).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. If !Jump, end instruction (next half-cycle is 7.2).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Address = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + int8( Operand ).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L = Address.L.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.H = Address.H.</t>
+    </r>
+  </si>
+  <si>
+    <t>Cycles: 5-7</t>
+  </si>
+  <si>
+    <t>OR (04)</t>
+  </si>
+  <si>
+    <t>Direct Page (Read)</t>
+  </si>
+  <si>
+    <t>OR (05)</t>
+  </si>
+  <si>
+    <t>OR (06)</t>
+  </si>
+  <si>
+    <t>Indirect X (Read)</t>
+  </si>
+  <si>
+    <t>OR (07)</t>
+  </si>
+  <si>
+    <t>X-Indexed Indirect (Read)</t>
+  </si>
+  <si>
+    <t>Store as Pointer.L.</t>
+  </si>
+  <si>
+    <t>OR (08)</t>
+  </si>
+  <si>
+    <t>OR (09)</t>
+  </si>
+  <si>
+    <t>Store as Operand0.</t>
+  </si>
+  <si>
+    <t>Store as Operand1.</t>
+  </si>
+  <si>
+    <t>Write Operand0.</t>
+  </si>
+  <si>
+    <t>Direct Page to Direct Page (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <t>OR1 (0A)</t>
+  </si>
+  <si>
+    <t>Absolute Boolean Bit</t>
+  </si>
+  <si>
+    <t>Read (Address &amp; $1FFF)</t>
+  </si>
+  <si>
+    <t>Bit = Address &gt;&gt; 13.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag |= ((Operand &amp; (1 &lt;&lt; Bit)) != 0).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> |= Operand. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> |= Operand. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Operand0 |= Operand1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand0 &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !Operand0.</t>
+    </r>
+  </si>
+  <si>
+    <t>ASL (0B)</t>
+  </si>
+  <si>
+    <t>Direct Page (Read/Modify/Write)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand &amp; $80). Operand &lt;&lt;= 1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !Operand.</t>
+    </r>
+  </si>
+  <si>
+    <t>ASL (0C)</t>
+  </si>
+  <si>
+    <t>PUSH (0D)</t>
+  </si>
+  <si>
     <r>
       <t>Write to u8(</t>
     </r>
@@ -312,17 +879,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L+0) | $0100</t>
+      <t>SP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>+0) | $0100</t>
     </r>
   </si>
   <si>
@@ -338,27 +905,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L-1) | $0100</t>
-    </r>
-  </si>
-  <si>
-    <t>SET1 (02)</t>
-  </si>
-  <si>
-    <t>Operand = (Operand &amp; ~1) | 1.</t>
-  </si>
-  <si>
-    <t>Write Operand.</t>
+      <t>SP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-1) | $0100</t>
+    </r>
   </si>
   <si>
     <r>
@@ -394,7 +952,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>SPW</t>
+      <t>PSW</t>
     </r>
     <r>
       <rPr>
@@ -425,20 +983,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> flag) &lt;&lt; 3).</t>
-    </r>
-  </si>
-  <si>
-    <t>Direct Page Bit (Read/Modify/Write)</t>
-  </si>
-  <si>
-    <t>BBS (03)</t>
-  </si>
-  <si>
-    <t>Direct Page Bit Relative</t>
-  </si>
-  <si>
-    <t>Set Jump to (Operand &amp; (1 &lt;&lt; 0)) == (1 &lt;&lt; 0).</t>
+      <t xml:space="preserve"> flag) &lt;&lt; 3)).</t>
+    </r>
   </si>
   <si>
     <r>
@@ -463,32 +1009,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>. If !Jump, end instruction (next half-cycle is 7.2).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Inc. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>. Address = (Operand | ((</t>
     </r>
     <r>
@@ -500,7 +1020,101 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>SPW</t>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3)).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3))</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Address = ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + Operand) &amp; $FF) | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
     </r>
     <r>
       <rPr>
@@ -515,152 +1129,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Address = </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> + int8( Operand ).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L = Address.L.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.H = Address.H.</t>
-    </r>
-  </si>
-  <si>
-    <t>Cycles: 5-7</t>
-  </si>
-  <si>
-    <t>OR (04)</t>
-  </si>
-  <si>
-    <t>Direct Page (Read)</t>
-  </si>
-  <si>
-    <t>OR (05)</t>
-  </si>
-  <si>
-    <t>OR (06)</t>
-  </si>
-  <si>
-    <t>Indirect X (Read)</t>
-  </si>
-  <si>
-    <r>
-      <t>Read (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>X</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> | ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SPW</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3))</t>
-    </r>
-  </si>
-  <si>
-    <t>OR (07)</t>
-  </si>
-  <si>
-    <t>X-Indexed Indirect (Read)</t>
-  </si>
-  <si>
-    <t>Store as Pointer.L.</t>
-  </si>
-  <si>
-    <r>
       <t>Read ((Address + 1) &amp; $FF) | ((</t>
     </r>
     <r>
@@ -672,7 +1140,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>SPW</t>
+      <t>PSW</t>
     </r>
     <r>
       <rPr>
@@ -708,105 +1176,63 @@
   </si>
   <si>
     <r>
-      <t>Address = ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>X</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> + Operand) &amp; $FF) | ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SPW</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; P flag) &lt;&lt; 3).</t>
-    </r>
-  </si>
-  <si>
-    <t>OR (08)</t>
-  </si>
-  <si>
-    <t>OR (09)</t>
-  </si>
-  <si>
-    <t>Store as Operand0.</t>
-  </si>
-  <si>
-    <t>Store as Operand1.</t>
-  </si>
-  <si>
-    <t>Write Operand0.</t>
-  </si>
-  <si>
-    <t>Direct Page to Direct Page (Read/Modify/Write)</t>
-  </si>
-  <si>
-    <t>OR1 (0A)</t>
-  </si>
-  <si>
-    <t>Absolute Boolean Bit</t>
-  </si>
-  <si>
-    <t>Read (Address &amp; $1FFF)</t>
-  </si>
-  <si>
-    <t>Bit = Address &gt;&gt; 13.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag |= ((Operand &amp; (1 &lt;&lt; Bit)) != 0).</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">Push </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> onto stack.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 1. </t>
+    </r>
+  </si>
+  <si>
+    <t>TSET1 (0E)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Operand |= </t>
+    </r>
     <r>
       <rPr>
         <b/>
@@ -826,7 +1252,57 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> |= Operand. </t>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Operand = (A - Operand). Z flag = (Operand == 0), N flag = (Operand &amp; $80).</t>
+  </si>
+  <si>
+    <r>
+      <t>Operand = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Operand). </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand == 0), </t>
     </r>
     <r>
       <rPr>
@@ -847,319 +1323,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> flag = (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; $80), </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = !</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Inc. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> |= Operand. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &amp; $80), </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = !</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Operand0 |= Operand1. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = (Operand0 &amp; $80), </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = !Operand0.</t>
-    </r>
-  </si>
-  <si>
-    <t>ASL (0B)</t>
-  </si>
-  <si>
-    <t>Direct Page (Read/Modify/Write)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = (Operand &amp; $80). Operand &lt;&lt;= 1. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = (Operand &amp; $80), </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> flag = !Operand.</t>
+      <t xml:space="preserve"> flag = (Operand &amp; $80).</t>
     </r>
   </si>
 </sst>
@@ -1728,7 +1892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C662"/>
+  <dimension ref="A1:C843"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -1740,7 +1904,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>12</v>
@@ -1764,15 +1928,15 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -1784,7 +1948,7 @@
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1806,7 +1970,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>5</v>
@@ -1814,14 +1978,14 @@
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="8"/>
     </row>
     <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>9</v>
@@ -1845,15 +2009,15 @@
         <v>2</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>5</v>
@@ -1865,7 +2029,7 @@
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1873,7 +2037,7 @@
         <v>1.2</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>6</v>
@@ -1905,10 +2069,10 @@
         <v>3.2</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1923,10 +2087,10 @@
         <v>4.2</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1935,7 +2099,7 @@
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1957,10 +2121,10 @@
         <v>6.2</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1975,10 +2139,10 @@
         <v>7.2</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1993,7 +2157,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>5</v>
@@ -2001,7 +2165,7 @@
     </row>
     <row r="80" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B80" s="9"/>
       <c r="C80" s="8"/>
@@ -2020,7 +2184,7 @@
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
       <c r="B120" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C120" s="21"/>
     </row>
@@ -2032,15 +2196,15 @@
         <v>2</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C122" t="s">
         <v>5</v>
@@ -2052,7 +2216,7 @@
       </c>
       <c r="B123" s="7"/>
       <c r="C123" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2060,7 +2224,7 @@
         <v>1.2</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>6</v>
@@ -2072,7 +2236,7 @@
       </c>
       <c r="B125" s="7"/>
       <c r="C125" s="2" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2100,7 +2264,7 @@
         <v>3.2</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C128" s="2" t="s">
         <v>40</v>
@@ -2118,7 +2282,7 @@
         <v>4.2</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>5</v>
@@ -2126,26 +2290,26 @@
     </row>
     <row r="131" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B131" s="9"/>
       <c r="C131" s="8"/>
     </row>
     <row r="178" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B178" s="11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C178" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="13"/>
       <c r="B179" s="20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C179" s="21"/>
     </row>
@@ -2157,15 +2321,15 @@
         <v>2</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="181" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C181" t="s">
         <v>5</v>
@@ -2177,7 +2341,7 @@
       </c>
       <c r="B182" s="7"/>
       <c r="C182" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2185,7 +2349,7 @@
         <v>1.2</v>
       </c>
       <c r="B183" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C183" s="2" t="s">
         <v>6</v>
@@ -2197,7 +2361,7 @@
       </c>
       <c r="B184" s="7"/>
       <c r="C184" s="2" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2217,7 +2381,7 @@
       </c>
       <c r="B186" s="7"/>
       <c r="C186" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="187" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2239,7 +2403,7 @@
         <v>4.2</v>
       </c>
       <c r="B189" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>6</v>
@@ -2251,7 +2415,7 @@
       </c>
       <c r="B190" s="7"/>
       <c r="C190" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2267,14 +2431,14 @@
       </c>
       <c r="B192" s="7"/>
       <c r="C192" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="3"/>
       <c r="B193" s="7"/>
       <c r="C193" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2290,7 +2454,7 @@
       </c>
       <c r="B195" s="7"/>
       <c r="C195" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2298,7 +2462,7 @@
         <v>7.2</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>5</v>
@@ -2306,14 +2470,14 @@
     </row>
     <row r="197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B197" s="9"/>
       <c r="C197" s="8"/>
     </row>
     <row r="237" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B237" s="11" t="s">
         <v>10</v>
@@ -2325,7 +2489,7 @@
     <row r="238" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="13"/>
       <c r="B238" s="17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C238" s="18"/>
     </row>
@@ -2337,15 +2501,15 @@
         <v>2</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="240" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C240" t="s">
         <v>5</v>
@@ -2357,7 +2521,7 @@
       </c>
       <c r="B241" s="7"/>
       <c r="C241" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="242" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2365,7 +2529,7 @@
         <v>1.2</v>
       </c>
       <c r="B242" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>6</v>
@@ -2377,7 +2541,7 @@
       </c>
       <c r="B243" s="7"/>
       <c r="C243" s="2" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
     </row>
     <row r="244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2397,7 +2561,7 @@
       </c>
       <c r="B245" s="7"/>
       <c r="C245" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2405,7 +2569,7 @@
         <v>3.2</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>5</v>
@@ -2413,26 +2577,26 @@
     </row>
     <row r="247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A247" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B247" s="9"/>
       <c r="C247" s="8"/>
     </row>
     <row r="296" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A296" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B296" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C296" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="297" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A297" s="13"/>
       <c r="B297" s="17" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C297" s="18"/>
     </row>
@@ -2444,15 +2608,15 @@
         <v>2</v>
       </c>
       <c r="C298" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="299" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A299" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C299" t="s">
         <v>5</v>
@@ -2464,7 +2628,7 @@
       </c>
       <c r="B300" s="7"/>
       <c r="C300" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2472,7 +2636,7 @@
         <v>1.2</v>
       </c>
       <c r="B301" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C301" s="2" t="s">
         <v>14</v>
@@ -2484,7 +2648,7 @@
       </c>
       <c r="B302" s="7"/>
       <c r="C302" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2492,10 +2656,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B303" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="304" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2504,7 +2668,7 @@
       </c>
       <c r="B304" s="7"/>
       <c r="C304" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="305" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2524,7 +2688,7 @@
       </c>
       <c r="B306" s="7"/>
       <c r="C306" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2532,7 +2696,7 @@
         <v>4.2</v>
       </c>
       <c r="B307" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C307" s="2" t="s">
         <v>5</v>
@@ -2540,14 +2704,14 @@
     </row>
     <row r="308" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A308" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B308" s="9"/>
       <c r="C308" s="8"/>
     </row>
     <row r="355" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A355" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B355" s="11" t="s">
         <v>10</v>
@@ -2559,7 +2723,7 @@
     <row r="356" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A356" s="13"/>
       <c r="B356" s="17" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C356" s="18"/>
     </row>
@@ -2571,15 +2735,15 @@
         <v>2</v>
       </c>
       <c r="C357" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="358" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A358" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B358" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C358" t="s">
         <v>5</v>
@@ -2591,7 +2755,7 @@
       </c>
       <c r="B359" s="7"/>
       <c r="C359" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2613,7 +2777,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B362" s="7" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="C362" s="2" t="s">
         <v>6</v>
@@ -2625,7 +2789,7 @@
       </c>
       <c r="B363" s="7"/>
       <c r="C363" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2633,7 +2797,7 @@
         <v>3.2</v>
       </c>
       <c r="B364" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C364" s="2" t="s">
         <v>5</v>
@@ -2641,14 +2805,14 @@
     </row>
     <row r="365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A365" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B365" s="9"/>
       <c r="C365" s="8"/>
     </row>
     <row r="414" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A414" s="10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B414" s="11" t="s">
         <v>3</v>
@@ -2660,7 +2824,7 @@
     <row r="415" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A415" s="13"/>
       <c r="B415" s="17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C415" s="18"/>
     </row>
@@ -2672,15 +2836,15 @@
         <v>2</v>
       </c>
       <c r="C416" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="417" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A417" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B417" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C417" t="s">
         <v>5</v>
@@ -2692,7 +2856,7 @@
       </c>
       <c r="B418" s="7"/>
       <c r="C418" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="419" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2700,7 +2864,7 @@
         <v>1.2</v>
       </c>
       <c r="B419" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C419" s="2" t="s">
         <v>6</v>
@@ -2712,7 +2876,7 @@
       </c>
       <c r="B420" s="7"/>
       <c r="C420" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2728,7 +2892,7 @@
       </c>
       <c r="B422" s="7"/>
       <c r="C422" s="2" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
     </row>
     <row r="423" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2739,7 +2903,7 @@
         <v>7</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2754,10 +2918,10 @@
         <v>4.2</v>
       </c>
       <c r="B425" s="22" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2777,7 +2941,7 @@
         <v>5.2</v>
       </c>
       <c r="B428" s="7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C428" s="2" t="s">
         <v>6</v>
@@ -2789,7 +2953,7 @@
       </c>
       <c r="B429" s="7"/>
       <c r="C429" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2797,7 +2961,7 @@
         <v>6.2</v>
       </c>
       <c r="B430" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C430" s="2" t="s">
         <v>5</v>
@@ -2805,14 +2969,14 @@
     </row>
     <row r="431" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A431" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B431" s="9"/>
       <c r="C431" s="8"/>
     </row>
     <row r="473" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A473" s="10" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B473" s="11" t="s">
         <v>12</v>
@@ -2824,7 +2988,7 @@
     <row r="474" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A474" s="13"/>
       <c r="B474" s="17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C474" s="18"/>
     </row>
@@ -2836,15 +3000,15 @@
         <v>2</v>
       </c>
       <c r="C475" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="476" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A476" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B476" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C476" t="s">
         <v>5</v>
@@ -2856,7 +3020,7 @@
       </c>
       <c r="B477" s="7"/>
       <c r="C477" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="478" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2864,7 +3028,7 @@
         <v>1.2</v>
       </c>
       <c r="B478" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C478" s="2" t="s">
         <v>6</v>
@@ -2876,7 +3040,7 @@
       </c>
       <c r="B479" s="7"/>
       <c r="C479" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2884,7 +3048,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B480" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C480" s="2" t="s">
         <v>5</v>
@@ -2892,26 +3056,26 @@
     </row>
     <row r="481" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A481" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B481" s="9"/>
       <c r="C481" s="8"/>
     </row>
     <row r="532" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A532" s="10" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B532" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C532" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A533" s="13"/>
       <c r="B533" s="20" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C533" s="21"/>
     </row>
@@ -2923,15 +3087,15 @@
         <v>2</v>
       </c>
       <c r="C534" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="535" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A535" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B535" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C535" t="s">
         <v>5</v>
@@ -2943,7 +3107,7 @@
       </c>
       <c r="B536" s="7"/>
       <c r="C536" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="537" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2951,7 +3115,7 @@
         <v>1.2</v>
       </c>
       <c r="B537" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C537" s="2" t="s">
         <v>6</v>
@@ -2963,7 +3127,7 @@
       </c>
       <c r="B538" s="7"/>
       <c r="C538" s="2" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
     </row>
     <row r="539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2974,7 +3138,7 @@
         <v>7</v>
       </c>
       <c r="C539" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2989,7 +3153,7 @@
         <v>3.2</v>
       </c>
       <c r="B541" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C541" s="2" t="s">
         <v>6</v>
@@ -3001,7 +3165,7 @@
       </c>
       <c r="B542" s="7"/>
       <c r="C542" s="2" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
     </row>
     <row r="543" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3012,7 +3176,7 @@
         <v>7</v>
       </c>
       <c r="C543" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3021,7 +3185,7 @@
       </c>
       <c r="B544" s="7"/>
       <c r="C544" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3029,10 +3193,10 @@
         <v>5.2</v>
       </c>
       <c r="B545" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C545" s="2" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3047,7 +3211,7 @@
         <v>6.2</v>
       </c>
       <c r="B547" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C547" s="2" t="s">
         <v>5</v>
@@ -3055,26 +3219,26 @@
     </row>
     <row r="548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A548" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B548" s="9"/>
       <c r="C548" s="8"/>
     </row>
     <row r="591" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A591" s="10" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B591" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C591" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="592" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A592" s="13"/>
       <c r="B592" s="17" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C592" s="18"/>
     </row>
@@ -3086,15 +3250,15 @@
         <v>2</v>
       </c>
       <c r="C593" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="594" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A594" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B594" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C594" t="s">
         <v>5</v>
@@ -3106,7 +3270,7 @@
       </c>
       <c r="B595" s="7"/>
       <c r="C595" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="596" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3114,7 +3278,7 @@
         <v>1.2</v>
       </c>
       <c r="B596" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C596" s="2" t="s">
         <v>14</v>
@@ -3126,7 +3290,7 @@
       </c>
       <c r="B597" s="7"/>
       <c r="C597" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="598" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3134,10 +3298,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B598" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C598" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="599" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3146,7 +3310,7 @@
       </c>
       <c r="B599" s="7"/>
       <c r="C599" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="600" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3154,7 +3318,7 @@
         <v>3.2</v>
       </c>
       <c r="B600" s="7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C600" s="2" t="s">
         <v>6</v>
@@ -3166,14 +3330,14 @@
       </c>
       <c r="B601" s="7"/>
       <c r="C601" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="602" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A602" s="3"/>
       <c r="B602" s="7"/>
       <c r="C602" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3195,7 +3359,7 @@
         <v>5.2</v>
       </c>
       <c r="B605" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C605" s="2" t="s">
         <v>5</v>
@@ -3203,14 +3367,14 @@
     </row>
     <row r="606" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A606" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B606" s="9"/>
       <c r="C606" s="8"/>
     </row>
     <row r="650" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A650" s="10" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B650" s="11" t="s">
         <v>13</v>
@@ -3222,7 +3386,7 @@
     <row r="651" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A651" s="13"/>
       <c r="B651" s="20" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C651" s="21"/>
     </row>
@@ -3234,15 +3398,15 @@
         <v>2</v>
       </c>
       <c r="C652" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="653" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A653" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B653" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C653" t="s">
         <v>5</v>
@@ -3254,7 +3418,7 @@
       </c>
       <c r="B654" s="7"/>
       <c r="C654" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="655" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3262,7 +3426,7 @@
         <v>1.2</v>
       </c>
       <c r="B655" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C655" s="2" t="s">
         <v>6</v>
@@ -3274,7 +3438,7 @@
       </c>
       <c r="B656" s="7"/>
       <c r="C656" s="2" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
     </row>
     <row r="657" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3294,7 +3458,7 @@
       </c>
       <c r="B658" s="7"/>
       <c r="C658" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="659" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3302,7 +3466,7 @@
         <v>3.2</v>
       </c>
       <c r="B659" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C659" s="2" t="s">
         <v>40</v>
@@ -3320,7 +3484,7 @@
         <v>4.2</v>
       </c>
       <c r="B661" s="7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C661" s="2" t="s">
         <v>5</v>
@@ -3328,18 +3492,449 @@
     </row>
     <row r="662" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A662" s="16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B662" s="9"/>
       <c r="C662" s="8"/>
     </row>
+    <row r="709" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A709" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B709" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C709" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="710" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A710" s="13"/>
+      <c r="B710" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C710" s="21"/>
+    </row>
+    <row r="711" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A711" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B711" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C711" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="712" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A712" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B712" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C712" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="713" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A713" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B713" s="7"/>
+      <c r="C713" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="714" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A714" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B714" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C714" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="715" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A715" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B715" s="7"/>
+      <c r="C715" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="716" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A716" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B716" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C716" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="717" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A717" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B717" s="7"/>
+      <c r="C717" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="718" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A718" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B718" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C718" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="719" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A719" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B719" s="7"/>
+      <c r="C719" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="720" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A720" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B720" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C720" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="721" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A721" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B721" s="7"/>
+      <c r="C721" s="2"/>
+    </row>
+    <row r="722" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A722" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B722" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C722" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="723" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A723" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B723" s="9"/>
+      <c r="C723" s="8"/>
+    </row>
+    <row r="768" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A768" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B768" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C768" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="769" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A769" s="13"/>
+      <c r="B769" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C769" s="18"/>
+    </row>
+    <row r="770" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A770" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B770" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C770" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="771" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A771" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B771" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C771" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="772" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A772" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B772" s="7"/>
+      <c r="C772" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="773" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A773" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B773" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C773" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="774" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A774" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B774" s="7"/>
+      <c r="C774" s="2"/>
+    </row>
+    <row r="775" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A775" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B775" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C775" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="776" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A776" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B776" s="7"/>
+      <c r="C776" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="777" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A777" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B777" s="7"/>
+      <c r="C777" s="2"/>
+    </row>
+    <row r="778" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A778" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B778" s="7"/>
+      <c r="C778" s="2"/>
+    </row>
+    <row r="779" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A779" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B779" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C779" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="780" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A780" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B780" s="9"/>
+      <c r="C780" s="8"/>
+    </row>
+    <row r="827" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A827" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B827" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C827" s="12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="828" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A828" s="13"/>
+      <c r="B828" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C828" s="21"/>
+    </row>
+    <row r="829" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A829" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B829" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C829" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="830" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A830" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B830" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C830" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="831" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A831" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B831" s="7"/>
+      <c r="C831" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="832" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A832" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B832" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C832" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="833" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A833" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B833" s="7"/>
+      <c r="C833" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="834" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A834" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B834" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C834" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="835" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A835" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B835" s="7"/>
+      <c r="C835" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="836" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A836" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B836" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C836" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="837" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A837" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B837" s="7"/>
+      <c r="C837" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="838" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A838" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B838" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C838" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="839" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A839" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B839" s="7"/>
+      <c r="C839" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A840" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B840" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C840" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A841" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B841" s="7"/>
+      <c r="C841" s="2"/>
+    </row>
+    <row r="842" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A842" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B842" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C842" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A843" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B843" s="9"/>
+      <c r="C843" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
     <mergeCell ref="B120:C120"/>
     <mergeCell ref="B179:C179"/>
     <mergeCell ref="B425:B426"/>
     <mergeCell ref="B533:C533"/>
     <mergeCell ref="B651:C651"/>
+    <mergeCell ref="B710:C710"/>
+    <mergeCell ref="B828:C828"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup scale="79" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
SPC-700 up to 0F.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66FFF95-91CD-43C0-81E9-524877467981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6264BDB9-D4C9-4025-929C-52606A9C58B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$883</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$944</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="93">
   <si>
     <t>Implied</t>
   </si>
@@ -1231,6 +1231,32 @@
   </si>
   <si>
     <r>
+      <t>Tmp = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - Operand).</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">Operand |= </t>
     </r>
     <r>
@@ -1256,33 +1282,6 @@
     </r>
   </si>
   <si>
-    <t>Operand = (A - Operand). Z flag = (Operand == 0), N flag = (Operand &amp; $80).</t>
-  </si>
-  <si>
-    <r>
-      <t>Operand = (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> - Operand). </t>
-    </r>
     <r>
       <rPr>
         <b/>
@@ -1302,7 +1301,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> flag = (Operand == 0), </t>
+      <t xml:space="preserve"> flag = (Tmp == 0), </t>
     </r>
     <r>
       <rPr>
@@ -1323,7 +1322,104 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> flag = (Operand &amp; $80).</t>
+      <t xml:space="preserve"> flag = (Tmp &amp; $80).</t>
+    </r>
+  </si>
+  <si>
+    <t>BRK (0F)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = 0, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = 1.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Write to u8(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-2) | $0100</t>
     </r>
   </si>
 </sst>
@@ -1892,7 +1988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C843"/>
+  <dimension ref="A1:C906"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -3867,64 +3963,267 @@
       </c>
       <c r="B837" s="7"/>
       <c r="C837" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="838" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A838" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B838" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="A838" s="3"/>
+      <c r="B838" s="7"/>
       <c r="C838" s="2" t="s">
-        <v>6</v>
+        <v>88</v>
       </c>
     </row>
     <row r="839" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A839" s="3">
-        <v>5.0999999999999996</v>
-      </c>
+      <c r="A839" s="3"/>
       <c r="B839" s="7"/>
       <c r="C839" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A840" s="3">
-        <v>5.2</v>
+        <v>4.2</v>
       </c>
       <c r="B840" s="7" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="C840" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A841" s="3">
-        <v>6.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="B841" s="7"/>
       <c r="C841" s="2"/>
     </row>
     <row r="842" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A842" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B842" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C842" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A843" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B843" s="7"/>
+      <c r="C843" s="2"/>
+    </row>
+    <row r="844" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A844" s="3">
         <v>6.2</v>
       </c>
-      <c r="B842" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C842" s="2" t="s">
+      <c r="B844" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C844" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A843" s="16" t="s">
+    <row r="845" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A845" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B843" s="9"/>
-      <c r="C843" s="8"/>
+      <c r="B845" s="9"/>
+      <c r="C845" s="8"/>
+    </row>
+    <row r="886" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A886" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B886" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C886" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="887" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A887" s="13"/>
+      <c r="B887" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C887" s="18"/>
+    </row>
+    <row r="888" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A888" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B888" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C888" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="889" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A889" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B889" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C889" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="890" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A890" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B890" s="7"/>
+      <c r="C890" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="891" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A891" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B891" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C891" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="892" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A892" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B892" s="7"/>
+      <c r="C892" s="2"/>
+    </row>
+    <row r="893" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A893" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B893" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C893" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="894" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A894" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B894" s="7"/>
+      <c r="C894" s="2"/>
+    </row>
+    <row r="895" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A895" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B895" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C895" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="896" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A896" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B896" s="7"/>
+      <c r="C896" s="2"/>
+    </row>
+    <row r="897" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A897" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B897" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C897" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="898" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A898" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B898" s="7"/>
+      <c r="C898" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="899" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A899" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B899" s="7"/>
+      <c r="C899" s="2"/>
+    </row>
+    <row r="900" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A900" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B900" s="7"/>
+      <c r="C900" s="2"/>
+    </row>
+    <row r="901" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A901" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B901" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C901" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="902" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A902" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B902" s="7"/>
+      <c r="C902" s="2"/>
+    </row>
+    <row r="903" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A903" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B903" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C903" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="904" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A904" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="B904" s="7"/>
+      <c r="C904" s="2"/>
+    </row>
+    <row r="905" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A905" s="3">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B905" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C905" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="906" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A906" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B906" s="9"/>
+      <c r="C906" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Instructions up to 14.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6264BDB9-D4C9-4025-929C-52606A9C58B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7A53ACD-E657-44F8-B015-BAF52C4E33BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$944</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$1218</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="107">
   <si>
     <t>Implied</t>
   </si>
@@ -92,6 +92,9 @@
     <t>Absolute (Read)</t>
   </si>
   <si>
+    <t>BPL (10)</t>
+  </si>
+  <si>
     <t>Size: 3</t>
   </si>
   <si>
@@ -1421,6 +1424,177 @@
       </rPr>
       <t>-2) | $0100</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. If !Jump, end instruction (next half-cycle is 4.2).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Set Jump to (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; $80) == $00.</t>
+    </r>
+  </si>
+  <si>
+    <t>TCALL1 (11)</t>
+  </si>
+  <si>
+    <t>Read $FFDC</t>
+  </si>
+  <si>
+    <t>Read $FFDD</t>
+  </si>
+  <si>
+    <t>CLR1 (12)</t>
+  </si>
+  <si>
+    <t>Operand = (Operand &amp; ~1) | 0.</t>
+  </si>
+  <si>
+    <t>BBC0 (13)</t>
+  </si>
+  <si>
+    <t>Set Jump to (Operand &amp; (1 &lt;&lt; 0)) == (0 &lt;&lt; 0).</t>
+  </si>
+  <si>
+    <t>Cycles: 2-4</t>
+  </si>
+  <si>
+    <t>OR (14)</t>
+  </si>
+  <si>
+    <r>
+      <t>Address = ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + Operand) &amp; $FF) | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag) &lt;&lt; 3).</t>
+    </r>
+  </si>
+  <si>
+    <t>X-Indexed Direct Page (Read)</t>
   </si>
 </sst>
 </file>
@@ -1988,7 +2162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C906"/>
+  <dimension ref="A1:C1193"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -2000,7 +2174,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>12</v>
@@ -2024,15 +2198,15 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -2044,7 +2218,7 @@
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2066,7 +2240,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>5</v>
@@ -2074,14 +2248,14 @@
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="8"/>
     </row>
     <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>9</v>
@@ -2105,15 +2279,15 @@
         <v>2</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>5</v>
@@ -2125,7 +2299,7 @@
       </c>
       <c r="B64" s="7"/>
       <c r="C64" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2133,7 +2307,7 @@
         <v>1.2</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>6</v>
@@ -2165,10 +2339,10 @@
         <v>3.2</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2183,10 +2357,10 @@
         <v>4.2</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2195,7 +2369,7 @@
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2217,10 +2391,10 @@
         <v>6.2</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2235,10 +2409,10 @@
         <v>7.2</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2253,7 +2427,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>5</v>
@@ -2261,14 +2435,14 @@
     </row>
     <row r="80" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B80" s="9"/>
       <c r="C80" s="8"/>
     </row>
     <row r="119" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B119" s="11" t="s">
         <v>13</v>
@@ -2280,7 +2454,7 @@
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
       <c r="B120" s="20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C120" s="21"/>
     </row>
@@ -2292,15 +2466,15 @@
         <v>2</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="122" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C122" t="s">
         <v>5</v>
@@ -2312,7 +2486,7 @@
       </c>
       <c r="B123" s="7"/>
       <c r="C123" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2320,7 +2494,7 @@
         <v>1.2</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>6</v>
@@ -2332,7 +2506,7 @@
       </c>
       <c r="B125" s="7"/>
       <c r="C125" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2352,7 +2526,7 @@
       </c>
       <c r="B127" s="7"/>
       <c r="C127" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2360,10 +2534,10 @@
         <v>3.2</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2378,7 +2552,7 @@
         <v>4.2</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>5</v>
@@ -2386,26 +2560,26 @@
     </row>
     <row r="131" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B131" s="9"/>
       <c r="C131" s="8"/>
     </row>
     <row r="178" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B178" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C178" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="13"/>
       <c r="B179" s="20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C179" s="21"/>
     </row>
@@ -2417,15 +2591,15 @@
         <v>2</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="181" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C181" t="s">
         <v>5</v>
@@ -2437,7 +2611,7 @@
       </c>
       <c r="B182" s="7"/>
       <c r="C182" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2445,7 +2619,7 @@
         <v>1.2</v>
       </c>
       <c r="B183" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C183" s="2" t="s">
         <v>6</v>
@@ -2457,7 +2631,7 @@
       </c>
       <c r="B184" s="7"/>
       <c r="C184" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2477,7 +2651,7 @@
       </c>
       <c r="B186" s="7"/>
       <c r="C186" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="187" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2499,7 +2673,7 @@
         <v>4.2</v>
       </c>
       <c r="B189" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>6</v>
@@ -2511,7 +2685,7 @@
       </c>
       <c r="B190" s="7"/>
       <c r="C190" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2527,14 +2701,14 @@
       </c>
       <c r="B192" s="7"/>
       <c r="C192" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="3"/>
       <c r="B193" s="7"/>
       <c r="C193" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2550,7 +2724,7 @@
       </c>
       <c r="B195" s="7"/>
       <c r="C195" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2558,7 +2732,7 @@
         <v>7.2</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>5</v>
@@ -2566,14 +2740,14 @@
     </row>
     <row r="197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B197" s="9"/>
       <c r="C197" s="8"/>
     </row>
     <row r="237" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B237" s="11" t="s">
         <v>10</v>
@@ -2585,7 +2759,7 @@
     <row r="238" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="13"/>
       <c r="B238" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C238" s="18"/>
     </row>
@@ -2597,15 +2771,15 @@
         <v>2</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="240" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C240" t="s">
         <v>5</v>
@@ -2617,7 +2791,7 @@
       </c>
       <c r="B241" s="7"/>
       <c r="C241" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="242" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2625,7 +2799,7 @@
         <v>1.2</v>
       </c>
       <c r="B242" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>6</v>
@@ -2637,7 +2811,7 @@
       </c>
       <c r="B243" s="7"/>
       <c r="C243" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2657,7 +2831,7 @@
       </c>
       <c r="B245" s="7"/>
       <c r="C245" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2665,7 +2839,7 @@
         <v>3.2</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>5</v>
@@ -2673,20 +2847,20 @@
     </row>
     <row r="247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A247" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B247" s="9"/>
       <c r="C247" s="8"/>
     </row>
     <row r="296" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A296" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B296" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C296" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="297" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2704,15 +2878,15 @@
         <v>2</v>
       </c>
       <c r="C298" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="299" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A299" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C299" t="s">
         <v>5</v>
@@ -2724,7 +2898,7 @@
       </c>
       <c r="B300" s="7"/>
       <c r="C300" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2732,7 +2906,7 @@
         <v>1.2</v>
       </c>
       <c r="B301" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C301" s="2" t="s">
         <v>14</v>
@@ -2744,7 +2918,7 @@
       </c>
       <c r="B302" s="7"/>
       <c r="C302" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2752,10 +2926,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B303" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C303" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="304" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2764,7 +2938,7 @@
       </c>
       <c r="B304" s="7"/>
       <c r="C304" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="305" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2784,7 +2958,7 @@
       </c>
       <c r="B306" s="7"/>
       <c r="C306" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2792,7 +2966,7 @@
         <v>4.2</v>
       </c>
       <c r="B307" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C307" s="2" t="s">
         <v>5</v>
@@ -2800,14 +2974,14 @@
     </row>
     <row r="308" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A308" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B308" s="9"/>
       <c r="C308" s="8"/>
     </row>
     <row r="355" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A355" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B355" s="11" t="s">
         <v>10</v>
@@ -2819,7 +2993,7 @@
     <row r="356" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A356" s="13"/>
       <c r="B356" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C356" s="18"/>
     </row>
@@ -2831,15 +3005,15 @@
         <v>2</v>
       </c>
       <c r="C357" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="358" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A358" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B358" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C358" t="s">
         <v>5</v>
@@ -2851,7 +3025,7 @@
       </c>
       <c r="B359" s="7"/>
       <c r="C359" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2873,7 +3047,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B362" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C362" s="2" t="s">
         <v>6</v>
@@ -2885,7 +3059,7 @@
       </c>
       <c r="B363" s="7"/>
       <c r="C363" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2893,7 +3067,7 @@
         <v>3.2</v>
       </c>
       <c r="B364" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C364" s="2" t="s">
         <v>5</v>
@@ -2901,14 +3075,14 @@
     </row>
     <row r="365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A365" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B365" s="9"/>
       <c r="C365" s="8"/>
     </row>
     <row r="414" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A414" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B414" s="11" t="s">
         <v>3</v>
@@ -2920,7 +3094,7 @@
     <row r="415" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A415" s="13"/>
       <c r="B415" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C415" s="18"/>
     </row>
@@ -2932,15 +3106,15 @@
         <v>2</v>
       </c>
       <c r="C416" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="417" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A417" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B417" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C417" t="s">
         <v>5</v>
@@ -2952,7 +3126,7 @@
       </c>
       <c r="B418" s="7"/>
       <c r="C418" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="419" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2960,7 +3134,7 @@
         <v>1.2</v>
       </c>
       <c r="B419" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C419" s="2" t="s">
         <v>6</v>
@@ -2972,7 +3146,7 @@
       </c>
       <c r="B420" s="7"/>
       <c r="C420" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2988,7 +3162,7 @@
       </c>
       <c r="B422" s="7"/>
       <c r="C422" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="423" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2999,7 +3173,7 @@
         <v>7</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3014,10 +3188,10 @@
         <v>4.2</v>
       </c>
       <c r="B425" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C425" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3037,7 +3211,7 @@
         <v>5.2</v>
       </c>
       <c r="B428" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C428" s="2" t="s">
         <v>6</v>
@@ -3049,7 +3223,7 @@
       </c>
       <c r="B429" s="7"/>
       <c r="C429" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3057,7 +3231,7 @@
         <v>6.2</v>
       </c>
       <c r="B430" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C430" s="2" t="s">
         <v>5</v>
@@ -3065,14 +3239,14 @@
     </row>
     <row r="431" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A431" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B431" s="9"/>
       <c r="C431" s="8"/>
     </row>
     <row r="473" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A473" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B473" s="11" t="s">
         <v>12</v>
@@ -3084,7 +3258,7 @@
     <row r="474" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A474" s="13"/>
       <c r="B474" s="17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C474" s="18"/>
     </row>
@@ -3096,15 +3270,15 @@
         <v>2</v>
       </c>
       <c r="C475" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="476" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A476" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B476" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C476" t="s">
         <v>5</v>
@@ -3116,7 +3290,7 @@
       </c>
       <c r="B477" s="7"/>
       <c r="C477" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="478" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3124,7 +3298,7 @@
         <v>1.2</v>
       </c>
       <c r="B478" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C478" s="2" t="s">
         <v>6</v>
@@ -3136,7 +3310,7 @@
       </c>
       <c r="B479" s="7"/>
       <c r="C479" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3144,7 +3318,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B480" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C480" s="2" t="s">
         <v>5</v>
@@ -3152,26 +3326,26 @@
     </row>
     <row r="481" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A481" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B481" s="9"/>
       <c r="C481" s="8"/>
     </row>
     <row r="532" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A532" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B532" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C532" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A533" s="13"/>
       <c r="B533" s="20" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C533" s="21"/>
     </row>
@@ -3183,15 +3357,15 @@
         <v>2</v>
       </c>
       <c r="C534" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="535" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A535" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B535" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C535" t="s">
         <v>5</v>
@@ -3203,7 +3377,7 @@
       </c>
       <c r="B536" s="7"/>
       <c r="C536" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="537" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3211,7 +3385,7 @@
         <v>1.2</v>
       </c>
       <c r="B537" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C537" s="2" t="s">
         <v>6</v>
@@ -3223,7 +3397,7 @@
       </c>
       <c r="B538" s="7"/>
       <c r="C538" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3234,7 +3408,7 @@
         <v>7</v>
       </c>
       <c r="C539" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3249,7 +3423,7 @@
         <v>3.2</v>
       </c>
       <c r="B541" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C541" s="2" t="s">
         <v>6</v>
@@ -3261,7 +3435,7 @@
       </c>
       <c r="B542" s="7"/>
       <c r="C542" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="543" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3272,7 +3446,7 @@
         <v>7</v>
       </c>
       <c r="C543" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3281,7 +3455,7 @@
       </c>
       <c r="B544" s="7"/>
       <c r="C544" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3289,10 +3463,10 @@
         <v>5.2</v>
       </c>
       <c r="B545" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C545" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3307,7 +3481,7 @@
         <v>6.2</v>
       </c>
       <c r="B547" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C547" s="2" t="s">
         <v>5</v>
@@ -3315,26 +3489,26 @@
     </row>
     <row r="548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A548" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B548" s="9"/>
       <c r="C548" s="8"/>
     </row>
     <row r="591" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A591" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B591" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C591" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="592" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A592" s="13"/>
       <c r="B592" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C592" s="18"/>
     </row>
@@ -3346,15 +3520,15 @@
         <v>2</v>
       </c>
       <c r="C593" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="594" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A594" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B594" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C594" t="s">
         <v>5</v>
@@ -3366,7 +3540,7 @@
       </c>
       <c r="B595" s="7"/>
       <c r="C595" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="596" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3374,7 +3548,7 @@
         <v>1.2</v>
       </c>
       <c r="B596" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C596" s="2" t="s">
         <v>14</v>
@@ -3386,7 +3560,7 @@
       </c>
       <c r="B597" s="7"/>
       <c r="C597" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="598" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3394,10 +3568,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B598" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C598" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="599" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3406,7 +3580,7 @@
       </c>
       <c r="B599" s="7"/>
       <c r="C599" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="600" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3414,7 +3588,7 @@
         <v>3.2</v>
       </c>
       <c r="B600" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C600" s="2" t="s">
         <v>6</v>
@@ -3426,14 +3600,14 @@
       </c>
       <c r="B601" s="7"/>
       <c r="C601" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="602" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A602" s="3"/>
       <c r="B602" s="7"/>
       <c r="C602" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3455,7 +3629,7 @@
         <v>5.2</v>
       </c>
       <c r="B605" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C605" s="2" t="s">
         <v>5</v>
@@ -3463,14 +3637,14 @@
     </row>
     <row r="606" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A606" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B606" s="9"/>
       <c r="C606" s="8"/>
     </row>
     <row r="650" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A650" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B650" s="11" t="s">
         <v>13</v>
@@ -3482,7 +3656,7 @@
     <row r="651" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A651" s="13"/>
       <c r="B651" s="20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C651" s="21"/>
     </row>
@@ -3494,15 +3668,15 @@
         <v>2</v>
       </c>
       <c r="C652" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="653" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A653" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B653" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C653" t="s">
         <v>5</v>
@@ -3514,7 +3688,7 @@
       </c>
       <c r="B654" s="7"/>
       <c r="C654" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="655" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3522,7 +3696,7 @@
         <v>1.2</v>
       </c>
       <c r="B655" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C655" s="2" t="s">
         <v>6</v>
@@ -3534,7 +3708,7 @@
       </c>
       <c r="B656" s="7"/>
       <c r="C656" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="657" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3554,7 +3728,7 @@
       </c>
       <c r="B658" s="7"/>
       <c r="C658" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="659" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3562,10 +3736,10 @@
         <v>3.2</v>
       </c>
       <c r="B659" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C659" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="660" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3580,7 +3754,7 @@
         <v>4.2</v>
       </c>
       <c r="B661" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C661" s="2" t="s">
         <v>5</v>
@@ -3588,20 +3762,20 @@
     </row>
     <row r="662" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A662" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B662" s="9"/>
       <c r="C662" s="8"/>
     </row>
     <row r="709" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A709" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B709" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C709" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="710" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3619,15 +3793,15 @@
         <v>2</v>
       </c>
       <c r="C711" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="712" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A712" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B712" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C712" t="s">
         <v>5</v>
@@ -3639,7 +3813,7 @@
       </c>
       <c r="B713" s="7"/>
       <c r="C713" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="714" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3647,7 +3821,7 @@
         <v>1.2</v>
       </c>
       <c r="B714" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C714" s="2" t="s">
         <v>14</v>
@@ -3659,7 +3833,7 @@
       </c>
       <c r="B715" s="7"/>
       <c r="C715" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="716" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3667,10 +3841,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B716" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C716" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="717" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3679,7 +3853,7 @@
       </c>
       <c r="B717" s="7"/>
       <c r="C717" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="718" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3699,7 +3873,7 @@
       </c>
       <c r="B719" s="7"/>
       <c r="C719" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="720" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3707,10 +3881,10 @@
         <v>4.2</v>
       </c>
       <c r="B720" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C720" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="721" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3725,7 +3899,7 @@
         <v>5.2</v>
       </c>
       <c r="B722" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C722" s="2" t="s">
         <v>5</v>
@@ -3733,14 +3907,14 @@
     </row>
     <row r="723" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A723" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B723" s="9"/>
       <c r="C723" s="8"/>
     </row>
     <row r="768" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A768" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B768" s="11" t="s">
         <v>13</v>
@@ -3764,15 +3938,15 @@
         <v>2</v>
       </c>
       <c r="C770" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="771" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A771" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B771" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C771" t="s">
         <v>5</v>
@@ -3784,7 +3958,7 @@
       </c>
       <c r="B772" s="7"/>
       <c r="C772" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="773" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3792,10 +3966,10 @@
         <v>1.2</v>
       </c>
       <c r="B773" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C773" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="774" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3810,10 +3984,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B775" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C775" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="776" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3822,7 +3996,7 @@
       </c>
       <c r="B776" s="7"/>
       <c r="C776" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="777" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3844,7 +4018,7 @@
         <v>4.2</v>
       </c>
       <c r="B779" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C779" s="2" t="s">
         <v>5</v>
@@ -3852,20 +4026,20 @@
     </row>
     <row r="780" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A780" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B780" s="9"/>
       <c r="C780" s="8"/>
     </row>
     <row r="827" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A827" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B827" s="11" t="s">
         <v>3</v>
       </c>
       <c r="C827" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="828" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3883,15 +4057,15 @@
         <v>2</v>
       </c>
       <c r="C829" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="830" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A830" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B830" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C830" t="s">
         <v>5</v>
@@ -3903,7 +4077,7 @@
       </c>
       <c r="B831" s="7"/>
       <c r="C831" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="832" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3911,7 +4085,7 @@
         <v>1.2</v>
       </c>
       <c r="B832" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C832" s="2" t="s">
         <v>14</v>
@@ -3923,7 +4097,7 @@
       </c>
       <c r="B833" s="7"/>
       <c r="C833" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="834" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3931,10 +4105,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B834" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C834" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="835" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3943,7 +4117,7 @@
       </c>
       <c r="B835" s="7"/>
       <c r="C835" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="836" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3963,21 +4137,21 @@
       </c>
       <c r="B837" s="7"/>
       <c r="C837" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="838" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A838" s="3"/>
       <c r="B838" s="7"/>
       <c r="C838" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="839" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A839" s="3"/>
       <c r="B839" s="7"/>
       <c r="C839" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3988,7 +4162,7 @@
         <v>7</v>
       </c>
       <c r="C840" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4003,10 +4177,10 @@
         <v>5.2</v>
       </c>
       <c r="B842" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C842" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4021,7 +4195,7 @@
         <v>6.2</v>
       </c>
       <c r="B844" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C844" s="2" t="s">
         <v>5</v>
@@ -4029,14 +4203,14 @@
     </row>
     <row r="845" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A845" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B845" s="9"/>
       <c r="C845" s="8"/>
     </row>
     <row r="886" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A886" s="10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B886" s="11" t="s">
         <v>9</v>
@@ -4060,15 +4234,15 @@
         <v>2</v>
       </c>
       <c r="C888" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="889" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A889" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B889" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C889" t="s">
         <v>5</v>
@@ -4080,7 +4254,7 @@
       </c>
       <c r="B890" s="7"/>
       <c r="C890" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="891" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4088,10 +4262,10 @@
         <v>1.2</v>
       </c>
       <c r="B891" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C891" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="892" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4106,10 +4280,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B893" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C893" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="894" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4124,10 +4298,10 @@
         <v>3.2</v>
       </c>
       <c r="B895" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C895" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="896" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4142,10 +4316,10 @@
         <v>4.2</v>
       </c>
       <c r="B897" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C897" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="898" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4154,7 +4328,7 @@
       </c>
       <c r="B898" s="7"/>
       <c r="C898" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="899" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4176,10 +4350,10 @@
         <v>6.2</v>
       </c>
       <c r="B901" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C901" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="902" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4194,10 +4368,10 @@
         <v>7.2</v>
       </c>
       <c r="B903" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C903" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="904" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4212,7 +4386,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B905" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C905" s="2" t="s">
         <v>5</v>
@@ -4220,19 +4394,762 @@
     </row>
     <row r="906" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A906" s="16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B906" s="9"/>
       <c r="C906" s="8"/>
     </row>
+    <row r="945" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A945" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B945" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C945" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="946" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A946" s="13"/>
+      <c r="B946" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C946" s="18"/>
+    </row>
+    <row r="947" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A947" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B947" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C947" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="948" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A948" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B948" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C948" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="949" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A949" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B949" s="7"/>
+      <c r="C949" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="950" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A950" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B950" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C950" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="951" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A951" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B951" s="7"/>
+      <c r="C951" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="952" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A952" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B952" s="7"/>
+      <c r="C952" s="2"/>
+    </row>
+    <row r="953" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A953" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B953" s="7"/>
+      <c r="C953" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="954" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A954" s="3"/>
+      <c r="B954" s="7"/>
+      <c r="C954" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="955" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A955" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B955" s="7"/>
+      <c r="C955" s="2"/>
+    </row>
+    <row r="956" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A956" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B956" s="7"/>
+      <c r="C956" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="957" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A957" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B957" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C957" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="958" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A958" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B958" s="9"/>
+      <c r="C958" s="8"/>
+    </row>
+    <row r="1004" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1004" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1004" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1004" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1005" s="13"/>
+      <c r="B1005" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1005" s="18"/>
+    </row>
+    <row r="1006" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1006" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1006" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1006" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1007" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1007" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1007" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1008" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B1008" s="7"/>
+      <c r="C1008" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1009" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B1009" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1009" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1010" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B1010" s="7"/>
+      <c r="C1010" s="2"/>
+    </row>
+    <row r="1011" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1011" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1011" s="7"/>
+      <c r="C1011" s="2"/>
+    </row>
+    <row r="1012" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1012" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B1012" s="7"/>
+      <c r="C1012" s="2"/>
+    </row>
+    <row r="1013" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1013" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B1013" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1013" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1014" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B1014" s="7"/>
+      <c r="C1014" s="2"/>
+    </row>
+    <row r="1015" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1015" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B1015" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1015" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1016" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B1016" s="7"/>
+      <c r="C1016" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1017" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B1017" s="7"/>
+      <c r="C1017" s="2"/>
+    </row>
+    <row r="1018" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1018" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B1018" s="7"/>
+      <c r="C1018" s="2"/>
+    </row>
+    <row r="1019" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1019" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B1019" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1019" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1020" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B1020" s="7"/>
+      <c r="C1020" s="2"/>
+    </row>
+    <row r="1021" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1021" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B1021" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1021" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1022" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="B1022" s="7"/>
+      <c r="C1022" s="2"/>
+    </row>
+    <row r="1023" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1023" s="3">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B1023" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1023" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1024" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1024" s="9"/>
+      <c r="C1024" s="8"/>
+    </row>
+    <row r="1063" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1063" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1063" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1063" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1064" s="13"/>
+      <c r="B1064" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1064" s="21"/>
+    </row>
+    <row r="1065" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1065" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1065" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1065" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1066" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1066" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1066" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1067" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B1067" s="7"/>
+      <c r="C1067" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1068" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B1068" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1068" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1069" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B1069" s="7"/>
+      <c r="C1069" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1070" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1070" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1070" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1071" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B1071" s="7"/>
+      <c r="C1071" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1072" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B1072" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1072" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1073" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B1073" s="7"/>
+      <c r="C1073" s="2"/>
+    </row>
+    <row r="1074" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1074" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B1074" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1074" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1075" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1075" s="9"/>
+      <c r="C1075" s="8"/>
+    </row>
+    <row r="1122" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1122" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1122" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1122" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1123" s="13"/>
+      <c r="B1123" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1123" s="18"/>
+    </row>
+    <row r="1124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1124" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1124" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1124" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1125" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1125" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1125" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1126" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B1126" s="7"/>
+      <c r="C1126" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1127" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B1127" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1127" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1128" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B1128" s="7"/>
+      <c r="C1128" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1129" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1129" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1129" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1130" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B1130" s="7"/>
+      <c r="C1130" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1131" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B1131" s="7"/>
+      <c r="C1131" s="2"/>
+    </row>
+    <row r="1132" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1132" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B1132" s="7"/>
+      <c r="C1132" s="2"/>
+    </row>
+    <row r="1133" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1133" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B1133" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1133" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1134" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B1134" s="7"/>
+      <c r="C1134" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1135" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B1135" s="7"/>
+      <c r="C1135" s="2"/>
+    </row>
+    <row r="1136" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1136" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B1136" s="7"/>
+      <c r="C1136" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1137" s="3"/>
+      <c r="B1137" s="7"/>
+      <c r="C1137" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1138" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B1138" s="7"/>
+      <c r="C1138" s="2"/>
+    </row>
+    <row r="1139" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1139" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B1139" s="7"/>
+      <c r="C1139" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1140" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B1140" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1140" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1141" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1141" s="9"/>
+      <c r="C1141" s="8"/>
+    </row>
+    <row r="1181" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1181" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1181" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1181" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1182" s="13"/>
+      <c r="B1182" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1182" s="21"/>
+    </row>
+    <row r="1183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1183" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1183" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1183" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1184" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1184" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1184" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1185" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B1185" s="7"/>
+      <c r="C1185" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1186" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B1186" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1186" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1187" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B1187" s="7"/>
+      <c r="C1187" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1188" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1188" s="7"/>
+      <c r="C1188" s="2"/>
+    </row>
+    <row r="1189" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1189" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B1189" s="7"/>
+      <c r="C1189" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1190" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B1190" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1190" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1191" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B1191" s="7"/>
+      <c r="C1191" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1192" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B1192" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1192" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1193" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1193" s="9"/>
+      <c r="C1193" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="B120:C120"/>
     <mergeCell ref="B179:C179"/>
     <mergeCell ref="B425:B426"/>
     <mergeCell ref="B533:C533"/>
     <mergeCell ref="B651:C651"/>
     <mergeCell ref="B710:C710"/>
+    <mergeCell ref="B1064:C1064"/>
+    <mergeCell ref="B1182:C1182"/>
     <mergeCell ref="B828:C828"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Instructions up to 17.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7A53ACD-E657-44F8-B015-BAF52C4E33BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FACB16F5-1831-419B-B1CE-0F29550D97C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$1218</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$1414</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="118">
   <si>
     <t>Implied</t>
   </si>
@@ -206,6 +206,9 @@
     <t>NOP (00)</t>
   </si>
   <si>
+    <t xml:space="preserve">Inc. PC. </t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Read </t>
     </r>
@@ -1179,6 +1182,53 @@
   </si>
   <si>
     <r>
+      <t>Address = (Operand | ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag) &lt;&lt; 3)).</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">Push </t>
     </r>
     <r>
@@ -1595,6 +1645,102 @@
   </si>
   <si>
     <t>X-Indexed Direct Page (Read)</t>
+  </si>
+  <si>
+    <t>OR (15)</t>
+  </si>
+  <si>
+    <t>X-Indexed Absolute (Read)</t>
+  </si>
+  <si>
+    <r>
+      <t>Pointer = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + Address).</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (16)</t>
+  </si>
+  <si>
+    <t>Y-Indexed Absolute (Read)</t>
+  </si>
+  <si>
+    <r>
+      <t>Pointer = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + Address).</t>
+    </r>
+  </si>
+  <si>
+    <t>OR (17)</t>
+  </si>
+  <si>
+    <t>Indirect Y-Indexed [d]+Y (Read)</t>
+  </si>
+  <si>
+    <r>
+      <t>Address = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + Pointer).</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2162,7 +2308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C1193"/>
+  <dimension ref="A1:C1375"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -2206,7 +2352,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -2240,7 +2386,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>5</v>
@@ -2255,7 +2401,7 @@
     </row>
     <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>9</v>
@@ -2287,7 +2433,7 @@
         <v>24</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>5</v>
@@ -2307,7 +2453,7 @@
         <v>1.2</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>6</v>
@@ -2339,7 +2485,7 @@
         <v>3.2</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>20</v>
@@ -2357,7 +2503,7 @@
         <v>4.2</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>21</v>
@@ -2369,7 +2515,7 @@
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2391,10 +2537,10 @@
         <v>6.2</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2409,10 +2555,10 @@
         <v>7.2</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2427,7 +2573,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>5</v>
@@ -2442,7 +2588,7 @@
     </row>
     <row r="119" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B119" s="11" t="s">
         <v>13</v>
@@ -2454,7 +2600,7 @@
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
       <c r="B120" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C120" s="21"/>
     </row>
@@ -2474,7 +2620,7 @@
         <v>24</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C122" t="s">
         <v>5</v>
@@ -2494,7 +2640,7 @@
         <v>1.2</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>6</v>
@@ -2506,7 +2652,7 @@
       </c>
       <c r="B125" s="7"/>
       <c r="C125" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2526,7 +2672,7 @@
       </c>
       <c r="B127" s="7"/>
       <c r="C127" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2537,7 +2683,7 @@
         <v>25</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2552,7 +2698,7 @@
         <v>4.2</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>5</v>
@@ -2567,10 +2713,10 @@
     </row>
     <row r="178" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B178" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C178" s="12" t="s">
         <v>18</v>
@@ -2579,7 +2725,7 @@
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="13"/>
       <c r="B179" s="20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C179" s="21"/>
     </row>
@@ -2599,7 +2745,7 @@
         <v>24</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C181" t="s">
         <v>5</v>
@@ -2619,7 +2765,7 @@
         <v>1.2</v>
       </c>
       <c r="B183" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C183" s="2" t="s">
         <v>6</v>
@@ -2631,7 +2777,7 @@
       </c>
       <c r="B184" s="7"/>
       <c r="C184" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2651,7 +2797,7 @@
       </c>
       <c r="B186" s="7"/>
       <c r="C186" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="187" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2673,7 +2819,7 @@
         <v>4.2</v>
       </c>
       <c r="B189" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>6</v>
@@ -2685,7 +2831,7 @@
       </c>
       <c r="B190" s="7"/>
       <c r="C190" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2701,14 +2847,14 @@
       </c>
       <c r="B192" s="7"/>
       <c r="C192" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="3"/>
       <c r="B193" s="7"/>
       <c r="C193" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2724,7 +2870,7 @@
       </c>
       <c r="B195" s="7"/>
       <c r="C195" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2732,7 +2878,7 @@
         <v>7.2</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>5</v>
@@ -2747,7 +2893,7 @@
     </row>
     <row r="237" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B237" s="11" t="s">
         <v>10</v>
@@ -2759,7 +2905,7 @@
     <row r="238" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="13"/>
       <c r="B238" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C238" s="18"/>
     </row>
@@ -2779,7 +2925,7 @@
         <v>24</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C240" t="s">
         <v>5</v>
@@ -2799,7 +2945,7 @@
         <v>1.2</v>
       </c>
       <c r="B242" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>6</v>
@@ -2811,7 +2957,7 @@
       </c>
       <c r="B243" s="7"/>
       <c r="C243" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2831,7 +2977,7 @@
       </c>
       <c r="B245" s="7"/>
       <c r="C245" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2839,7 +2985,7 @@
         <v>3.2</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>5</v>
@@ -2854,7 +3000,7 @@
     </row>
     <row r="296" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A296" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B296" s="11" t="s">
         <v>13</v>
@@ -2886,7 +3032,7 @@
         <v>24</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C299" t="s">
         <v>5</v>
@@ -2906,7 +3052,7 @@
         <v>1.2</v>
       </c>
       <c r="B301" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C301" s="2" t="s">
         <v>14</v>
@@ -2926,7 +3072,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B303" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C303" s="2" t="s">
         <v>29</v>
@@ -2958,7 +3104,7 @@
       </c>
       <c r="B306" s="7"/>
       <c r="C306" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2966,7 +3112,7 @@
         <v>4.2</v>
       </c>
       <c r="B307" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C307" s="2" t="s">
         <v>5</v>
@@ -2981,7 +3127,7 @@
     </row>
     <row r="355" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A355" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B355" s="11" t="s">
         <v>10</v>
@@ -2993,7 +3139,7 @@
     <row r="356" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A356" s="13"/>
       <c r="B356" s="17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C356" s="18"/>
     </row>
@@ -3013,7 +3159,7 @@
         <v>24</v>
       </c>
       <c r="B358" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C358" t="s">
         <v>5</v>
@@ -3047,7 +3193,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B362" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C362" s="2" t="s">
         <v>6</v>
@@ -3059,7 +3205,7 @@
       </c>
       <c r="B363" s="7"/>
       <c r="C363" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3067,7 +3213,7 @@
         <v>3.2</v>
       </c>
       <c r="B364" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C364" s="2" t="s">
         <v>5</v>
@@ -3082,7 +3228,7 @@
     </row>
     <row r="414" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A414" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B414" s="11" t="s">
         <v>3</v>
@@ -3094,7 +3240,7 @@
     <row r="415" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A415" s="13"/>
       <c r="B415" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C415" s="18"/>
     </row>
@@ -3114,7 +3260,7 @@
         <v>24</v>
       </c>
       <c r="B417" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C417" t="s">
         <v>5</v>
@@ -3134,7 +3280,7 @@
         <v>1.2</v>
       </c>
       <c r="B419" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C419" s="2" t="s">
         <v>6</v>
@@ -3162,7 +3308,7 @@
       </c>
       <c r="B422" s="7"/>
       <c r="C422" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="423" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3173,7 +3319,7 @@
         <v>7</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3188,7 +3334,7 @@
         <v>4.2</v>
       </c>
       <c r="B425" s="22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C425" s="2" t="s">
         <v>22</v>
@@ -3223,7 +3369,7 @@
       </c>
       <c r="B429" s="7"/>
       <c r="C429" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3231,7 +3377,7 @@
         <v>6.2</v>
       </c>
       <c r="B430" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C430" s="2" t="s">
         <v>5</v>
@@ -3246,7 +3392,7 @@
     </row>
     <row r="473" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A473" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B473" s="11" t="s">
         <v>12</v>
@@ -3278,7 +3424,7 @@
         <v>24</v>
       </c>
       <c r="B476" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C476" t="s">
         <v>5</v>
@@ -3298,7 +3444,7 @@
         <v>1.2</v>
       </c>
       <c r="B478" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C478" s="2" t="s">
         <v>6</v>
@@ -3310,7 +3456,7 @@
       </c>
       <c r="B479" s="7"/>
       <c r="C479" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3318,7 +3464,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B480" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C480" s="2" t="s">
         <v>5</v>
@@ -3333,7 +3479,7 @@
     </row>
     <row r="532" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A532" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B532" s="11" t="s">
         <v>3</v>
@@ -3345,7 +3491,7 @@
     <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A533" s="13"/>
       <c r="B533" s="20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C533" s="21"/>
     </row>
@@ -3365,7 +3511,7 @@
         <v>24</v>
       </c>
       <c r="B535" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C535" t="s">
         <v>5</v>
@@ -3385,7 +3531,7 @@
         <v>1.2</v>
       </c>
       <c r="B537" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C537" s="2" t="s">
         <v>6</v>
@@ -3397,7 +3543,7 @@
       </c>
       <c r="B538" s="7"/>
       <c r="C538" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3408,7 +3554,7 @@
         <v>7</v>
       </c>
       <c r="C539" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3423,7 +3569,7 @@
         <v>3.2</v>
       </c>
       <c r="B541" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C541" s="2" t="s">
         <v>6</v>
@@ -3435,7 +3581,7 @@
       </c>
       <c r="B542" s="7"/>
       <c r="C542" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="543" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3446,7 +3592,7 @@
         <v>7</v>
       </c>
       <c r="C543" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3455,7 +3601,7 @@
       </c>
       <c r="B544" s="7"/>
       <c r="C544" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3466,7 +3612,7 @@
         <v>25</v>
       </c>
       <c r="C545" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3481,7 +3627,7 @@
         <v>6.2</v>
       </c>
       <c r="B547" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C547" s="2" t="s">
         <v>5</v>
@@ -3496,7 +3642,7 @@
     </row>
     <row r="591" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A591" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B591" s="11" t="s">
         <v>11</v>
@@ -3508,7 +3654,7 @@
     <row r="592" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A592" s="13"/>
       <c r="B592" s="17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C592" s="18"/>
     </row>
@@ -3528,7 +3674,7 @@
         <v>24</v>
       </c>
       <c r="B594" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C594" t="s">
         <v>5</v>
@@ -3548,7 +3694,7 @@
         <v>1.2</v>
       </c>
       <c r="B596" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C596" s="2" t="s">
         <v>14</v>
@@ -3568,7 +3714,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B598" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C598" s="2" t="s">
         <v>29</v>
@@ -3588,7 +3734,7 @@
         <v>3.2</v>
       </c>
       <c r="B600" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C600" s="2" t="s">
         <v>6</v>
@@ -3600,14 +3746,14 @@
       </c>
       <c r="B601" s="7"/>
       <c r="C601" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="602" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A602" s="3"/>
       <c r="B602" s="7"/>
       <c r="C602" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3629,7 +3775,7 @@
         <v>5.2</v>
       </c>
       <c r="B605" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C605" s="2" t="s">
         <v>5</v>
@@ -3644,7 +3790,7 @@
     </row>
     <row r="650" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A650" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B650" s="11" t="s">
         <v>13</v>
@@ -3656,7 +3802,7 @@
     <row r="651" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A651" s="13"/>
       <c r="B651" s="20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C651" s="21"/>
     </row>
@@ -3676,7 +3822,7 @@
         <v>24</v>
       </c>
       <c r="B653" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C653" t="s">
         <v>5</v>
@@ -3696,7 +3842,7 @@
         <v>1.2</v>
       </c>
       <c r="B655" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C655" s="2" t="s">
         <v>6</v>
@@ -3708,7 +3854,7 @@
       </c>
       <c r="B656" s="7"/>
       <c r="C656" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="657" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3728,7 +3874,7 @@
       </c>
       <c r="B658" s="7"/>
       <c r="C658" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="659" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3739,7 +3885,7 @@
         <v>25</v>
       </c>
       <c r="C659" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="660" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3754,7 +3900,7 @@
         <v>4.2</v>
       </c>
       <c r="B661" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C661" s="2" t="s">
         <v>5</v>
@@ -3769,7 +3915,7 @@
     </row>
     <row r="709" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A709" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B709" s="11" t="s">
         <v>11</v>
@@ -3801,7 +3947,7 @@
         <v>24</v>
       </c>
       <c r="B712" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C712" t="s">
         <v>5</v>
@@ -3821,7 +3967,7 @@
         <v>1.2</v>
       </c>
       <c r="B714" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C714" s="2" t="s">
         <v>14</v>
@@ -3841,7 +3987,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B716" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C716" s="2" t="s">
         <v>29</v>
@@ -3873,7 +4019,7 @@
       </c>
       <c r="B719" s="7"/>
       <c r="C719" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="720" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3884,7 +4030,7 @@
         <v>25</v>
       </c>
       <c r="C720" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="721" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3899,7 +4045,7 @@
         <v>5.2</v>
       </c>
       <c r="B722" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C722" s="2" t="s">
         <v>5</v>
@@ -3914,7 +4060,7 @@
     </row>
     <row r="768" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A768" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B768" s="11" t="s">
         <v>13</v>
@@ -3946,7 +4092,7 @@
         <v>24</v>
       </c>
       <c r="B771" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C771" t="s">
         <v>5</v>
@@ -3966,7 +4112,7 @@
         <v>1.2</v>
       </c>
       <c r="B773" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C773" s="2" t="s">
         <v>28</v>
@@ -3984,10 +4130,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B775" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C775" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="776" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3996,7 +4142,7 @@
       </c>
       <c r="B776" s="7"/>
       <c r="C776" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="777" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4018,7 +4164,7 @@
         <v>4.2</v>
       </c>
       <c r="B779" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C779" s="2" t="s">
         <v>5</v>
@@ -4033,7 +4179,7 @@
     </row>
     <row r="827" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A827" s="10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B827" s="11" t="s">
         <v>3</v>
@@ -4065,7 +4211,7 @@
         <v>24</v>
       </c>
       <c r="B830" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C830" t="s">
         <v>5</v>
@@ -4085,7 +4231,7 @@
         <v>1.2</v>
       </c>
       <c r="B832" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C832" s="2" t="s">
         <v>14</v>
@@ -4105,7 +4251,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B834" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C834" s="2" t="s">
         <v>29</v>
@@ -4137,21 +4283,21 @@
       </c>
       <c r="B837" s="7"/>
       <c r="C837" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="838" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A838" s="3"/>
       <c r="B838" s="7"/>
       <c r="C838" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="839" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A839" s="3"/>
       <c r="B839" s="7"/>
       <c r="C839" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4180,7 +4326,7 @@
         <v>25</v>
       </c>
       <c r="C842" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4195,7 +4341,7 @@
         <v>6.2</v>
       </c>
       <c r="B844" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C844" s="2" t="s">
         <v>5</v>
@@ -4210,7 +4356,7 @@
     </row>
     <row r="886" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A886" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B886" s="11" t="s">
         <v>9</v>
@@ -4242,7 +4388,7 @@
         <v>24</v>
       </c>
       <c r="B889" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C889" t="s">
         <v>5</v>
@@ -4262,7 +4408,7 @@
         <v>1.2</v>
       </c>
       <c r="B891" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C891" s="2" t="s">
         <v>28</v>
@@ -4280,7 +4426,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B893" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C893" s="2" t="s">
         <v>20</v>
@@ -4298,7 +4444,7 @@
         <v>3.2</v>
       </c>
       <c r="B895" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C895" s="2" t="s">
         <v>21</v>
@@ -4316,10 +4462,10 @@
         <v>4.2</v>
       </c>
       <c r="B897" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C897" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="898" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4328,7 +4474,7 @@
       </c>
       <c r="B898" s="7"/>
       <c r="C898" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="899" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4350,10 +4496,10 @@
         <v>6.2</v>
       </c>
       <c r="B901" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C901" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="902" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4368,10 +4514,10 @@
         <v>7.2</v>
       </c>
       <c r="B903" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C903" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="904" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4386,7 +4532,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B905" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C905" s="2" t="s">
         <v>5</v>
@@ -4404,7 +4550,7 @@
         <v>17</v>
       </c>
       <c r="B945" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C945" s="12" t="s">
         <v>4</v>
@@ -4433,7 +4579,7 @@
         <v>24</v>
       </c>
       <c r="B948" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C948" t="s">
         <v>5</v>
@@ -4445,7 +4591,7 @@
       </c>
       <c r="B949" s="7"/>
       <c r="C949" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="950" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4453,7 +4599,7 @@
         <v>1.2</v>
       </c>
       <c r="B950" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C950" s="2" t="s">
         <v>6</v>
@@ -4465,7 +4611,7 @@
       </c>
       <c r="B951" s="7"/>
       <c r="C951" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="952" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4481,14 +4627,14 @@
       </c>
       <c r="B953" s="7"/>
       <c r="C953" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="954" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A954" s="3"/>
       <c r="B954" s="7"/>
       <c r="C954" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="955" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4504,7 +4650,7 @@
       </c>
       <c r="B956" s="7"/>
       <c r="C956" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="957" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4512,7 +4658,7 @@
         <v>4.2</v>
       </c>
       <c r="B957" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C957" s="2" t="s">
         <v>5</v>
@@ -4527,7 +4673,7 @@
     </row>
     <row r="1004" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1004" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B1004" s="11" t="s">
         <v>9</v>
@@ -4559,7 +4705,7 @@
         <v>24</v>
       </c>
       <c r="B1007" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1007" t="s">
         <v>5</v>
@@ -4579,7 +4725,7 @@
         <v>1.2</v>
       </c>
       <c r="B1009" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1009" s="2" t="s">
         <v>6</v>
@@ -4611,7 +4757,7 @@
         <v>3.2</v>
       </c>
       <c r="B1013" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1013" s="2" t="s">
         <v>20</v>
@@ -4629,7 +4775,7 @@
         <v>4.2</v>
       </c>
       <c r="B1015" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C1015" s="2" t="s">
         <v>21</v>
@@ -4641,7 +4787,7 @@
       </c>
       <c r="B1016" s="7"/>
       <c r="C1016" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="1017" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4663,10 +4809,10 @@
         <v>6.2</v>
       </c>
       <c r="B1019" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C1019" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="1020" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4681,10 +4827,10 @@
         <v>7.2</v>
       </c>
       <c r="B1021" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C1021" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="1022" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4699,7 +4845,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B1023" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1023" s="2" t="s">
         <v>5</v>
@@ -4714,7 +4860,7 @@
     </row>
     <row r="1063" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1063" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B1063" s="11" t="s">
         <v>13</v>
@@ -4726,7 +4872,7 @@
     <row r="1064" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1064" s="13"/>
       <c r="B1064" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1064" s="21"/>
     </row>
@@ -4746,7 +4892,7 @@
         <v>24</v>
       </c>
       <c r="B1066" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1066" t="s">
         <v>5</v>
@@ -4766,7 +4912,7 @@
         <v>1.2</v>
       </c>
       <c r="B1068" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1068" s="2" t="s">
         <v>6</v>
@@ -4778,7 +4924,7 @@
       </c>
       <c r="B1069" s="7"/>
       <c r="C1069" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1070" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4798,7 +4944,7 @@
       </c>
       <c r="B1071" s="7"/>
       <c r="C1071" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="1072" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4809,7 +4955,7 @@
         <v>25</v>
       </c>
       <c r="C1072" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="1073" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4824,7 +4970,7 @@
         <v>4.2</v>
       </c>
       <c r="B1074" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1074" s="2" t="s">
         <v>5</v>
@@ -4839,10 +4985,10 @@
     </row>
     <row r="1122" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1122" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B1122" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C1122" s="12" t="s">
         <v>18</v>
@@ -4851,7 +4997,7 @@
     <row r="1123" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1123" s="13"/>
       <c r="B1123" s="17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C1123" s="18"/>
     </row>
@@ -4871,7 +5017,7 @@
         <v>24</v>
       </c>
       <c r="B1125" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1125" t="s">
         <v>5</v>
@@ -4891,7 +5037,7 @@
         <v>1.2</v>
       </c>
       <c r="B1127" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1127" s="2" t="s">
         <v>6</v>
@@ -4903,7 +5049,7 @@
       </c>
       <c r="B1128" s="7"/>
       <c r="C1128" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="1129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4923,7 +5069,7 @@
       </c>
       <c r="B1130" s="7"/>
       <c r="C1130" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="1131" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4945,7 +5091,7 @@
         <v>4.2</v>
       </c>
       <c r="B1133" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1133" s="2" t="s">
         <v>6</v>
@@ -4957,7 +5103,7 @@
       </c>
       <c r="B1134" s="7"/>
       <c r="C1134" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="1135" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4973,14 +5119,14 @@
       </c>
       <c r="B1136" s="7"/>
       <c r="C1136" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="1137" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1137" s="3"/>
       <c r="B1137" s="7"/>
       <c r="C1137" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="1138" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4996,7 +5142,7 @@
       </c>
       <c r="B1139" s="7"/>
       <c r="C1139" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="1140" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5004,7 +5150,7 @@
         <v>7.2</v>
       </c>
       <c r="B1140" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1140" s="2" t="s">
         <v>5</v>
@@ -5019,7 +5165,7 @@
     </row>
     <row r="1181" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1181" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B1181" s="11" t="s">
         <v>13</v>
@@ -5031,7 +5177,7 @@
     <row r="1182" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1182" s="13"/>
       <c r="B1182" s="20" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C1182" s="21"/>
     </row>
@@ -5051,7 +5197,7 @@
         <v>24</v>
       </c>
       <c r="B1184" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1184" t="s">
         <v>5</v>
@@ -5071,7 +5217,7 @@
         <v>1.2</v>
       </c>
       <c r="B1186" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1186" s="2" t="s">
         <v>6</v>
@@ -5099,7 +5245,7 @@
       </c>
       <c r="B1189" s="7"/>
       <c r="C1189" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="1190" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5119,7 +5265,7 @@
       </c>
       <c r="B1191" s="7"/>
       <c r="C1191" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="1192" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5127,7 +5273,7 @@
         <v>4.2</v>
       </c>
       <c r="B1192" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1192" s="2" t="s">
         <v>5</v>
@@ -5140,8 +5286,460 @@
       <c r="B1193" s="9"/>
       <c r="C1193" s="8"/>
     </row>
+    <row r="1240" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1240" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1240" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1240" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1241" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1241" s="13"/>
+      <c r="B1241" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1241" s="18"/>
+    </row>
+    <row r="1242" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1242" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1242" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1242" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1243" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1243" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1243" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1243" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1244" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B1244" s="7"/>
+      <c r="C1244" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1245" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1245" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B1245" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1245" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1246" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1246" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B1246" s="7"/>
+      <c r="C1246" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1247" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1247" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1247" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1248" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1248" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B1248" s="7"/>
+      <c r="C1248" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1249" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1249" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B1249" s="7"/>
+      <c r="C1249" s="2"/>
+    </row>
+    <row r="1250" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1250" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B1250" s="7"/>
+      <c r="C1250" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="1251" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1251" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B1251" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1251" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1252" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1252" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B1252" s="7"/>
+      <c r="C1252" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="1253" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1253" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B1253" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1253" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1254" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1254" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1254" s="9"/>
+      <c r="C1254" s="8"/>
+    </row>
+    <row r="1299" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1299" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1299" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1299" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1300" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1300" s="13"/>
+      <c r="B1300" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1300" s="18"/>
+    </row>
+    <row r="1301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1301" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1301" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1301" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1302" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1302" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1302" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1302" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1303" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B1303" s="7"/>
+      <c r="C1303" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1304" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1304" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B1304" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1304" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="1305" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1305" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B1305" s="7"/>
+      <c r="C1305" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1306" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1306" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1306" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1306" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1307" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B1307" s="7"/>
+      <c r="C1307" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1308" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1308" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B1308" s="7"/>
+      <c r="C1308" s="2"/>
+    </row>
+    <row r="1309" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1309" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B1309" s="7"/>
+      <c r="C1309" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="1310" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1310" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B1310" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1310" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1311" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B1311" s="7"/>
+      <c r="C1311" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1312" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B1312" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1312" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1313" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1313" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1313" s="9"/>
+      <c r="C1313" s="8"/>
+    </row>
+    <row r="1358" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1358" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1358" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1358" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1359" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1359" s="13"/>
+      <c r="B1359" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1359" s="21"/>
+    </row>
+    <row r="1360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1360" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1360" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1360" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1361" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1361" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1361" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1362" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1362" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B1362" s="7"/>
+      <c r="C1362" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1363" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1363" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B1363" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1363" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1364" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B1364" s="7"/>
+      <c r="C1364" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1365" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B1365" s="7"/>
+      <c r="C1365" s="2"/>
+    </row>
+    <row r="1366" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1366" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B1366" s="7"/>
+      <c r="C1366" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1367" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B1367" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1367" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1368" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B1368" s="7"/>
+      <c r="C1368" s="2"/>
+    </row>
+    <row r="1369" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1369" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B1369" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1369" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1370" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1370" s="3"/>
+      <c r="B1370" s="22"/>
+      <c r="C1370" s="2"/>
+    </row>
+    <row r="1371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1371" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B1371" s="7"/>
+      <c r="C1371" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="1372" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1372" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B1372" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1372" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1373" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1373" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B1373" s="7"/>
+      <c r="C1373" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="1374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1374" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B1374" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1374" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1375" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1375" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1375" s="9"/>
+      <c r="C1375" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="B120:C120"/>
     <mergeCell ref="B179:C179"/>
     <mergeCell ref="B425:B426"/>
@@ -5150,6 +5748,8 @@
     <mergeCell ref="B710:C710"/>
     <mergeCell ref="B1064:C1064"/>
     <mergeCell ref="B1182:C1182"/>
+    <mergeCell ref="B1369:B1370"/>
+    <mergeCell ref="B1359:C1359"/>
     <mergeCell ref="B828:C828"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Instructions up to 2D.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A382F0C3-5890-4CFD-8D95-6D1F86205245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FFC4898-6508-449A-972B-C58A6906D5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$2478</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$2714</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="171">
   <si>
     <t>Implied</t>
   </si>
@@ -212,6 +212,9 @@
     <t>NOP (00)</t>
   </si>
   <si>
+    <t>Read PC</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Read </t>
     </r>
@@ -2852,6 +2855,159 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> flag = !Operand0.</t>
+    </r>
+  </si>
+  <si>
+    <t>OR1 (2A)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag |= ((Operand &amp; (1 &lt;&lt; Bit)) == 0).</t>
+    </r>
+  </si>
+  <si>
+    <t>Absolute Boolean Bit /m.b</t>
+  </si>
+  <si>
+    <t>ROL (2B)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tmp = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand &amp; $80). Operand = (Operand &lt;&lt; 1) | Tmp. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Operand &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !Operand.</t>
+    </r>
+  </si>
+  <si>
+    <t>ROL (2C)</t>
+  </si>
+  <si>
+    <t>PUSH (2D)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Push </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> onto stack.</t>
     </r>
   </si>
 </sst>
@@ -3420,7 +3576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C2436"/>
+  <dimension ref="A1:C2668"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -3464,7 +3620,7 @@
         <v>22</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -3498,7 +3654,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>5</v>
@@ -3513,7 +3669,7 @@
     </row>
     <row r="60" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>9</v>
@@ -3545,7 +3701,7 @@
         <v>22</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>5</v>
@@ -3565,7 +3721,7 @@
         <v>1.2</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>6</v>
@@ -3597,7 +3753,7 @@
         <v>3.2</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>18</v>
@@ -3615,7 +3771,7 @@
         <v>4.2</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>19</v>
@@ -3627,7 +3783,7 @@
       </c>
       <c r="B72" s="7"/>
       <c r="C72" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3649,10 +3805,10 @@
         <v>6.2</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3667,10 +3823,10 @@
         <v>7.2</v>
       </c>
       <c r="B77" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3685,7 +3841,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>5</v>
@@ -3700,7 +3856,7 @@
     </row>
     <row r="119" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B119" s="11" t="s">
         <v>13</v>
@@ -3712,7 +3868,7 @@
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
       <c r="B120" s="20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C120" s="21"/>
     </row>
@@ -3732,7 +3888,7 @@
         <v>22</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C122" t="s">
         <v>5</v>
@@ -3752,7 +3908,7 @@
         <v>1.2</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>6</v>
@@ -3764,7 +3920,7 @@
       </c>
       <c r="B125" s="7"/>
       <c r="C125" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3784,7 +3940,7 @@
       </c>
       <c r="B127" s="7"/>
       <c r="C127" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="128" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3795,7 +3951,7 @@
         <v>23</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3810,7 +3966,7 @@
         <v>4.2</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>5</v>
@@ -3825,10 +3981,10 @@
     </row>
     <row r="178" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B178" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C178" s="12" t="s">
         <v>16</v>
@@ -3837,7 +3993,7 @@
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="13"/>
       <c r="B179" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C179" s="21"/>
     </row>
@@ -3857,7 +4013,7 @@
         <v>22</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C181" t="s">
         <v>5</v>
@@ -3877,7 +4033,7 @@
         <v>1.2</v>
       </c>
       <c r="B183" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C183" s="2" t="s">
         <v>6</v>
@@ -3889,7 +4045,7 @@
       </c>
       <c r="B184" s="7"/>
       <c r="C184" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3909,7 +4065,7 @@
       </c>
       <c r="B186" s="7"/>
       <c r="C186" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="187" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3931,7 +4087,7 @@
         <v>4.2</v>
       </c>
       <c r="B189" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>6</v>
@@ -3943,7 +4099,7 @@
       </c>
       <c r="B190" s="7"/>
       <c r="C190" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3959,14 +4115,14 @@
       </c>
       <c r="B192" s="7"/>
       <c r="C192" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="3"/>
       <c r="B193" s="7"/>
       <c r="C193" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3982,7 +4138,7 @@
       </c>
       <c r="B195" s="7"/>
       <c r="C195" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3990,7 +4146,7 @@
         <v>7.2</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C196" s="2" t="s">
         <v>5</v>
@@ -4005,7 +4161,7 @@
     </row>
     <row r="237" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B237" s="11" t="s">
         <v>10</v>
@@ -4017,7 +4173,7 @@
     <row r="238" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="13"/>
       <c r="B238" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C238" s="18"/>
     </row>
@@ -4037,7 +4193,7 @@
         <v>22</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C240" t="s">
         <v>5</v>
@@ -4057,7 +4213,7 @@
         <v>1.2</v>
       </c>
       <c r="B242" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C242" s="2" t="s">
         <v>6</v>
@@ -4069,7 +4225,7 @@
       </c>
       <c r="B243" s="7"/>
       <c r="C243" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4089,7 +4245,7 @@
       </c>
       <c r="B245" s="7"/>
       <c r="C245" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4097,7 +4253,7 @@
         <v>3.2</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C246" s="2" t="s">
         <v>5</v>
@@ -4112,7 +4268,7 @@
     </row>
     <row r="296" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A296" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B296" s="11" t="s">
         <v>13</v>
@@ -4124,7 +4280,7 @@
     <row r="297" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A297" s="13"/>
       <c r="B297" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C297" s="18"/>
     </row>
@@ -4144,7 +4300,7 @@
         <v>22</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C299" t="s">
         <v>5</v>
@@ -4164,7 +4320,7 @@
         <v>1.2</v>
       </c>
       <c r="B301" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C301" s="2" t="s">
         <v>14</v>
@@ -4184,7 +4340,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B303" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C303" s="2" t="s">
         <v>30</v>
@@ -4216,7 +4372,7 @@
       </c>
       <c r="B306" s="7"/>
       <c r="C306" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4224,7 +4380,7 @@
         <v>4.2</v>
       </c>
       <c r="B307" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C307" s="2" t="s">
         <v>5</v>
@@ -4239,7 +4395,7 @@
     </row>
     <row r="355" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A355" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B355" s="11" t="s">
         <v>10</v>
@@ -4251,7 +4407,7 @@
     <row r="356" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A356" s="13"/>
       <c r="B356" s="20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C356" s="21"/>
     </row>
@@ -4271,7 +4427,7 @@
         <v>22</v>
       </c>
       <c r="B358" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C358" t="s">
         <v>5</v>
@@ -4305,7 +4461,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B362" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C362" s="2" t="s">
         <v>6</v>
@@ -4317,7 +4473,7 @@
       </c>
       <c r="B363" s="7"/>
       <c r="C363" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4325,7 +4481,7 @@
         <v>3.2</v>
       </c>
       <c r="B364" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C364" s="2" t="s">
         <v>5</v>
@@ -4340,7 +4496,7 @@
     </row>
     <row r="414" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A414" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B414" s="11" t="s">
         <v>3</v>
@@ -4352,7 +4508,7 @@
     <row r="415" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A415" s="13"/>
       <c r="B415" s="17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C415" s="18"/>
     </row>
@@ -4372,7 +4528,7 @@
         <v>22</v>
       </c>
       <c r="B417" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C417" t="s">
         <v>5</v>
@@ -4392,7 +4548,7 @@
         <v>1.2</v>
       </c>
       <c r="B419" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C419" s="2" t="s">
         <v>6</v>
@@ -4420,7 +4576,7 @@
       </c>
       <c r="B422" s="7"/>
       <c r="C422" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="423" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4431,7 +4587,7 @@
         <v>7</v>
       </c>
       <c r="C423" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4446,7 +4602,7 @@
         <v>4.2</v>
       </c>
       <c r="B425" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C425" s="2" t="s">
         <v>20</v>
@@ -4481,7 +4637,7 @@
       </c>
       <c r="B429" s="7"/>
       <c r="C429" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4489,7 +4645,7 @@
         <v>6.2</v>
       </c>
       <c r="B430" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C430" s="2" t="s">
         <v>5</v>
@@ -4504,7 +4660,7 @@
     </row>
     <row r="473" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A473" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B473" s="11" t="s">
         <v>12</v>
@@ -4536,7 +4692,7 @@
         <v>22</v>
       </c>
       <c r="B476" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C476" t="s">
         <v>5</v>
@@ -4556,7 +4712,7 @@
         <v>1.2</v>
       </c>
       <c r="B478" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C478" s="2" t="s">
         <v>6</v>
@@ -4568,7 +4724,7 @@
       </c>
       <c r="B479" s="7"/>
       <c r="C479" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4576,7 +4732,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B480" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C480" s="2" t="s">
         <v>5</v>
@@ -4591,7 +4747,7 @@
     </row>
     <row r="532" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A532" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B532" s="11" t="s">
         <v>3</v>
@@ -4603,7 +4759,7 @@
     <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A533" s="13"/>
       <c r="B533" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C533" s="21"/>
     </row>
@@ -4623,7 +4779,7 @@
         <v>22</v>
       </c>
       <c r="B535" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C535" t="s">
         <v>5</v>
@@ -4643,7 +4799,7 @@
         <v>1.2</v>
       </c>
       <c r="B537" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C537" s="2" t="s">
         <v>6</v>
@@ -4655,7 +4811,7 @@
       </c>
       <c r="B538" s="7"/>
       <c r="C538" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4666,7 +4822,7 @@
         <v>7</v>
       </c>
       <c r="C539" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4681,7 +4837,7 @@
         <v>3.2</v>
       </c>
       <c r="B541" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C541" s="2" t="s">
         <v>6</v>
@@ -4693,7 +4849,7 @@
       </c>
       <c r="B542" s="7"/>
       <c r="C542" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="543" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4704,7 +4860,7 @@
         <v>7</v>
       </c>
       <c r="C543" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4713,7 +4869,7 @@
       </c>
       <c r="B544" s="7"/>
       <c r="C544" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4724,7 +4880,7 @@
         <v>23</v>
       </c>
       <c r="C545" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4739,7 +4895,7 @@
         <v>6.2</v>
       </c>
       <c r="B547" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C547" s="2" t="s">
         <v>5</v>
@@ -4754,7 +4910,7 @@
     </row>
     <row r="591" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A591" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B591" s="11" t="s">
         <v>11</v>
@@ -4766,7 +4922,7 @@
     <row r="592" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A592" s="13"/>
       <c r="B592" s="17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C592" s="18"/>
     </row>
@@ -4786,7 +4942,7 @@
         <v>22</v>
       </c>
       <c r="B594" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C594" t="s">
         <v>5</v>
@@ -4806,7 +4962,7 @@
         <v>1.2</v>
       </c>
       <c r="B596" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C596" s="2" t="s">
         <v>14</v>
@@ -4826,7 +4982,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B598" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C598" s="2" t="s">
         <v>30</v>
@@ -4846,7 +5002,7 @@
         <v>3.2</v>
       </c>
       <c r="B600" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C600" s="2" t="s">
         <v>6</v>
@@ -4858,14 +5014,14 @@
       </c>
       <c r="B601" s="7"/>
       <c r="C601" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="602" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A602" s="3"/>
       <c r="B602" s="7"/>
       <c r="C602" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4887,7 +5043,7 @@
         <v>5.2</v>
       </c>
       <c r="B605" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C605" s="2" t="s">
         <v>5</v>
@@ -4902,7 +5058,7 @@
     </row>
     <row r="650" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A650" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B650" s="11" t="s">
         <v>13</v>
@@ -4914,7 +5070,7 @@
     <row r="651" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A651" s="13"/>
       <c r="B651" s="20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C651" s="21"/>
     </row>
@@ -4934,7 +5090,7 @@
         <v>22</v>
       </c>
       <c r="B653" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C653" t="s">
         <v>5</v>
@@ -4954,7 +5110,7 @@
         <v>1.2</v>
       </c>
       <c r="B655" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C655" s="2" t="s">
         <v>6</v>
@@ -4966,7 +5122,7 @@
       </c>
       <c r="B656" s="7"/>
       <c r="C656" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="657" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4986,7 +5142,7 @@
       </c>
       <c r="B658" s="7"/>
       <c r="C658" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="659" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4997,7 +5153,7 @@
         <v>23</v>
       </c>
       <c r="C659" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="660" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5012,7 +5168,7 @@
         <v>4.2</v>
       </c>
       <c r="B661" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C661" s="2" t="s">
         <v>5</v>
@@ -5027,7 +5183,7 @@
     </row>
     <row r="709" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A709" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B709" s="11" t="s">
         <v>11</v>
@@ -5039,7 +5195,7 @@
     <row r="710" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A710" s="13"/>
       <c r="B710" s="20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C710" s="21"/>
     </row>
@@ -5059,7 +5215,7 @@
         <v>22</v>
       </c>
       <c r="B712" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C712" t="s">
         <v>5</v>
@@ -5079,7 +5235,7 @@
         <v>1.2</v>
       </c>
       <c r="B714" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C714" s="2" t="s">
         <v>14</v>
@@ -5099,7 +5255,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B716" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C716" s="2" t="s">
         <v>30</v>
@@ -5131,7 +5287,7 @@
       </c>
       <c r="B719" s="7"/>
       <c r="C719" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="720" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5142,7 +5298,7 @@
         <v>23</v>
       </c>
       <c r="C720" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="721" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5157,7 +5313,7 @@
         <v>5.2</v>
       </c>
       <c r="B722" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C722" s="2" t="s">
         <v>5</v>
@@ -5172,7 +5328,7 @@
     </row>
     <row r="768" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A768" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B768" s="11" t="s">
         <v>13</v>
@@ -5204,7 +5360,7 @@
         <v>22</v>
       </c>
       <c r="B771" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C771" t="s">
         <v>5</v>
@@ -5224,7 +5380,7 @@
         <v>1.2</v>
       </c>
       <c r="B773" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C773" s="2" t="s">
         <v>26</v>
@@ -5242,10 +5398,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B775" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C775" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="776" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5254,7 +5410,7 @@
       </c>
       <c r="B776" s="7"/>
       <c r="C776" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="777" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5276,7 +5432,7 @@
         <v>4.2</v>
       </c>
       <c r="B779" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C779" s="2" t="s">
         <v>5</v>
@@ -5291,7 +5447,7 @@
     </row>
     <row r="827" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A827" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B827" s="11" t="s">
         <v>3</v>
@@ -5303,7 +5459,7 @@
     <row r="828" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A828" s="13"/>
       <c r="B828" s="20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C828" s="21"/>
     </row>
@@ -5323,7 +5479,7 @@
         <v>22</v>
       </c>
       <c r="B830" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C830" t="s">
         <v>5</v>
@@ -5343,7 +5499,7 @@
         <v>1.2</v>
       </c>
       <c r="B832" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C832" s="2" t="s">
         <v>14</v>
@@ -5363,7 +5519,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B834" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C834" s="2" t="s">
         <v>30</v>
@@ -5395,21 +5551,21 @@
       </c>
       <c r="B837" s="7"/>
       <c r="C837" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="838" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A838" s="3"/>
       <c r="B838" s="7"/>
       <c r="C838" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="839" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A839" s="3"/>
       <c r="B839" s="7"/>
       <c r="C839" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5438,7 +5594,7 @@
         <v>23</v>
       </c>
       <c r="C842" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5453,7 +5609,7 @@
         <v>6.2</v>
       </c>
       <c r="B844" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C844" s="2" t="s">
         <v>5</v>
@@ -5468,7 +5624,7 @@
     </row>
     <row r="886" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A886" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B886" s="11" t="s">
         <v>9</v>
@@ -5500,7 +5656,7 @@
         <v>22</v>
       </c>
       <c r="B889" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C889" t="s">
         <v>5</v>
@@ -5520,7 +5676,7 @@
         <v>1.2</v>
       </c>
       <c r="B891" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C891" s="2" t="s">
         <v>26</v>
@@ -5538,7 +5694,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B893" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C893" s="2" t="s">
         <v>18</v>
@@ -5556,7 +5712,7 @@
         <v>3.2</v>
       </c>
       <c r="B895" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C895" s="2" t="s">
         <v>19</v>
@@ -5574,10 +5730,10 @@
         <v>4.2</v>
       </c>
       <c r="B897" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C897" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="898" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5586,7 +5742,7 @@
       </c>
       <c r="B898" s="7"/>
       <c r="C898" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="899" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5608,10 +5764,10 @@
         <v>6.2</v>
       </c>
       <c r="B901" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C901" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="902" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5626,10 +5782,10 @@
         <v>7.2</v>
       </c>
       <c r="B903" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C903" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="904" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5644,7 +5800,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B905" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C905" s="2" t="s">
         <v>5</v>
@@ -5662,7 +5818,7 @@
         <v>15</v>
       </c>
       <c r="B945" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C945" s="12" t="s">
         <v>4</v>
@@ -5691,7 +5847,7 @@
         <v>22</v>
       </c>
       <c r="B948" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C948" t="s">
         <v>5</v>
@@ -5703,7 +5859,7 @@
       </c>
       <c r="B949" s="7"/>
       <c r="C949" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="950" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5711,7 +5867,7 @@
         <v>1.2</v>
       </c>
       <c r="B950" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C950" s="2" t="s">
         <v>6</v>
@@ -5723,7 +5879,7 @@
       </c>
       <c r="B951" s="7"/>
       <c r="C951" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="952" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5739,14 +5895,14 @@
       </c>
       <c r="B953" s="7"/>
       <c r="C953" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="954" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A954" s="3"/>
       <c r="B954" s="7"/>
       <c r="C954" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="955" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5762,7 +5918,7 @@
       </c>
       <c r="B956" s="7"/>
       <c r="C956" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="957" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5770,7 +5926,7 @@
         <v>4.2</v>
       </c>
       <c r="B957" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C957" s="2" t="s">
         <v>5</v>
@@ -5785,7 +5941,7 @@
     </row>
     <row r="1004" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1004" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B1004" s="11" t="s">
         <v>9</v>
@@ -5817,7 +5973,7 @@
         <v>22</v>
       </c>
       <c r="B1007" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1007" t="s">
         <v>5</v>
@@ -5837,7 +5993,7 @@
         <v>1.2</v>
       </c>
       <c r="B1009" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1009" s="2" t="s">
         <v>6</v>
@@ -5869,7 +6025,7 @@
         <v>3.2</v>
       </c>
       <c r="B1013" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C1013" s="2" t="s">
         <v>18</v>
@@ -5887,7 +6043,7 @@
         <v>4.2</v>
       </c>
       <c r="B1015" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C1015" s="2" t="s">
         <v>19</v>
@@ -5899,7 +6055,7 @@
       </c>
       <c r="B1016" s="7"/>
       <c r="C1016" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="1017" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5921,10 +6077,10 @@
         <v>6.2</v>
       </c>
       <c r="B1019" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C1019" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="1020" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5939,10 +6095,10 @@
         <v>7.2</v>
       </c>
       <c r="B1021" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C1021" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="1022" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5957,7 +6113,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B1023" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1023" s="2" t="s">
         <v>5</v>
@@ -5972,7 +6128,7 @@
     </row>
     <row r="1063" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1063" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1063" s="11" t="s">
         <v>13</v>
@@ -5984,7 +6140,7 @@
     <row r="1064" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1064" s="13"/>
       <c r="B1064" s="20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C1064" s="21"/>
     </row>
@@ -6004,7 +6160,7 @@
         <v>22</v>
       </c>
       <c r="B1066" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1066" t="s">
         <v>5</v>
@@ -6024,7 +6180,7 @@
         <v>1.2</v>
       </c>
       <c r="B1068" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1068" s="2" t="s">
         <v>6</v>
@@ -6036,7 +6192,7 @@
       </c>
       <c r="B1069" s="7"/>
       <c r="C1069" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="1070" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6056,7 +6212,7 @@
       </c>
       <c r="B1071" s="7"/>
       <c r="C1071" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="1072" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6067,7 +6223,7 @@
         <v>23</v>
       </c>
       <c r="C1072" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="1073" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6082,7 +6238,7 @@
         <v>4.2</v>
       </c>
       <c r="B1074" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1074" s="2" t="s">
         <v>5</v>
@@ -6097,10 +6253,10 @@
     </row>
     <row r="1122" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1122" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B1122" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C1122" s="12" t="s">
         <v>16</v>
@@ -6109,7 +6265,7 @@
     <row r="1123" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1123" s="13"/>
       <c r="B1123" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C1123" s="21"/>
     </row>
@@ -6129,7 +6285,7 @@
         <v>22</v>
       </c>
       <c r="B1125" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1125" t="s">
         <v>5</v>
@@ -6149,7 +6305,7 @@
         <v>1.2</v>
       </c>
       <c r="B1127" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1127" s="2" t="s">
         <v>6</v>
@@ -6161,7 +6317,7 @@
       </c>
       <c r="B1128" s="7"/>
       <c r="C1128" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="1129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6181,7 +6337,7 @@
       </c>
       <c r="B1130" s="7"/>
       <c r="C1130" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="1131" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6203,7 +6359,7 @@
         <v>4.2</v>
       </c>
       <c r="B1133" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1133" s="2" t="s">
         <v>6</v>
@@ -6215,7 +6371,7 @@
       </c>
       <c r="B1134" s="7"/>
       <c r="C1134" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="1135" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6231,14 +6387,14 @@
       </c>
       <c r="B1136" s="7"/>
       <c r="C1136" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="1137" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1137" s="3"/>
       <c r="B1137" s="7"/>
       <c r="C1137" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="1138" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6254,7 +6410,7 @@
       </c>
       <c r="B1139" s="7"/>
       <c r="C1139" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="1140" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6262,7 +6418,7 @@
         <v>7.2</v>
       </c>
       <c r="B1140" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1140" s="2" t="s">
         <v>5</v>
@@ -6277,7 +6433,7 @@
     </row>
     <row r="1181" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1181" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B1181" s="11" t="s">
         <v>13</v>
@@ -6289,7 +6445,7 @@
     <row r="1182" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1182" s="13"/>
       <c r="B1182" s="20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C1182" s="21"/>
     </row>
@@ -6309,7 +6465,7 @@
         <v>22</v>
       </c>
       <c r="B1184" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1184" t="s">
         <v>5</v>
@@ -6329,7 +6485,7 @@
         <v>1.2</v>
       </c>
       <c r="B1186" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1186" s="2" t="s">
         <v>6</v>
@@ -6357,7 +6513,7 @@
       </c>
       <c r="B1189" s="7"/>
       <c r="C1189" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="1190" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6377,7 +6533,7 @@
       </c>
       <c r="B1191" s="7"/>
       <c r="C1191" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="1192" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6385,7 +6541,7 @@
         <v>4.2</v>
       </c>
       <c r="B1192" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1192" s="2" t="s">
         <v>5</v>
@@ -6400,7 +6556,7 @@
     </row>
     <row r="1240" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1240" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B1240" s="11" t="s">
         <v>11</v>
@@ -6412,7 +6568,7 @@
     <row r="1241" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1241" s="13"/>
       <c r="B1241" s="20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C1241" s="21"/>
     </row>
@@ -6432,7 +6588,7 @@
         <v>22</v>
       </c>
       <c r="B1243" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1243" t="s">
         <v>5</v>
@@ -6452,7 +6608,7 @@
         <v>1.2</v>
       </c>
       <c r="B1245" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1245" s="2" t="s">
         <v>14</v>
@@ -6472,7 +6628,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1247" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1247" s="2" t="s">
         <v>30</v>
@@ -6500,7 +6656,7 @@
       </c>
       <c r="B1250" s="7"/>
       <c r="C1250" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="1251" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6520,7 +6676,7 @@
       </c>
       <c r="B1252" s="7"/>
       <c r="C1252" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="1253" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6528,7 +6684,7 @@
         <v>5.2</v>
       </c>
       <c r="B1253" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1253" s="2" t="s">
         <v>5</v>
@@ -6543,7 +6699,7 @@
     </row>
     <row r="1299" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1299" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1299" s="11" t="s">
         <v>11</v>
@@ -6555,7 +6711,7 @@
     <row r="1300" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1300" s="13"/>
       <c r="B1300" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C1300" s="21"/>
     </row>
@@ -6575,7 +6731,7 @@
         <v>22</v>
       </c>
       <c r="B1302" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1302" t="s">
         <v>5</v>
@@ -6595,7 +6751,7 @@
         <v>1.2</v>
       </c>
       <c r="B1304" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1304" s="2" t="s">
         <v>14</v>
@@ -6615,7 +6771,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1306" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1306" s="2" t="s">
         <v>30</v>
@@ -6643,7 +6799,7 @@
       </c>
       <c r="B1309" s="7"/>
       <c r="C1309" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="1310" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6663,7 +6819,7 @@
       </c>
       <c r="B1311" s="7"/>
       <c r="C1311" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="1312" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6671,7 +6827,7 @@
         <v>5.2</v>
       </c>
       <c r="B1312" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1312" s="2" t="s">
         <v>5</v>
@@ -6686,7 +6842,7 @@
     </row>
     <row r="1358" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1358" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B1358" s="11" t="s">
         <v>3</v>
@@ -6698,7 +6854,7 @@
     <row r="1359" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1359" s="13"/>
       <c r="B1359" s="20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C1359" s="21"/>
     </row>
@@ -6718,7 +6874,7 @@
         <v>22</v>
       </c>
       <c r="B1361" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1361" t="s">
         <v>5</v>
@@ -6738,7 +6894,7 @@
         <v>1.2</v>
       </c>
       <c r="B1363" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1363" s="2" t="s">
         <v>6</v>
@@ -6766,7 +6922,7 @@
       </c>
       <c r="B1366" s="7"/>
       <c r="C1366" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="1367" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6777,7 +6933,7 @@
         <v>7</v>
       </c>
       <c r="C1367" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="1368" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6792,7 +6948,7 @@
         <v>4.2</v>
       </c>
       <c r="B1369" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C1369" s="2" t="s">
         <v>20</v>
@@ -6809,7 +6965,7 @@
       </c>
       <c r="B1371" s="7"/>
       <c r="C1371" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="1372" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6829,7 +6985,7 @@
       </c>
       <c r="B1373" s="7"/>
       <c r="C1373" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="1374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6837,7 +6993,7 @@
         <v>6.2</v>
       </c>
       <c r="B1374" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1374" s="2" t="s">
         <v>5</v>
@@ -6852,7 +7008,7 @@
     </row>
     <row r="1417" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1417" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B1417" s="11" t="s">
         <v>11</v>
@@ -6864,7 +7020,7 @@
     <row r="1418" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1418" s="13"/>
       <c r="B1418" s="20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C1418" s="21"/>
     </row>
@@ -6884,7 +7040,7 @@
         <v>22</v>
       </c>
       <c r="B1420" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1420" t="s">
         <v>5</v>
@@ -6904,10 +7060,10 @@
         <v>1.2</v>
       </c>
       <c r="B1422" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1422" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="1423" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6924,7 +7080,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1424" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1424" s="2" t="s">
         <v>6</v>
@@ -6936,7 +7092,7 @@
       </c>
       <c r="B1425" s="7"/>
       <c r="C1425" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="1426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6947,7 +7103,7 @@
         <v>7</v>
       </c>
       <c r="C1426" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="1427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6956,7 +7112,7 @@
       </c>
       <c r="B1427" s="7"/>
       <c r="C1427" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="1428" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6967,7 +7123,7 @@
         <v>23</v>
       </c>
       <c r="C1428" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="1429" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6982,7 +7138,7 @@
         <v>5.2</v>
       </c>
       <c r="B1430" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1430" s="2" t="s">
         <v>5</v>
@@ -6997,7 +7153,7 @@
     </row>
     <row r="1476" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1476" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B1476" s="11" t="s">
         <v>11</v>
@@ -7009,7 +7165,7 @@
     <row r="1477" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1477" s="13"/>
       <c r="B1477" s="17" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C1477" s="18"/>
     </row>
@@ -7029,7 +7185,7 @@
         <v>22</v>
       </c>
       <c r="B1479" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1479" t="s">
         <v>5</v>
@@ -7049,7 +7205,7 @@
         <v>1.2</v>
       </c>
       <c r="B1481" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1481" s="2" t="s">
         <v>26</v>
@@ -7067,10 +7223,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1483" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C1483" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="1484" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7085,10 +7241,10 @@
         <v>3.2</v>
       </c>
       <c r="B1485" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C1485" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="1486" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7097,7 +7253,7 @@
       </c>
       <c r="B1486" s="7"/>
       <c r="C1486" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="1487" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7105,10 +7261,10 @@
         <v>4.2</v>
       </c>
       <c r="B1487" s="22" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C1487" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="1488" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7128,7 +7284,7 @@
         <v>5.2</v>
       </c>
       <c r="B1490" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1490" s="2" t="s">
         <v>5</v>
@@ -7143,7 +7299,7 @@
     </row>
     <row r="1535" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1535" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B1535" s="11" t="s">
         <v>3</v>
@@ -7155,7 +7311,7 @@
     <row r="1536" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1536" s="13"/>
       <c r="B1536" s="20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C1536" s="21"/>
     </row>
@@ -7175,7 +7331,7 @@
         <v>22</v>
       </c>
       <c r="B1538" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1538" t="s">
         <v>5</v>
@@ -7195,7 +7351,7 @@
         <v>1.2</v>
       </c>
       <c r="B1540" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1540" s="2" t="s">
         <v>6</v>
@@ -7207,7 +7363,7 @@
       </c>
       <c r="B1541" s="7"/>
       <c r="C1541" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="1542" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7227,21 +7383,21 @@
       </c>
       <c r="B1543" s="7"/>
       <c r="C1543" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="1544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1544" s="3"/>
       <c r="B1544" s="7"/>
       <c r="C1544" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="1545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1545" s="3"/>
       <c r="B1545" s="7"/>
       <c r="C1545" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="1546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7252,7 +7408,7 @@
         <v>23</v>
       </c>
       <c r="C1546" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="1547" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7267,7 +7423,7 @@
         <v>4.2</v>
       </c>
       <c r="B1548" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C1548" s="2" t="s">
         <v>6</v>
@@ -7284,7 +7440,7 @@
       </c>
       <c r="B1550" s="7"/>
       <c r="C1550" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="1551" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7292,10 +7448,10 @@
         <v>5.2</v>
       </c>
       <c r="B1551" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C1551" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="1552" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7315,7 +7471,7 @@
         <v>6.2</v>
       </c>
       <c r="B1554" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1554" s="2" t="s">
         <v>5</v>
@@ -7330,7 +7486,7 @@
     </row>
     <row r="1594" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1594" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B1594" s="11" t="s">
         <v>11</v>
@@ -7342,7 +7498,7 @@
     <row r="1595" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1595" s="13"/>
       <c r="B1595" s="20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C1595" s="21"/>
     </row>
@@ -7362,7 +7518,7 @@
         <v>22</v>
       </c>
       <c r="B1597" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1597" t="s">
         <v>5</v>
@@ -7382,7 +7538,7 @@
         <v>1.2</v>
       </c>
       <c r="B1599" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1599" s="2" t="s">
         <v>6</v>
@@ -7410,7 +7566,7 @@
       </c>
       <c r="B1602" s="7"/>
       <c r="C1602" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="1603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7430,7 +7586,7 @@
       </c>
       <c r="B1604" s="7"/>
       <c r="C1604" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="1605" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7441,7 +7597,7 @@
         <v>23</v>
       </c>
       <c r="C1605" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="1606" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7456,7 +7612,7 @@
         <v>5.2</v>
       </c>
       <c r="B1607" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1607" s="2" t="s">
         <v>5</v>
@@ -7471,7 +7627,7 @@
     </row>
     <row r="1653" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1653" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B1653" s="11" t="s">
         <v>12</v>
@@ -7483,7 +7639,7 @@
     <row r="1654" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1654" s="13"/>
       <c r="B1654" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C1654" s="18"/>
     </row>
@@ -7503,7 +7659,7 @@
         <v>22</v>
       </c>
       <c r="B1656" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1656" t="s">
         <v>5</v>
@@ -7523,7 +7679,7 @@
         <v>1.2</v>
       </c>
       <c r="B1658" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1658" s="2" t="s">
         <v>26</v>
@@ -7535,7 +7691,7 @@
       </c>
       <c r="B1659" s="7"/>
       <c r="C1659" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="1660" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7543,7 +7699,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1660" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1660" s="2" t="s">
         <v>5</v>
@@ -7558,7 +7714,7 @@
     </row>
     <row r="1712" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1712" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B1712" s="11" t="s">
         <v>12</v>
@@ -7590,7 +7746,7 @@
         <v>22</v>
       </c>
       <c r="B1715" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1715" t="s">
         <v>5</v>
@@ -7618,7 +7774,7 @@
       </c>
       <c r="B1718" s="7"/>
       <c r="C1718" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="1719" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7626,7 +7782,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1719" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1719" s="2" t="s">
         <v>5</v>
@@ -7641,7 +7797,7 @@
     </row>
     <row r="1771" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1771" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B1771" s="11" t="s">
         <v>13</v>
@@ -7653,7 +7809,7 @@
     <row r="1772" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1772" s="13"/>
       <c r="B1772" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C1772" s="18"/>
     </row>
@@ -7673,7 +7829,7 @@
         <v>22</v>
       </c>
       <c r="B1774" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1774" t="s">
         <v>5</v>
@@ -7693,7 +7849,7 @@
         <v>1.2</v>
       </c>
       <c r="B1776" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1776" s="2" t="s">
         <v>14</v>
@@ -7713,7 +7869,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1778" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1778" s="2" t="s">
         <v>30</v>
@@ -7745,7 +7901,7 @@
       </c>
       <c r="B1781" s="7"/>
       <c r="C1781" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="1782" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7753,7 +7909,7 @@
         <v>4.2</v>
       </c>
       <c r="B1782" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1782" s="2" t="s">
         <v>5</v>
@@ -7768,7 +7924,7 @@
     </row>
     <row r="1830" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1830" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B1830" s="11" t="s">
         <v>3</v>
@@ -7780,7 +7936,7 @@
     <row r="1831" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1831" s="13"/>
       <c r="B1831" s="20" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C1831" s="21"/>
     </row>
@@ -7800,7 +7956,7 @@
         <v>22</v>
       </c>
       <c r="B1833" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1833" t="s">
         <v>5</v>
@@ -7820,7 +7976,7 @@
         <v>1.2</v>
       </c>
       <c r="B1835" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1835" s="2" t="s">
         <v>14</v>
@@ -7840,7 +7996,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1837" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1837" s="2" t="s">
         <v>30</v>
@@ -7866,7 +8022,7 @@
       </c>
       <c r="B1840" s="7"/>
       <c r="C1840" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="1841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7877,7 +8033,7 @@
         <v>31</v>
       </c>
       <c r="C1841" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="1842" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7895,7 +8051,7 @@
         <v>32</v>
       </c>
       <c r="C1843" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="1844" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7910,7 +8066,7 @@
         <v>6.2</v>
       </c>
       <c r="B1845" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1845" s="2" t="s">
         <v>5</v>
@@ -7925,7 +8081,7 @@
     </row>
     <row r="1889" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1889" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B1889" s="11" t="s">
         <v>12</v>
@@ -7957,7 +8113,7 @@
         <v>22</v>
       </c>
       <c r="B1892" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1892" t="s">
         <v>5</v>
@@ -7985,7 +8141,7 @@
       </c>
       <c r="B1895" s="7"/>
       <c r="C1895" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="1896" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7993,7 +8149,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B1896" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1896" s="2" t="s">
         <v>5</v>
@@ -8008,7 +8164,7 @@
     </row>
     <row r="1948" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1948" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B1948" s="11" t="s">
         <v>9</v>
@@ -8040,7 +8196,7 @@
         <v>22</v>
       </c>
       <c r="B1951" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1951" t="s">
         <v>5</v>
@@ -8060,7 +8216,7 @@
         <v>1.2</v>
       </c>
       <c r="B1953" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1953" s="2" t="s">
         <v>6</v>
@@ -8092,7 +8248,7 @@
         <v>3.2</v>
       </c>
       <c r="B1957" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C1957" s="2" t="s">
         <v>18</v>
@@ -8110,7 +8266,7 @@
         <v>4.2</v>
       </c>
       <c r="B1959" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C1959" s="2" t="s">
         <v>19</v>
@@ -8122,7 +8278,7 @@
       </c>
       <c r="B1960" s="7"/>
       <c r="C1960" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="1961" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8144,10 +8300,10 @@
         <v>6.2</v>
       </c>
       <c r="B1963" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C1963" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="1964" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8162,10 +8318,10 @@
         <v>7.2</v>
       </c>
       <c r="B1965" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C1965" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="1966" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8180,7 +8336,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="B1967" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C1967" s="2" t="s">
         <v>5</v>
@@ -8195,7 +8351,7 @@
     </row>
     <row r="2007" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2007" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B2007" s="11" t="s">
         <v>13</v>
@@ -8207,7 +8363,7 @@
     <row r="2008" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2008" s="13"/>
       <c r="B2008" s="20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C2008" s="21"/>
     </row>
@@ -8227,7 +8383,7 @@
         <v>22</v>
       </c>
       <c r="B2010" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2010" t="s">
         <v>5</v>
@@ -8247,7 +8403,7 @@
         <v>1.2</v>
       </c>
       <c r="B2012" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2012" s="2" t="s">
         <v>6</v>
@@ -8259,7 +8415,7 @@
       </c>
       <c r="B2013" s="7"/>
       <c r="C2013" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2014" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8279,7 +8435,7 @@
       </c>
       <c r="B2015" s="7"/>
       <c r="C2015" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2016" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8290,7 +8446,7 @@
         <v>23</v>
       </c>
       <c r="C2016" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2017" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8305,7 +8461,7 @@
         <v>4.2</v>
       </c>
       <c r="B2018" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2018" s="2" t="s">
         <v>5</v>
@@ -8320,10 +8476,10 @@
     </row>
     <row r="2066" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2066" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B2066" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2066" s="12" t="s">
         <v>16</v>
@@ -8332,7 +8488,7 @@
     <row r="2067" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2067" s="13"/>
       <c r="B2067" s="17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C2067" s="18"/>
     </row>
@@ -8352,7 +8508,7 @@
         <v>22</v>
       </c>
       <c r="B2069" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2069" t="s">
         <v>5</v>
@@ -8372,7 +8528,7 @@
         <v>1.2</v>
       </c>
       <c r="B2071" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2071" s="2" t="s">
         <v>6</v>
@@ -8384,7 +8540,7 @@
       </c>
       <c r="B2072" s="7"/>
       <c r="C2072" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2073" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8404,7 +8560,7 @@
       </c>
       <c r="B2074" s="7"/>
       <c r="C2074" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2075" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8426,7 +8582,7 @@
         <v>4.2</v>
       </c>
       <c r="B2077" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2077" s="2" t="s">
         <v>6</v>
@@ -8438,7 +8594,7 @@
       </c>
       <c r="B2078" s="7"/>
       <c r="C2078" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2079" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8454,14 +8610,14 @@
       </c>
       <c r="B2080" s="7"/>
       <c r="C2080" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2081" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2081" s="3"/>
       <c r="B2081" s="7"/>
       <c r="C2081" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2082" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8477,7 +8633,7 @@
       </c>
       <c r="B2083" s="7"/>
       <c r="C2083" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2084" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8485,7 +8641,7 @@
         <v>7.2</v>
       </c>
       <c r="B2084" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2084" s="2" t="s">
         <v>5</v>
@@ -8500,7 +8656,7 @@
     </row>
     <row r="2125" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2125" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B2125" s="11" t="s">
         <v>10</v>
@@ -8512,7 +8668,7 @@
     <row r="2126" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2126" s="13"/>
       <c r="B2126" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C2126" s="18"/>
     </row>
@@ -8532,7 +8688,7 @@
         <v>22</v>
       </c>
       <c r="B2128" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2128" t="s">
         <v>5</v>
@@ -8552,7 +8708,7 @@
         <v>1.2</v>
       </c>
       <c r="B2130" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2130" s="2" t="s">
         <v>6</v>
@@ -8564,7 +8720,7 @@
       </c>
       <c r="B2131" s="7"/>
       <c r="C2131" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2132" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8584,7 +8740,7 @@
       </c>
       <c r="B2133" s="7"/>
       <c r="C2133" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2134" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8592,7 +8748,7 @@
         <v>3.2</v>
       </c>
       <c r="B2134" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2134" s="2" t="s">
         <v>5</v>
@@ -8619,7 +8775,7 @@
     <row r="2185" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2185" s="13"/>
       <c r="B2185" s="17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C2185" s="18"/>
     </row>
@@ -8639,7 +8795,7 @@
         <v>22</v>
       </c>
       <c r="B2187" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2187" t="s">
         <v>5</v>
@@ -8659,7 +8815,7 @@
         <v>1.2</v>
       </c>
       <c r="B2189" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2189" s="2" t="s">
         <v>14</v>
@@ -8679,7 +8835,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B2191" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2191" s="2" t="s">
         <v>30</v>
@@ -8711,7 +8867,7 @@
       </c>
       <c r="B2194" s="7"/>
       <c r="C2194" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2195" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8719,7 +8875,7 @@
         <v>4.2</v>
       </c>
       <c r="B2195" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2195" s="2" t="s">
         <v>5</v>
@@ -8734,7 +8890,7 @@
     </row>
     <row r="2243" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2243" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B2243" s="11" t="s">
         <v>10</v>
@@ -8746,7 +8902,7 @@
     <row r="2244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2244" s="13"/>
       <c r="B2244" s="17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C2244" s="18"/>
     </row>
@@ -8766,7 +8922,7 @@
         <v>22</v>
       </c>
       <c r="B2246" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2246" t="s">
         <v>5</v>
@@ -8800,7 +8956,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B2250" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C2250" s="2" t="s">
         <v>6</v>
@@ -8812,7 +8968,7 @@
       </c>
       <c r="B2251" s="7"/>
       <c r="C2251" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2252" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8820,7 +8976,7 @@
         <v>3.2</v>
       </c>
       <c r="B2252" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2252" s="2" t="s">
         <v>5</v>
@@ -8847,7 +9003,7 @@
     <row r="2303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2303" s="13"/>
       <c r="B2303" s="20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C2303" s="21"/>
     </row>
@@ -8867,7 +9023,7 @@
         <v>22</v>
       </c>
       <c r="B2305" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2305" t="s">
         <v>5</v>
@@ -8887,7 +9043,7 @@
         <v>1.2</v>
       </c>
       <c r="B2307" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2307" s="2" t="s">
         <v>6</v>
@@ -8915,7 +9071,7 @@
       </c>
       <c r="B2310" s="7"/>
       <c r="C2310" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2311" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8926,7 +9082,7 @@
         <v>7</v>
       </c>
       <c r="C2311" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2312" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8941,7 +9097,7 @@
         <v>4.2</v>
       </c>
       <c r="B2313" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2313" s="2" t="s">
         <v>20</v>
@@ -8976,7 +9132,7 @@
       </c>
       <c r="B2317" s="7"/>
       <c r="C2317" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2318" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8984,7 +9140,7 @@
         <v>6.2</v>
       </c>
       <c r="B2318" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2318" s="2" t="s">
         <v>5</v>
@@ -8999,7 +9155,7 @@
     </row>
     <row r="2361" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2361" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B2361" s="11" t="s">
         <v>12</v>
@@ -9031,7 +9187,7 @@
         <v>22</v>
       </c>
       <c r="B2364" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2364" t="s">
         <v>5</v>
@@ -9051,7 +9207,7 @@
         <v>1.2</v>
       </c>
       <c r="B2366" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2366" s="2" t="s">
         <v>6</v>
@@ -9063,7 +9219,7 @@
       </c>
       <c r="B2367" s="7"/>
       <c r="C2367" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2368" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9071,7 +9227,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B2368" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2368" s="2" t="s">
         <v>5</v>
@@ -9098,7 +9254,7 @@
     <row r="2421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2421" s="13"/>
       <c r="B2421" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C2421" s="21"/>
     </row>
@@ -9118,7 +9274,7 @@
         <v>22</v>
       </c>
       <c r="B2423" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2423" t="s">
         <v>5</v>
@@ -9138,7 +9294,7 @@
         <v>1.2</v>
       </c>
       <c r="B2425" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2425" s="2" t="s">
         <v>6</v>
@@ -9150,7 +9306,7 @@
       </c>
       <c r="B2426" s="7"/>
       <c r="C2426" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9161,7 +9317,7 @@
         <v>7</v>
       </c>
       <c r="C2427" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2428" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9176,7 +9332,7 @@
         <v>3.2</v>
       </c>
       <c r="B2429" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2429" s="2" t="s">
         <v>6</v>
@@ -9188,7 +9344,7 @@
       </c>
       <c r="B2430" s="7"/>
       <c r="C2430" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2431" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9199,7 +9355,7 @@
         <v>7</v>
       </c>
       <c r="C2431" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2432" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9208,7 +9364,7 @@
       </c>
       <c r="B2432" s="7"/>
       <c r="C2432" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2433" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9219,7 +9375,7 @@
         <v>23</v>
       </c>
       <c r="C2433" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2434" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9234,7 +9390,7 @@
         <v>6.2</v>
       </c>
       <c r="B2435" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C2435" s="2" t="s">
         <v>5</v>
@@ -9247,8 +9403,555 @@
       <c r="B2436" s="9"/>
       <c r="C2436" s="8"/>
     </row>
+    <row r="2479" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2479" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2479" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2479" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2480" s="13"/>
+      <c r="B2480" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C2480" s="18"/>
+    </row>
+    <row r="2481" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2481" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2481" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2481" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2482" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2482" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2482" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2482" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2483" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2483" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2483" s="7"/>
+      <c r="C2483" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2484" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2484" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B2484" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2484" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2485" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2485" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B2485" s="7"/>
+      <c r="C2485" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2486" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2486" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B2486" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2486" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2487" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2487" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B2487" s="7"/>
+      <c r="C2487" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2488" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2488" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B2488" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2488" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2489" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2489" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B2489" s="7"/>
+      <c r="C2489" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2490" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2490" s="3"/>
+      <c r="B2490" s="7"/>
+      <c r="C2490" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2491" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2491" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B2491" s="7"/>
+      <c r="C2491" s="2"/>
+    </row>
+    <row r="2492" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2492" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B2492" s="7"/>
+      <c r="C2492" s="2"/>
+    </row>
+    <row r="2493" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2493" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B2493" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2493" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2494" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2494" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2494" s="9"/>
+      <c r="C2494" s="8"/>
+    </row>
+    <row r="2538" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2538" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2538" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2538" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2539" s="13"/>
+      <c r="B2539" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2539" s="21"/>
+    </row>
+    <row r="2540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2540" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2540" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2540" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2541" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2541" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2541" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2541" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2542" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2542" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2542" s="7"/>
+      <c r="C2542" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2543" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2543" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B2543" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2543" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2544" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2544" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B2544" s="7"/>
+      <c r="C2544" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2545" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2545" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B2545" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2545" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2546" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2546" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B2546" s="7"/>
+      <c r="C2546" s="22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2547" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2547" s="3"/>
+      <c r="B2547" s="7"/>
+      <c r="C2547" s="22"/>
+    </row>
+    <row r="2548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2548" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B2548" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2548" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2549" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2549" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B2549" s="7"/>
+      <c r="C2549" s="2"/>
+    </row>
+    <row r="2550" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2550" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B2550" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2550" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2551" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2551" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2551" s="9"/>
+      <c r="C2551" s="8"/>
+    </row>
+    <row r="2597" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2597" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2597" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2597" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2598" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2598" s="13"/>
+      <c r="B2598" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2598" s="21"/>
+    </row>
+    <row r="2599" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2599" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2599" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2599" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2600" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2600" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2600" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2600" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2601" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2601" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2601" s="7"/>
+      <c r="C2601" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2602" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2602" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B2602" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2602" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2603" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B2603" s="7"/>
+      <c r="C2603" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2604" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2604" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B2604" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2604" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2605" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2605" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B2605" s="7"/>
+      <c r="C2605" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2606" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2606" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B2606" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2606" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2607" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2607" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B2607" s="7"/>
+      <c r="C2607" s="22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2608" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2608" s="3"/>
+      <c r="B2608" s="7"/>
+      <c r="C2608" s="22"/>
+    </row>
+    <row r="2609" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2609" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B2609" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2609" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2610" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2610" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B2610" s="7"/>
+      <c r="C2610" s="2"/>
+    </row>
+    <row r="2611" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2611" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B2611" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2611" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2612" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2612" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2612" s="9"/>
+      <c r="C2612" s="8"/>
+    </row>
+    <row r="2656" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2656" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2656" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2656" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2657" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2657" s="13"/>
+      <c r="B2657" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2657" s="18"/>
+    </row>
+    <row r="2658" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2658" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2658" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2658" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2659" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2659" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2659" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2659" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2660" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2660" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2660" s="7"/>
+      <c r="C2660" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2661" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2661" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B2661" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2661" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2662" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2662" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B2662" s="7"/>
+      <c r="C2662" s="2"/>
+    </row>
+    <row r="2663" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2663" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B2663" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2663" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2664" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2664" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B2664" s="7"/>
+      <c r="C2664" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2665" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2665" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B2665" s="7"/>
+      <c r="C2665" s="2"/>
+    </row>
+    <row r="2666" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2666" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B2666" s="7"/>
+      <c r="C2666" s="2"/>
+    </row>
+    <row r="2667" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2667" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B2667" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2667" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2668" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2668" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2668" s="9"/>
+      <c r="C2668" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="30">
     <mergeCell ref="B120:C120"/>
     <mergeCell ref="B179:C179"/>
     <mergeCell ref="B425:B426"/>
@@ -9261,6 +9964,9 @@
     <mergeCell ref="B2313:B2314"/>
     <mergeCell ref="B2303:C2303"/>
     <mergeCell ref="B2421:C2421"/>
+    <mergeCell ref="B2539:C2539"/>
+    <mergeCell ref="C2546:C2547"/>
+    <mergeCell ref="B2598:C2598"/>
     <mergeCell ref="B1064:C1064"/>
     <mergeCell ref="B1123:C1123"/>
     <mergeCell ref="B1182:C1182"/>
@@ -9270,6 +9976,7 @@
     <mergeCell ref="B1300:C1300"/>
     <mergeCell ref="B1418:C1418"/>
     <mergeCell ref="B1487:B1488"/>
+    <mergeCell ref="C2607:C2608"/>
     <mergeCell ref="B828:C828"/>
     <mergeCell ref="B1536:C1536"/>
     <mergeCell ref="B1595:C1595"/>

</xml_diff>

<commit_message>
Fixed Direct Page Indexed Indirect X addressing in 5A22, Absolute Bit addressing in SPC-700.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6085109C-7CC7-45E5-AF3A-95F1BA18C898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4DE6DDC-508C-4BEE-BAA0-ADC697C9A0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
+    <workbookView xWindow="9450" yWindow="420" windowWidth="16575" windowHeight="14745" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5748,13 +5748,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6382,10 +6382,10 @@
     </row>
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
-      <c r="B120" s="20" t="s">
+      <c r="B120" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C120" s="21"/>
+      <c r="C120" s="22"/>
     </row>
     <row r="121" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
@@ -6507,10 +6507,10 @@
     </row>
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="13"/>
-      <c r="B179" s="20" t="s">
+      <c r="B179" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C179" s="21"/>
+      <c r="C179" s="22"/>
     </row>
     <row r="180" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="5" t="s">
@@ -6921,10 +6921,10 @@
     </row>
     <row r="356" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A356" s="13"/>
-      <c r="B356" s="20" t="s">
+      <c r="B356" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="C356" s="21"/>
+      <c r="C356" s="22"/>
     </row>
     <row r="357" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A357" s="5" t="s">
@@ -7116,7 +7116,7 @@
       <c r="A425" s="3">
         <v>4.2</v>
       </c>
-      <c r="B425" s="22" t="s">
+      <c r="B425" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C425" s="2" t="s">
@@ -7125,7 +7125,7 @@
     </row>
     <row r="426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A426" s="3"/>
-      <c r="B426" s="22"/>
+      <c r="B426" s="20"/>
       <c r="C426" s="2"/>
     </row>
     <row r="427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7273,10 +7273,10 @@
     </row>
     <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A533" s="13"/>
-      <c r="B533" s="20" t="s">
+      <c r="B533" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="C533" s="21"/>
+      <c r="C533" s="22"/>
     </row>
     <row r="534" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A534" s="5" t="s">
@@ -7528,30 +7528,30 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B601" s="7"/>
-      <c r="C601" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="C601" s="2"/>
     </row>
     <row r="602" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A602" s="3"/>
+      <c r="A602" s="3">
+        <v>4.2</v>
+      </c>
       <c r="B602" s="7"/>
-      <c r="C602" s="2" t="s">
-        <v>74</v>
-      </c>
+      <c r="C602" s="2"/>
     </row>
     <row r="603" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A603" s="3">
-        <v>4.2</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="B603" s="7"/>
-      <c r="C603" s="2"/>
+      <c r="C603" s="2" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="604" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A604" s="3">
-        <v>5.0999999999999996</v>
-      </c>
+      <c r="A604" s="3"/>
       <c r="B604" s="7"/>
-      <c r="C604" s="2"/>
+      <c r="C604" s="2" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="605" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A605" s="3">
@@ -7584,10 +7584,10 @@
     </row>
     <row r="651" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A651" s="13"/>
-      <c r="B651" s="20" t="s">
+      <c r="B651" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="C651" s="21"/>
+      <c r="C651" s="22"/>
     </row>
     <row r="652" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A652" s="5" t="s">
@@ -7709,10 +7709,10 @@
     </row>
     <row r="710" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A710" s="13"/>
-      <c r="B710" s="20" t="s">
+      <c r="B710" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C710" s="21"/>
+      <c r="C710" s="22"/>
     </row>
     <row r="711" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A711" s="5" t="s">
@@ -7973,10 +7973,10 @@
     </row>
     <row r="828" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A828" s="13"/>
-      <c r="B828" s="20" t="s">
+      <c r="B828" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C828" s="21"/>
+      <c r="C828" s="22"/>
     </row>
     <row r="829" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A829" s="5" t="s">
@@ -8654,10 +8654,10 @@
     </row>
     <row r="1064" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1064" s="13"/>
-      <c r="B1064" s="20" t="s">
+      <c r="B1064" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C1064" s="21"/>
+      <c r="C1064" s="22"/>
     </row>
     <row r="1065" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1065" s="5" t="s">
@@ -8779,10 +8779,10 @@
     </row>
     <row r="1123" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1123" s="13"/>
-      <c r="B1123" s="20" t="s">
+      <c r="B1123" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C1123" s="21"/>
+      <c r="C1123" s="22"/>
     </row>
     <row r="1124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1124" s="5" t="s">
@@ -8959,10 +8959,10 @@
     </row>
     <row r="1182" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1182" s="13"/>
-      <c r="B1182" s="20" t="s">
+      <c r="B1182" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C1182" s="21"/>
+      <c r="C1182" s="22"/>
     </row>
     <row r="1183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1183" s="5" t="s">
@@ -9082,10 +9082,10 @@
     </row>
     <row r="1241" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1241" s="13"/>
-      <c r="B1241" s="20" t="s">
+      <c r="B1241" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="C1241" s="21"/>
+      <c r="C1241" s="22"/>
     </row>
     <row r="1242" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1242" s="5" t="s">
@@ -9225,10 +9225,10 @@
     </row>
     <row r="1300" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1300" s="13"/>
-      <c r="B1300" s="20" t="s">
+      <c r="B1300" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C1300" s="21"/>
+      <c r="C1300" s="22"/>
     </row>
     <row r="1301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1301" s="5" t="s">
@@ -9368,10 +9368,10 @@
     </row>
     <row r="1359" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1359" s="13"/>
-      <c r="B1359" s="20" t="s">
+      <c r="B1359" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C1359" s="21"/>
+      <c r="C1359" s="22"/>
     </row>
     <row r="1360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1360" s="5" t="s">
@@ -9462,7 +9462,7 @@
       <c r="A1369" s="3">
         <v>4.2</v>
       </c>
-      <c r="B1369" s="22" t="s">
+      <c r="B1369" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C1369" s="2" t="s">
@@ -9471,7 +9471,7 @@
     </row>
     <row r="1370" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1370" s="3"/>
-      <c r="B1370" s="22"/>
+      <c r="B1370" s="20"/>
       <c r="C1370" s="2"/>
     </row>
     <row r="1371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9534,10 +9534,10 @@
     </row>
     <row r="1418" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1418" s="13"/>
-      <c r="B1418" s="20" t="s">
+      <c r="B1418" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="C1418" s="21"/>
+      <c r="C1418" s="22"/>
     </row>
     <row r="1419" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1419" s="5" t="s">
@@ -9775,7 +9775,7 @@
       <c r="A1487" s="3">
         <v>4.2</v>
       </c>
-      <c r="B1487" s="22" t="s">
+      <c r="B1487" s="20" t="s">
         <v>137</v>
       </c>
       <c r="C1487" s="2" t="s">
@@ -9784,7 +9784,7 @@
     </row>
     <row r="1488" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1488" s="3"/>
-      <c r="B1488" s="22"/>
+      <c r="B1488" s="20"/>
       <c r="C1488" s="2"/>
     </row>
     <row r="1489" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9825,10 +9825,10 @@
     </row>
     <row r="1536" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1536" s="13"/>
-      <c r="B1536" s="20" t="s">
+      <c r="B1536" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="C1536" s="21"/>
+      <c r="C1536" s="22"/>
     </row>
     <row r="1537" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1537" s="5" t="s">
@@ -9937,7 +9937,7 @@
       <c r="A1548" s="3">
         <v>4.2</v>
       </c>
-      <c r="B1548" s="22" t="s">
+      <c r="B1548" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C1548" s="2" t="s">
@@ -9946,7 +9946,7 @@
     </row>
     <row r="1549" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1549" s="3"/>
-      <c r="B1549" s="22"/>
+      <c r="B1549" s="20"/>
       <c r="C1549" s="2"/>
     </row>
     <row r="1550" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9962,7 +9962,7 @@
       <c r="A1551" s="3">
         <v>5.2</v>
       </c>
-      <c r="B1551" s="22" t="s">
+      <c r="B1551" s="20" t="s">
         <v>150</v>
       </c>
       <c r="C1551" s="2" t="s">
@@ -9971,7 +9971,7 @@
     </row>
     <row r="1552" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1552" s="3"/>
-      <c r="B1552" s="22"/>
+      <c r="B1552" s="20"/>
       <c r="C1552" s="2"/>
     </row>
     <row r="1553" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10012,10 +10012,10 @@
     </row>
     <row r="1595" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1595" s="13"/>
-      <c r="B1595" s="20" t="s">
+      <c r="B1595" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C1595" s="21"/>
+      <c r="C1595" s="22"/>
     </row>
     <row r="1596" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1596" s="5" t="s">
@@ -10450,10 +10450,10 @@
     </row>
     <row r="1831" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1831" s="13"/>
-      <c r="B1831" s="20" t="s">
+      <c r="B1831" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="C1831" s="21"/>
+      <c r="C1831" s="22"/>
     </row>
     <row r="1832" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1832" s="5" t="s">
@@ -10877,10 +10877,10 @@
     </row>
     <row r="2008" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2008" s="13"/>
-      <c r="B2008" s="20" t="s">
+      <c r="B2008" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C2008" s="21"/>
+      <c r="C2008" s="22"/>
     </row>
     <row r="2009" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2009" s="5" t="s">
@@ -11517,10 +11517,10 @@
     </row>
     <row r="2303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2303" s="13"/>
-      <c r="B2303" s="20" t="s">
+      <c r="B2303" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C2303" s="21"/>
+      <c r="C2303" s="22"/>
     </row>
     <row r="2304" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2304" s="5" t="s">
@@ -11611,7 +11611,7 @@
       <c r="A2313" s="3">
         <v>4.2</v>
       </c>
-      <c r="B2313" s="22" t="s">
+      <c r="B2313" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C2313" s="2" t="s">
@@ -11620,7 +11620,7 @@
     </row>
     <row r="2314" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2314" s="3"/>
-      <c r="B2314" s="22"/>
+      <c r="B2314" s="20"/>
       <c r="C2314" s="2"/>
     </row>
     <row r="2315" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11768,10 +11768,10 @@
     </row>
     <row r="2421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2421" s="13"/>
-      <c r="B2421" s="20" t="s">
+      <c r="B2421" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="C2421" s="21"/>
+      <c r="C2421" s="22"/>
     </row>
     <row r="2422" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2422" s="5" t="s">
@@ -12023,30 +12023,30 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B2489" s="7"/>
-      <c r="C2489" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="C2489" s="2"/>
     </row>
     <row r="2490" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2490" s="3"/>
+      <c r="A2490" s="3">
+        <v>4.2</v>
+      </c>
       <c r="B2490" s="7"/>
-      <c r="C2490" s="2" t="s">
-        <v>173</v>
-      </c>
+      <c r="C2490" s="2"/>
     </row>
     <row r="2491" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2491" s="3">
-        <v>4.2</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="B2491" s="7"/>
-      <c r="C2491" s="2"/>
+      <c r="C2491" s="2" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="2492" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2492" s="3">
-        <v>5.0999999999999996</v>
-      </c>
+      <c r="A2492" s="3"/>
       <c r="B2492" s="7"/>
-      <c r="C2492" s="2"/>
+      <c r="C2492" s="2" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="2493" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2493" s="3">
@@ -12079,10 +12079,10 @@
     </row>
     <row r="2539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2539" s="13"/>
-      <c r="B2539" s="20" t="s">
+      <c r="B2539" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="C2539" s="21"/>
+      <c r="C2539" s="22"/>
     </row>
     <row r="2540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2540" s="5" t="s">
@@ -12151,14 +12151,14 @@
         <v>3.1</v>
       </c>
       <c r="B2546" s="7"/>
-      <c r="C2546" s="22" t="s">
+      <c r="C2546" s="20" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="2547" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2547" s="3"/>
       <c r="B2547" s="7"/>
-      <c r="C2547" s="22"/>
+      <c r="C2547" s="20"/>
     </row>
     <row r="2548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2548" s="3">
@@ -12209,10 +12209,10 @@
     </row>
     <row r="2598" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2598" s="13"/>
-      <c r="B2598" s="20" t="s">
+      <c r="B2598" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C2598" s="21"/>
+      <c r="C2598" s="22"/>
     </row>
     <row r="2599" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2599" s="5" t="s">
@@ -12301,14 +12301,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B2607" s="7"/>
-      <c r="C2607" s="22" t="s">
+      <c r="C2607" s="20" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="2608" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2608" s="3"/>
       <c r="B2608" s="7"/>
-      <c r="C2608" s="22"/>
+      <c r="C2608" s="20"/>
     </row>
     <row r="2609" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2609" s="3">
@@ -13097,10 +13097,10 @@
     </row>
     <row r="2952" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2952" s="13"/>
-      <c r="B2952" s="20" t="s">
+      <c r="B2952" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C2952" s="21"/>
+      <c r="C2952" s="22"/>
     </row>
     <row r="2953" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2953" s="5" t="s">
@@ -13222,10 +13222,10 @@
     </row>
     <row r="3011" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3011" s="13"/>
-      <c r="B3011" s="20" t="s">
+      <c r="B3011" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C3011" s="21"/>
+      <c r="C3011" s="22"/>
     </row>
     <row r="3012" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3012" s="5" t="s">
@@ -13402,10 +13402,10 @@
     </row>
     <row r="3070" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3070" s="13"/>
-      <c r="B3070" s="20" t="s">
+      <c r="B3070" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C3070" s="21"/>
+      <c r="C3070" s="22"/>
     </row>
     <row r="3071" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3071" s="5" t="s">
@@ -13525,10 +13525,10 @@
     </row>
     <row r="3129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3129" s="13"/>
-      <c r="B3129" s="20" t="s">
+      <c r="B3129" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="C3129" s="21"/>
+      <c r="C3129" s="22"/>
     </row>
     <row r="3130" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3130" s="5" t="s">
@@ -13668,10 +13668,10 @@
     </row>
     <row r="3188" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3188" s="13"/>
-      <c r="B3188" s="20" t="s">
+      <c r="B3188" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C3188" s="21"/>
+      <c r="C3188" s="22"/>
     </row>
     <row r="3189" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3189" s="5" t="s">
@@ -13811,10 +13811,10 @@
     </row>
     <row r="3247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3247" s="13"/>
-      <c r="B3247" s="20" t="s">
+      <c r="B3247" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C3247" s="21"/>
+      <c r="C3247" s="22"/>
     </row>
     <row r="3248" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3248" s="5" t="s">
@@ -13905,7 +13905,7 @@
       <c r="A3257" s="3">
         <v>4.2</v>
       </c>
-      <c r="B3257" s="22" t="s">
+      <c r="B3257" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C3257" s="2" t="s">
@@ -13914,7 +13914,7 @@
     </row>
     <row r="3258" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3258" s="3"/>
-      <c r="B3258" s="22"/>
+      <c r="B3258" s="20"/>
       <c r="C3258" s="2"/>
     </row>
     <row r="3259" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -13977,10 +13977,10 @@
     </row>
     <row r="3306" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3306" s="13"/>
-      <c r="B3306" s="20" t="s">
+      <c r="B3306" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="C3306" s="21"/>
+      <c r="C3306" s="22"/>
     </row>
     <row r="3307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3307" s="5" t="s">
@@ -14122,10 +14122,10 @@
     </row>
     <row r="3365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3365" s="13"/>
-      <c r="B3365" s="20" t="s">
+      <c r="B3365" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="C3365" s="21"/>
+      <c r="C3365" s="22"/>
     </row>
     <row r="3366" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3366" s="5" t="s">
@@ -14218,7 +14218,7 @@
       <c r="A3375" s="3">
         <v>4.2</v>
       </c>
-      <c r="B3375" s="22" t="s">
+      <c r="B3375" s="20" t="s">
         <v>137</v>
       </c>
       <c r="C3375" s="2" t="s">
@@ -14227,7 +14227,7 @@
     </row>
     <row r="3376" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3376" s="3"/>
-      <c r="B3376" s="22"/>
+      <c r="B3376" s="20"/>
       <c r="C3376" s="2"/>
     </row>
     <row r="3377" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -14268,10 +14268,10 @@
     </row>
     <row r="3424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3424" s="13"/>
-      <c r="B3424" s="20" t="s">
+      <c r="B3424" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="C3424" s="21"/>
+      <c r="C3424" s="22"/>
     </row>
     <row r="3425" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3425" s="5" t="s">
@@ -14380,7 +14380,7 @@
       <c r="A3436" s="3">
         <v>4.2</v>
       </c>
-      <c r="B3436" s="22" t="s">
+      <c r="B3436" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C3436" s="2" t="s">
@@ -14389,7 +14389,7 @@
     </row>
     <row r="3437" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3437" s="3"/>
-      <c r="B3437" s="22"/>
+      <c r="B3437" s="20"/>
       <c r="C3437" s="2"/>
     </row>
     <row r="3438" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -14405,7 +14405,7 @@
       <c r="A3439" s="3">
         <v>5.2</v>
       </c>
-      <c r="B3439" s="22" t="s">
+      <c r="B3439" s="20" t="s">
         <v>150</v>
       </c>
       <c r="C3439" s="2" t="s">
@@ -14414,7 +14414,7 @@
     </row>
     <row r="3440" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3440" s="3"/>
-      <c r="B3440" s="22"/>
+      <c r="B3440" s="20"/>
       <c r="C3440" s="2"/>
     </row>
     <row r="3441" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -14455,10 +14455,10 @@
     </row>
     <row r="3483" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3483" s="13"/>
-      <c r="B3483" s="20" t="s">
+      <c r="B3483" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C3483" s="21"/>
+      <c r="C3483" s="22"/>
     </row>
     <row r="3484" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3484" s="5" t="s">
@@ -14543,14 +14543,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B3492" s="7"/>
-      <c r="C3492" s="22" t="s">
+      <c r="C3492" s="20" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="3493" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3493" s="3"/>
       <c r="B3493" s="7"/>
-      <c r="C3493" s="22"/>
+      <c r="C3493" s="20"/>
     </row>
     <row r="3494" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3494" s="3">
@@ -15339,10 +15339,10 @@
     </row>
     <row r="3896" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3896" s="13"/>
-      <c r="B3896" s="20" t="s">
+      <c r="B3896" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C3896" s="21"/>
+      <c r="C3896" s="22"/>
     </row>
     <row r="3897" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3897" s="5" t="s">
@@ -15464,10 +15464,10 @@
     </row>
     <row r="3955" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3955" s="13"/>
-      <c r="B3955" s="20" t="s">
+      <c r="B3955" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C3955" s="21"/>
+      <c r="C3955" s="22"/>
     </row>
     <row r="3956" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3956" s="5" t="s">
@@ -15979,10 +15979,10 @@
     </row>
     <row r="4191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4191" s="13"/>
-      <c r="B4191" s="20" t="s">
+      <c r="B4191" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C4191" s="21"/>
+      <c r="C4191" s="22"/>
     </row>
     <row r="4192" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4192" s="5" t="s">
@@ -16073,7 +16073,7 @@
       <c r="A4201" s="3">
         <v>4.2</v>
       </c>
-      <c r="B4201" s="22" t="s">
+      <c r="B4201" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C4201" s="2" t="s">
@@ -16082,7 +16082,7 @@
     </row>
     <row r="4202" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4202" s="3"/>
-      <c r="B4202" s="22"/>
+      <c r="B4202" s="20"/>
       <c r="C4202" s="2"/>
     </row>
     <row r="4203" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -16230,10 +16230,10 @@
     </row>
     <row r="4309" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4309" s="13"/>
-      <c r="B4309" s="20" t="s">
+      <c r="B4309" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="C4309" s="21"/>
+      <c r="C4309" s="22"/>
     </row>
     <row r="4310" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4310" s="5" t="s">
@@ -16393,10 +16393,10 @@
     </row>
     <row r="4368" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4368" s="13"/>
-      <c r="B4368" s="20" t="s">
+      <c r="B4368" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="C4368" s="21"/>
+      <c r="C4368" s="22"/>
     </row>
     <row r="4369" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4369" s="5" t="s">
@@ -16527,10 +16527,10 @@
     </row>
     <row r="4427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4427" s="13"/>
-      <c r="B4427" s="20" t="s">
+      <c r="B4427" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="C4427" s="21"/>
+      <c r="C4427" s="22"/>
     </row>
     <row r="4428" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4428" s="5" t="s">
@@ -16652,10 +16652,10 @@
     </row>
     <row r="4486" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4486" s="13"/>
-      <c r="B4486" s="20" t="s">
+      <c r="B4486" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C4486" s="21"/>
+      <c r="C4486" s="22"/>
     </row>
     <row r="4487" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4487" s="5" t="s">
@@ -16916,10 +16916,10 @@
     </row>
     <row r="4604" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4604" s="13"/>
-      <c r="B4604" s="20" t="s">
+      <c r="B4604" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C4604" s="21"/>
+      <c r="C4604" s="22"/>
     </row>
     <row r="4605" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4605" s="5" t="s">
@@ -17561,10 +17561,10 @@
     </row>
     <row r="4840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4840" s="13"/>
-      <c r="B4840" s="20" t="s">
+      <c r="B4840" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C4840" s="21"/>
+      <c r="C4840" s="22"/>
     </row>
     <row r="4841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4841" s="5" t="s">
@@ -17866,10 +17866,10 @@
     </row>
     <row r="4958" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4958" s="13"/>
-      <c r="B4958" s="20" t="s">
+      <c r="B4958" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C4958" s="21"/>
+      <c r="C4958" s="22"/>
     </row>
     <row r="4959" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4959" s="5" t="s">
@@ -17989,10 +17989,10 @@
     </row>
     <row r="5017" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5017" s="13"/>
-      <c r="B5017" s="20" t="s">
+      <c r="B5017" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="C5017" s="21"/>
+      <c r="C5017" s="22"/>
     </row>
     <row r="5018" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5018" s="5" t="s">
@@ -18132,10 +18132,10 @@
     </row>
     <row r="5076" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5076" s="13"/>
-      <c r="B5076" s="20" t="s">
+      <c r="B5076" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C5076" s="21"/>
+      <c r="C5076" s="22"/>
     </row>
     <row r="5077" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5077" s="5" t="s">
@@ -18275,10 +18275,10 @@
     </row>
     <row r="5135" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5135" s="13"/>
-      <c r="B5135" s="20" t="s">
+      <c r="B5135" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C5135" s="21"/>
+      <c r="C5135" s="22"/>
     </row>
     <row r="5136" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5136" s="5" t="s">
@@ -18369,7 +18369,7 @@
       <c r="A5145" s="3">
         <v>4.2</v>
       </c>
-      <c r="B5145" s="22" t="s">
+      <c r="B5145" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C5145" s="2" t="s">
@@ -18378,7 +18378,7 @@
     </row>
     <row r="5146" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5146" s="3"/>
-      <c r="B5146" s="22"/>
+      <c r="B5146" s="20"/>
       <c r="C5146" s="2"/>
     </row>
     <row r="5147" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18441,10 +18441,10 @@
     </row>
     <row r="5194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5194" s="13"/>
-      <c r="B5194" s="20" t="s">
+      <c r="B5194" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="C5194" s="21"/>
+      <c r="C5194" s="22"/>
     </row>
     <row r="5195" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5195" s="5" t="s">
@@ -18586,10 +18586,10 @@
     </row>
     <row r="5253" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5253" s="13"/>
-      <c r="B5253" s="20" t="s">
+      <c r="B5253" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="C5253" s="21"/>
+      <c r="C5253" s="22"/>
     </row>
     <row r="5254" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5254" s="5" t="s">
@@ -18682,7 +18682,7 @@
       <c r="A5263" s="3">
         <v>4.2</v>
       </c>
-      <c r="B5263" s="22" t="s">
+      <c r="B5263" s="20" t="s">
         <v>137</v>
       </c>
       <c r="C5263" s="2" t="s">
@@ -18691,7 +18691,7 @@
     </row>
     <row r="5264" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5264" s="3"/>
-      <c r="B5264" s="22"/>
+      <c r="B5264" s="20"/>
       <c r="C5264" s="2"/>
     </row>
     <row r="5265" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18810,7 +18810,7 @@
       <c r="A5320" s="3">
         <v>3.2</v>
       </c>
-      <c r="B5320" s="22" t="s">
+      <c r="B5320" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C5320" s="2" t="s">
@@ -18819,7 +18819,7 @@
     </row>
     <row r="5321" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5321" s="3"/>
-      <c r="B5321" s="22"/>
+      <c r="B5321" s="20"/>
       <c r="C5321" s="2"/>
     </row>
     <row r="5322" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18862,10 +18862,10 @@
     </row>
     <row r="5371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5371" s="13"/>
-      <c r="B5371" s="20" t="s">
+      <c r="B5371" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C5371" s="21"/>
+      <c r="C5371" s="22"/>
     </row>
     <row r="5372" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5372" s="5" t="s">
@@ -19677,10 +19677,10 @@
     </row>
     <row r="5784" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5784" s="13"/>
-      <c r="B5784" s="20" t="s">
+      <c r="B5784" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C5784" s="21"/>
+      <c r="C5784" s="22"/>
     </row>
     <row r="5785" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5785" s="5" t="s">
@@ -19802,10 +19802,10 @@
     </row>
     <row r="5843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5843" s="13"/>
-      <c r="B5843" s="20" t="s">
+      <c r="B5843" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C5843" s="21"/>
+      <c r="C5843" s="22"/>
     </row>
     <row r="5844" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5844" s="5" t="s">
@@ -20317,10 +20317,10 @@
     </row>
     <row r="6079" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6079" s="13"/>
-      <c r="B6079" s="20" t="s">
+      <c r="B6079" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="C6079" s="21"/>
+      <c r="C6079" s="22"/>
     </row>
     <row r="6080" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6080" s="5" t="s">
@@ -20411,7 +20411,7 @@
       <c r="A6089" s="3">
         <v>4.2</v>
       </c>
-      <c r="B6089" s="22" t="s">
+      <c r="B6089" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C6089" s="2" t="s">
@@ -20420,7 +20420,7 @@
     </row>
     <row r="6090" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6090" s="3"/>
-      <c r="B6090" s="22"/>
+      <c r="B6090" s="20"/>
       <c r="C6090" s="2"/>
     </row>
     <row r="6091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -20568,10 +20568,10 @@
     </row>
     <row r="6197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6197" s="13"/>
-      <c r="B6197" s="20" t="s">
+      <c r="B6197" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="C6197" s="21"/>
+      <c r="C6197" s="22"/>
     </row>
     <row r="6198" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6198" s="5" t="s">
@@ -20865,10 +20865,10 @@
     </row>
     <row r="6315" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6315" s="13"/>
-      <c r="B6315" s="20" t="s">
+      <c r="B6315" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="C6315" s="21"/>
+      <c r="C6315" s="22"/>
     </row>
     <row r="6316" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6316" s="5" t="s">
@@ -20937,14 +20937,14 @@
         <v>3.1</v>
       </c>
       <c r="B6322" s="7"/>
-      <c r="C6322" s="22" t="s">
+      <c r="C6322" s="20" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="6323" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6323" s="3"/>
       <c r="B6323" s="7"/>
-      <c r="C6323" s="22"/>
+      <c r="C6323" s="20"/>
     </row>
     <row r="6324" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6324" s="3">
@@ -20995,10 +20995,10 @@
     </row>
     <row r="6374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6374" s="13"/>
-      <c r="B6374" s="20" t="s">
+      <c r="B6374" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="C6374" s="21"/>
+      <c r="C6374" s="22"/>
     </row>
     <row r="6375" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6375" s="5" t="s">
@@ -21900,10 +21900,10 @@
     </row>
     <row r="6728" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6728" s="13"/>
-      <c r="B6728" s="20" t="s">
+      <c r="B6728" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C6728" s="21"/>
+      <c r="C6728" s="22"/>
     </row>
     <row r="6729" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6729" s="5" t="s">
@@ -22025,10 +22025,10 @@
     </row>
     <row r="6787" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6787" s="13"/>
-      <c r="B6787" s="20" t="s">
+      <c r="B6787" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="C6787" s="21"/>
+      <c r="C6787" s="22"/>
     </row>
     <row r="6788" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6788" s="5" t="s">
@@ -22205,10 +22205,10 @@
     </row>
     <row r="6846" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6846" s="13"/>
-      <c r="B6846" s="20" t="s">
+      <c r="B6846" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C6846" s="21"/>
+      <c r="C6846" s="22"/>
     </row>
     <row r="6847" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6847" s="5" t="s">
@@ -22328,10 +22328,10 @@
     </row>
     <row r="6905" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6905" s="13"/>
-      <c r="B6905" s="20" t="s">
+      <c r="B6905" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="C6905" s="21"/>
+      <c r="C6905" s="22"/>
     </row>
     <row r="6906" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6906" s="5" t="s">
@@ -22471,10 +22471,10 @@
     </row>
     <row r="6964" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6964" s="13"/>
-      <c r="B6964" s="20" t="s">
+      <c r="B6964" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C6964" s="21"/>
+      <c r="C6964" s="22"/>
     </row>
     <row r="6965" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6965" s="5" t="s">
@@ -22614,10 +22614,10 @@
     </row>
     <row r="7023" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7023" s="13"/>
-      <c r="B7023" s="20" t="s">
+      <c r="B7023" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C7023" s="21"/>
+      <c r="C7023" s="22"/>
     </row>
     <row r="7024" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7024" s="5" t="s">
@@ -22708,7 +22708,7 @@
       <c r="A7033" s="3">
         <v>4.2</v>
       </c>
-      <c r="B7033" s="22" t="s">
+      <c r="B7033" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C7033" s="2" t="s">
@@ -22717,7 +22717,7 @@
     </row>
     <row r="7034" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7034" s="3"/>
-      <c r="B7034" s="22"/>
+      <c r="B7034" s="20"/>
       <c r="C7034" s="2"/>
     </row>
     <row r="7035" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -22780,10 +22780,10 @@
     </row>
     <row r="7082" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7082" s="13"/>
-      <c r="B7082" s="20" t="s">
+      <c r="B7082" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="C7082" s="21"/>
+      <c r="C7082" s="22"/>
     </row>
     <row r="7083" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7083" s="5" t="s">
@@ -22925,10 +22925,10 @@
     </row>
     <row r="7141" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7141" s="13"/>
-      <c r="B7141" s="20" t="s">
+      <c r="B7141" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="C7141" s="21"/>
+      <c r="C7141" s="22"/>
     </row>
     <row r="7142" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7142" s="5" t="s">
@@ -23021,7 +23021,7 @@
       <c r="A7151" s="3">
         <v>4.2</v>
       </c>
-      <c r="B7151" s="22" t="s">
+      <c r="B7151" s="20" t="s">
         <v>137</v>
       </c>
       <c r="C7151" s="2" t="s">
@@ -23030,7 +23030,7 @@
     </row>
     <row r="7152" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7152" s="3"/>
-      <c r="B7152" s="22"/>
+      <c r="B7152" s="20"/>
       <c r="C7152" s="2"/>
     </row>
     <row r="7153" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -23060,56 +23060,11 @@
     </row>
   </sheetData>
   <mergeCells count="83">
-    <mergeCell ref="B7151:B7152"/>
-    <mergeCell ref="B7141:C7141"/>
-    <mergeCell ref="B6787:C6787"/>
-    <mergeCell ref="B6846:C6846"/>
-    <mergeCell ref="B6905:C6905"/>
-    <mergeCell ref="B6964:C6964"/>
-    <mergeCell ref="B7023:C7023"/>
-    <mergeCell ref="B7033:B7034"/>
-    <mergeCell ref="B7082:C7082"/>
-    <mergeCell ref="B5371:C5371"/>
-    <mergeCell ref="B5784:C5784"/>
-    <mergeCell ref="B5843:C5843"/>
-    <mergeCell ref="B6079:C6079"/>
-    <mergeCell ref="B6089:B6090"/>
-    <mergeCell ref="B5135:C5135"/>
-    <mergeCell ref="B5145:B5146"/>
-    <mergeCell ref="B5194:C5194"/>
-    <mergeCell ref="B5253:C5253"/>
-    <mergeCell ref="B5263:B5264"/>
-    <mergeCell ref="B5320:B5321"/>
-    <mergeCell ref="B4486:C4486"/>
-    <mergeCell ref="B4604:C4604"/>
-    <mergeCell ref="B4840:C4840"/>
-    <mergeCell ref="B4958:C4958"/>
-    <mergeCell ref="B5017:C5017"/>
-    <mergeCell ref="B5076:C5076"/>
-    <mergeCell ref="B3955:C3955"/>
-    <mergeCell ref="B4191:C4191"/>
-    <mergeCell ref="B4201:B4202"/>
-    <mergeCell ref="B4309:C4309"/>
-    <mergeCell ref="B4368:C4368"/>
-    <mergeCell ref="B4427:C4427"/>
-    <mergeCell ref="B2952:C2952"/>
-    <mergeCell ref="B3011:C3011"/>
-    <mergeCell ref="B3070:C3070"/>
-    <mergeCell ref="B3129:C3129"/>
-    <mergeCell ref="B3188:C3188"/>
-    <mergeCell ref="B3247:C3247"/>
-    <mergeCell ref="B3257:B3258"/>
-    <mergeCell ref="B3306:C3306"/>
-    <mergeCell ref="B120:C120"/>
-    <mergeCell ref="B179:C179"/>
-    <mergeCell ref="B425:B426"/>
-    <mergeCell ref="B533:C533"/>
-    <mergeCell ref="B651:C651"/>
-    <mergeCell ref="B710:C710"/>
-    <mergeCell ref="B356:C356"/>
-    <mergeCell ref="B6197:C6197"/>
-    <mergeCell ref="B6315:C6315"/>
-    <mergeCell ref="C6322:C6323"/>
+    <mergeCell ref="B1595:C1595"/>
+    <mergeCell ref="B1548:B1549"/>
+    <mergeCell ref="B1551:B1552"/>
+    <mergeCell ref="B3365:C3365"/>
+    <mergeCell ref="B3375:B3376"/>
     <mergeCell ref="B6374:C6374"/>
     <mergeCell ref="B6728:C6728"/>
     <mergeCell ref="B1831:C1831"/>
@@ -23120,6 +23075,17 @@
     <mergeCell ref="B2539:C2539"/>
     <mergeCell ref="C2546:C2547"/>
     <mergeCell ref="B2598:C2598"/>
+    <mergeCell ref="C2607:C2608"/>
+    <mergeCell ref="B3424:C3424"/>
+    <mergeCell ref="B3436:B3437"/>
+    <mergeCell ref="B3439:B3440"/>
+    <mergeCell ref="B3483:C3483"/>
+    <mergeCell ref="C3492:C3493"/>
+    <mergeCell ref="B710:C710"/>
+    <mergeCell ref="B356:C356"/>
+    <mergeCell ref="B6197:C6197"/>
+    <mergeCell ref="B6315:C6315"/>
+    <mergeCell ref="C6322:C6323"/>
     <mergeCell ref="B1064:C1064"/>
     <mergeCell ref="B1123:C1123"/>
     <mergeCell ref="B1182:C1182"/>
@@ -23129,20 +23095,54 @@
     <mergeCell ref="B1300:C1300"/>
     <mergeCell ref="B1418:C1418"/>
     <mergeCell ref="B1487:B1488"/>
-    <mergeCell ref="C2607:C2608"/>
     <mergeCell ref="B828:C828"/>
     <mergeCell ref="B1536:C1536"/>
-    <mergeCell ref="B1595:C1595"/>
-    <mergeCell ref="B1548:B1549"/>
-    <mergeCell ref="B1551:B1552"/>
-    <mergeCell ref="B3365:C3365"/>
-    <mergeCell ref="B3375:B3376"/>
-    <mergeCell ref="B3424:C3424"/>
-    <mergeCell ref="B3436:B3437"/>
-    <mergeCell ref="B3439:B3440"/>
-    <mergeCell ref="B3483:C3483"/>
-    <mergeCell ref="C3492:C3493"/>
+    <mergeCell ref="B120:C120"/>
+    <mergeCell ref="B179:C179"/>
+    <mergeCell ref="B425:B426"/>
+    <mergeCell ref="B533:C533"/>
+    <mergeCell ref="B651:C651"/>
+    <mergeCell ref="B4427:C4427"/>
+    <mergeCell ref="B2952:C2952"/>
+    <mergeCell ref="B3011:C3011"/>
+    <mergeCell ref="B3070:C3070"/>
+    <mergeCell ref="B3129:C3129"/>
+    <mergeCell ref="B3188:C3188"/>
+    <mergeCell ref="B3247:C3247"/>
+    <mergeCell ref="B3257:B3258"/>
+    <mergeCell ref="B3306:C3306"/>
     <mergeCell ref="B3896:C3896"/>
+    <mergeCell ref="B3955:C3955"/>
+    <mergeCell ref="B4191:C4191"/>
+    <mergeCell ref="B4201:B4202"/>
+    <mergeCell ref="B4309:C4309"/>
+    <mergeCell ref="B4368:C4368"/>
+    <mergeCell ref="B5320:B5321"/>
+    <mergeCell ref="B4486:C4486"/>
+    <mergeCell ref="B4604:C4604"/>
+    <mergeCell ref="B4840:C4840"/>
+    <mergeCell ref="B4958:C4958"/>
+    <mergeCell ref="B5017:C5017"/>
+    <mergeCell ref="B5076:C5076"/>
+    <mergeCell ref="B5135:C5135"/>
+    <mergeCell ref="B5145:B5146"/>
+    <mergeCell ref="B5194:C5194"/>
+    <mergeCell ref="B5253:C5253"/>
+    <mergeCell ref="B5263:B5264"/>
+    <mergeCell ref="B5371:C5371"/>
+    <mergeCell ref="B5784:C5784"/>
+    <mergeCell ref="B5843:C5843"/>
+    <mergeCell ref="B6079:C6079"/>
+    <mergeCell ref="B6089:B6090"/>
+    <mergeCell ref="B7151:B7152"/>
+    <mergeCell ref="B7141:C7141"/>
+    <mergeCell ref="B6787:C6787"/>
+    <mergeCell ref="B6846:C6846"/>
+    <mergeCell ref="B6905:C6905"/>
+    <mergeCell ref="B6964:C6964"/>
+    <mergeCell ref="B7023:C7023"/>
+    <mergeCell ref="B7033:B7034"/>
+    <mergeCell ref="B7082:C7082"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup scale="79" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added SPC-700 instruction 7A.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4DE6DDC-508C-4BEE-BAA0-ADC697C9A0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487C70B7-6801-4E42-919B-E5022E7D4F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9450" yWindow="420" windowWidth="16575" windowHeight="14745" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$7165</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$7259</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2757" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2788" uniqueCount="322">
   <si>
     <t>Implied</t>
   </si>
@@ -5524,6 +5524,306 @@
   </si>
   <si>
     <t>CMP (79)</t>
+  </si>
+  <si>
+    <t>ADDW (7A)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (YA == $0000).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Tmp = u32(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) + u32(Operand16.L).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Tmp &gt; $FF).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = u8(Tmp).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Tmp = u32(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) + u32(Operand16.H) + u32(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>H</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ^ Operand16.H ^ u8(Tmp)) &amp; $10).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (~(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ^ Operand16.H) &amp; (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ^ u8(Tmp)) &amp; $80).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (u8(Tmp) &amp; $80).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = u8(Tmp).</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -5748,13 +6048,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6091,7 +6391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C7155"/>
+  <dimension ref="A1:C7223"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -6382,10 +6682,10 @@
     </row>
     <row r="120" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
-      <c r="B120" s="21" t="s">
+      <c r="B120" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C120" s="22"/>
+      <c r="C120" s="21"/>
     </row>
     <row r="121" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
@@ -6507,10 +6807,10 @@
     </row>
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="13"/>
-      <c r="B179" s="21" t="s">
+      <c r="B179" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C179" s="22"/>
+      <c r="C179" s="21"/>
     </row>
     <row r="180" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="5" t="s">
@@ -6921,10 +7221,10 @@
     </row>
     <row r="356" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A356" s="13"/>
-      <c r="B356" s="21" t="s">
+      <c r="B356" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="C356" s="22"/>
+      <c r="C356" s="21"/>
     </row>
     <row r="357" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A357" s="5" t="s">
@@ -7116,7 +7416,7 @@
       <c r="A425" s="3">
         <v>4.2</v>
       </c>
-      <c r="B425" s="20" t="s">
+      <c r="B425" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C425" s="2" t="s">
@@ -7125,7 +7425,7 @@
     </row>
     <row r="426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A426" s="3"/>
-      <c r="B426" s="20"/>
+      <c r="B426" s="22"/>
       <c r="C426" s="2"/>
     </row>
     <row r="427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7273,10 +7573,10 @@
     </row>
     <row r="533" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A533" s="13"/>
-      <c r="B533" s="21" t="s">
+      <c r="B533" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="C533" s="22"/>
+      <c r="C533" s="21"/>
     </row>
     <row r="534" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A534" s="5" t="s">
@@ -7584,10 +7884,10 @@
     </row>
     <row r="651" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A651" s="13"/>
-      <c r="B651" s="21" t="s">
+      <c r="B651" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="C651" s="22"/>
+      <c r="C651" s="21"/>
     </row>
     <row r="652" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A652" s="5" t="s">
@@ -7709,10 +8009,10 @@
     </row>
     <row r="710" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A710" s="13"/>
-      <c r="B710" s="21" t="s">
+      <c r="B710" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="C710" s="22"/>
+      <c r="C710" s="21"/>
     </row>
     <row r="711" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A711" s="5" t="s">
@@ -7973,10 +8273,10 @@
     </row>
     <row r="828" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A828" s="13"/>
-      <c r="B828" s="21" t="s">
+      <c r="B828" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="C828" s="22"/>
+      <c r="C828" s="21"/>
     </row>
     <row r="829" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A829" s="5" t="s">
@@ -8654,10 +8954,10 @@
     </row>
     <row r="1064" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1064" s="13"/>
-      <c r="B1064" s="21" t="s">
+      <c r="B1064" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C1064" s="22"/>
+      <c r="C1064" s="21"/>
     </row>
     <row r="1065" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1065" s="5" t="s">
@@ -8779,10 +9079,10 @@
     </row>
     <row r="1123" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1123" s="13"/>
-      <c r="B1123" s="21" t="s">
+      <c r="B1123" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C1123" s="22"/>
+      <c r="C1123" s="21"/>
     </row>
     <row r="1124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1124" s="5" t="s">
@@ -8959,10 +9259,10 @@
     </row>
     <row r="1182" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1182" s="13"/>
-      <c r="B1182" s="21" t="s">
+      <c r="B1182" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="C1182" s="22"/>
+      <c r="C1182" s="21"/>
     </row>
     <row r="1183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1183" s="5" t="s">
@@ -9082,10 +9382,10 @@
     </row>
     <row r="1241" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1241" s="13"/>
-      <c r="B1241" s="21" t="s">
+      <c r="B1241" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="C1241" s="22"/>
+      <c r="C1241" s="21"/>
     </row>
     <row r="1242" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1242" s="5" t="s">
@@ -9225,10 +9525,10 @@
     </row>
     <row r="1300" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1300" s="13"/>
-      <c r="B1300" s="21" t="s">
+      <c r="B1300" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="C1300" s="22"/>
+      <c r="C1300" s="21"/>
     </row>
     <row r="1301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1301" s="5" t="s">
@@ -9368,10 +9668,10 @@
     </row>
     <row r="1359" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1359" s="13"/>
-      <c r="B1359" s="21" t="s">
+      <c r="B1359" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C1359" s="22"/>
+      <c r="C1359" s="21"/>
     </row>
     <row r="1360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1360" s="5" t="s">
@@ -9462,7 +9762,7 @@
       <c r="A1369" s="3">
         <v>4.2</v>
       </c>
-      <c r="B1369" s="20" t="s">
+      <c r="B1369" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C1369" s="2" t="s">
@@ -9471,7 +9771,7 @@
     </row>
     <row r="1370" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1370" s="3"/>
-      <c r="B1370" s="20"/>
+      <c r="B1370" s="22"/>
       <c r="C1370" s="2"/>
     </row>
     <row r="1371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9534,10 +9834,10 @@
     </row>
     <row r="1418" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1418" s="13"/>
-      <c r="B1418" s="21" t="s">
+      <c r="B1418" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="C1418" s="22"/>
+      <c r="C1418" s="21"/>
     </row>
     <row r="1419" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1419" s="5" t="s">
@@ -9775,7 +10075,7 @@
       <c r="A1487" s="3">
         <v>4.2</v>
       </c>
-      <c r="B1487" s="20" t="s">
+      <c r="B1487" s="22" t="s">
         <v>137</v>
       </c>
       <c r="C1487" s="2" t="s">
@@ -9784,7 +10084,7 @@
     </row>
     <row r="1488" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1488" s="3"/>
-      <c r="B1488" s="20"/>
+      <c r="B1488" s="22"/>
       <c r="C1488" s="2"/>
     </row>
     <row r="1489" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9825,10 +10125,10 @@
     </row>
     <row r="1536" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1536" s="13"/>
-      <c r="B1536" s="21" t="s">
+      <c r="B1536" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="C1536" s="22"/>
+      <c r="C1536" s="21"/>
     </row>
     <row r="1537" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1537" s="5" t="s">
@@ -9937,7 +10237,7 @@
       <c r="A1548" s="3">
         <v>4.2</v>
       </c>
-      <c r="B1548" s="20" t="s">
+      <c r="B1548" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C1548" s="2" t="s">
@@ -9946,7 +10246,7 @@
     </row>
     <row r="1549" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1549" s="3"/>
-      <c r="B1549" s="20"/>
+      <c r="B1549" s="22"/>
       <c r="C1549" s="2"/>
     </row>
     <row r="1550" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -9962,7 +10262,7 @@
       <c r="A1551" s="3">
         <v>5.2</v>
       </c>
-      <c r="B1551" s="20" t="s">
+      <c r="B1551" s="22" t="s">
         <v>150</v>
       </c>
       <c r="C1551" s="2" t="s">
@@ -9971,7 +10271,7 @@
     </row>
     <row r="1552" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1552" s="3"/>
-      <c r="B1552" s="20"/>
+      <c r="B1552" s="22"/>
       <c r="C1552" s="2"/>
     </row>
     <row r="1553" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -10012,10 +10312,10 @@
     </row>
     <row r="1595" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1595" s="13"/>
-      <c r="B1595" s="21" t="s">
+      <c r="B1595" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="C1595" s="22"/>
+      <c r="C1595" s="21"/>
     </row>
     <row r="1596" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1596" s="5" t="s">
@@ -10450,10 +10750,10 @@
     </row>
     <row r="1831" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1831" s="13"/>
-      <c r="B1831" s="21" t="s">
+      <c r="B1831" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="C1831" s="22"/>
+      <c r="C1831" s="21"/>
     </row>
     <row r="1832" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1832" s="5" t="s">
@@ -10877,10 +11177,10 @@
     </row>
     <row r="2008" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2008" s="13"/>
-      <c r="B2008" s="21" t="s">
+      <c r="B2008" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C2008" s="22"/>
+      <c r="C2008" s="21"/>
     </row>
     <row r="2009" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2009" s="5" t="s">
@@ -11517,10 +11817,10 @@
     </row>
     <row r="2303" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2303" s="13"/>
-      <c r="B2303" s="21" t="s">
+      <c r="B2303" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="C2303" s="22"/>
+      <c r="C2303" s="21"/>
     </row>
     <row r="2304" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2304" s="5" t="s">
@@ -11611,7 +11911,7 @@
       <c r="A2313" s="3">
         <v>4.2</v>
       </c>
-      <c r="B2313" s="20" t="s">
+      <c r="B2313" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C2313" s="2" t="s">
@@ -11620,7 +11920,7 @@
     </row>
     <row r="2314" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2314" s="3"/>
-      <c r="B2314" s="20"/>
+      <c r="B2314" s="22"/>
       <c r="C2314" s="2"/>
     </row>
     <row r="2315" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -11768,10 +12068,10 @@
     </row>
     <row r="2421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2421" s="13"/>
-      <c r="B2421" s="21" t="s">
+      <c r="B2421" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="C2421" s="22"/>
+      <c r="C2421" s="21"/>
     </row>
     <row r="2422" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2422" s="5" t="s">
@@ -12079,10 +12379,10 @@
     </row>
     <row r="2539" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2539" s="13"/>
-      <c r="B2539" s="21" t="s">
+      <c r="B2539" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="C2539" s="22"/>
+      <c r="C2539" s="21"/>
     </row>
     <row r="2540" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2540" s="5" t="s">
@@ -12151,14 +12451,14 @@
         <v>3.1</v>
       </c>
       <c r="B2546" s="7"/>
-      <c r="C2546" s="20" t="s">
+      <c r="C2546" s="22" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="2547" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2547" s="3"/>
       <c r="B2547" s="7"/>
-      <c r="C2547" s="20"/>
+      <c r="C2547" s="22"/>
     </row>
     <row r="2548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2548" s="3">
@@ -12209,10 +12509,10 @@
     </row>
     <row r="2598" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2598" s="13"/>
-      <c r="B2598" s="21" t="s">
+      <c r="B2598" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="C2598" s="22"/>
+      <c r="C2598" s="21"/>
     </row>
     <row r="2599" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2599" s="5" t="s">
@@ -12301,14 +12601,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B2607" s="7"/>
-      <c r="C2607" s="20" t="s">
+      <c r="C2607" s="22" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="2608" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2608" s="3"/>
       <c r="B2608" s="7"/>
-      <c r="C2608" s="20"/>
+      <c r="C2608" s="22"/>
     </row>
     <row r="2609" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2609" s="3">
@@ -13097,10 +13397,10 @@
     </row>
     <row r="2952" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2952" s="13"/>
-      <c r="B2952" s="21" t="s">
+      <c r="B2952" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C2952" s="22"/>
+      <c r="C2952" s="21"/>
     </row>
     <row r="2953" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2953" s="5" t="s">
@@ -13222,10 +13522,10 @@
     </row>
     <row r="3011" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3011" s="13"/>
-      <c r="B3011" s="21" t="s">
+      <c r="B3011" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C3011" s="22"/>
+      <c r="C3011" s="21"/>
     </row>
     <row r="3012" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3012" s="5" t="s">
@@ -13402,10 +13702,10 @@
     </row>
     <row r="3070" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3070" s="13"/>
-      <c r="B3070" s="21" t="s">
+      <c r="B3070" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="C3070" s="22"/>
+      <c r="C3070" s="21"/>
     </row>
     <row r="3071" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3071" s="5" t="s">
@@ -13525,10 +13825,10 @@
     </row>
     <row r="3129" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3129" s="13"/>
-      <c r="B3129" s="21" t="s">
+      <c r="B3129" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="C3129" s="22"/>
+      <c r="C3129" s="21"/>
     </row>
     <row r="3130" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3130" s="5" t="s">
@@ -13668,10 +13968,10 @@
     </row>
     <row r="3188" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3188" s="13"/>
-      <c r="B3188" s="21" t="s">
+      <c r="B3188" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="C3188" s="22"/>
+      <c r="C3188" s="21"/>
     </row>
     <row r="3189" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3189" s="5" t="s">
@@ -13811,10 +14111,10 @@
     </row>
     <row r="3247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3247" s="13"/>
-      <c r="B3247" s="21" t="s">
+      <c r="B3247" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C3247" s="22"/>
+      <c r="C3247" s="21"/>
     </row>
     <row r="3248" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3248" s="5" t="s">
@@ -13905,7 +14205,7 @@
       <c r="A3257" s="3">
         <v>4.2</v>
       </c>
-      <c r="B3257" s="20" t="s">
+      <c r="B3257" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C3257" s="2" t="s">
@@ -13914,7 +14214,7 @@
     </row>
     <row r="3258" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3258" s="3"/>
-      <c r="B3258" s="20"/>
+      <c r="B3258" s="22"/>
       <c r="C3258" s="2"/>
     </row>
     <row r="3259" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -13977,10 +14277,10 @@
     </row>
     <row r="3306" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3306" s="13"/>
-      <c r="B3306" s="21" t="s">
+      <c r="B3306" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="C3306" s="22"/>
+      <c r="C3306" s="21"/>
     </row>
     <row r="3307" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3307" s="5" t="s">
@@ -14122,10 +14422,10 @@
     </row>
     <row r="3365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3365" s="13"/>
-      <c r="B3365" s="21" t="s">
+      <c r="B3365" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="C3365" s="22"/>
+      <c r="C3365" s="21"/>
     </row>
     <row r="3366" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3366" s="5" t="s">
@@ -14218,7 +14518,7 @@
       <c r="A3375" s="3">
         <v>4.2</v>
       </c>
-      <c r="B3375" s="20" t="s">
+      <c r="B3375" s="22" t="s">
         <v>137</v>
       </c>
       <c r="C3375" s="2" t="s">
@@ -14227,7 +14527,7 @@
     </row>
     <row r="3376" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3376" s="3"/>
-      <c r="B3376" s="20"/>
+      <c r="B3376" s="22"/>
       <c r="C3376" s="2"/>
     </row>
     <row r="3377" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -14268,10 +14568,10 @@
     </row>
     <row r="3424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3424" s="13"/>
-      <c r="B3424" s="21" t="s">
+      <c r="B3424" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="C3424" s="22"/>
+      <c r="C3424" s="21"/>
     </row>
     <row r="3425" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3425" s="5" t="s">
@@ -14380,7 +14680,7 @@
       <c r="A3436" s="3">
         <v>4.2</v>
       </c>
-      <c r="B3436" s="20" t="s">
+      <c r="B3436" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C3436" s="2" t="s">
@@ -14389,7 +14689,7 @@
     </row>
     <row r="3437" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3437" s="3"/>
-      <c r="B3437" s="20"/>
+      <c r="B3437" s="22"/>
       <c r="C3437" s="2"/>
     </row>
     <row r="3438" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -14405,7 +14705,7 @@
       <c r="A3439" s="3">
         <v>5.2</v>
       </c>
-      <c r="B3439" s="20" t="s">
+      <c r="B3439" s="22" t="s">
         <v>150</v>
       </c>
       <c r="C3439" s="2" t="s">
@@ -14414,7 +14714,7 @@
     </row>
     <row r="3440" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3440" s="3"/>
-      <c r="B3440" s="20"/>
+      <c r="B3440" s="22"/>
       <c r="C3440" s="2"/>
     </row>
     <row r="3441" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -14455,10 +14755,10 @@
     </row>
     <row r="3483" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3483" s="13"/>
-      <c r="B3483" s="21" t="s">
+      <c r="B3483" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="C3483" s="22"/>
+      <c r="C3483" s="21"/>
     </row>
     <row r="3484" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3484" s="5" t="s">
@@ -14543,14 +14843,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B3492" s="7"/>
-      <c r="C3492" s="20" t="s">
+      <c r="C3492" s="22" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="3493" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3493" s="3"/>
       <c r="B3493" s="7"/>
-      <c r="C3493" s="20"/>
+      <c r="C3493" s="22"/>
     </row>
     <row r="3494" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3494" s="3">
@@ -15339,10 +15639,10 @@
     </row>
     <row r="3896" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3896" s="13"/>
-      <c r="B3896" s="21" t="s">
+      <c r="B3896" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C3896" s="22"/>
+      <c r="C3896" s="21"/>
     </row>
     <row r="3897" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3897" s="5" t="s">
@@ -15464,10 +15764,10 @@
     </row>
     <row r="3955" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3955" s="13"/>
-      <c r="B3955" s="21" t="s">
+      <c r="B3955" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C3955" s="22"/>
+      <c r="C3955" s="21"/>
     </row>
     <row r="3956" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3956" s="5" t="s">
@@ -15979,10 +16279,10 @@
     </row>
     <row r="4191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4191" s="13"/>
-      <c r="B4191" s="21" t="s">
+      <c r="B4191" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="C4191" s="22"/>
+      <c r="C4191" s="21"/>
     </row>
     <row r="4192" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4192" s="5" t="s">
@@ -16073,7 +16373,7 @@
       <c r="A4201" s="3">
         <v>4.2</v>
       </c>
-      <c r="B4201" s="20" t="s">
+      <c r="B4201" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C4201" s="2" t="s">
@@ -16082,7 +16382,7 @@
     </row>
     <row r="4202" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4202" s="3"/>
-      <c r="B4202" s="20"/>
+      <c r="B4202" s="22"/>
       <c r="C4202" s="2"/>
     </row>
     <row r="4203" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -16230,10 +16530,10 @@
     </row>
     <row r="4309" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4309" s="13"/>
-      <c r="B4309" s="21" t="s">
+      <c r="B4309" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="C4309" s="22"/>
+      <c r="C4309" s="21"/>
     </row>
     <row r="4310" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4310" s="5" t="s">
@@ -16393,10 +16693,10 @@
     </row>
     <row r="4368" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4368" s="13"/>
-      <c r="B4368" s="21" t="s">
+      <c r="B4368" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="C4368" s="22"/>
+      <c r="C4368" s="21"/>
     </row>
     <row r="4369" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4369" s="5" t="s">
@@ -16527,10 +16827,10 @@
     </row>
     <row r="4427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4427" s="13"/>
-      <c r="B4427" s="21" t="s">
+      <c r="B4427" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="C4427" s="22"/>
+      <c r="C4427" s="21"/>
     </row>
     <row r="4428" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4428" s="5" t="s">
@@ -16652,10 +16952,10 @@
     </row>
     <row r="4486" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4486" s="13"/>
-      <c r="B4486" s="21" t="s">
+      <c r="B4486" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="C4486" s="22"/>
+      <c r="C4486" s="21"/>
     </row>
     <row r="4487" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4487" s="5" t="s">
@@ -16916,10 +17216,10 @@
     </row>
     <row r="4604" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4604" s="13"/>
-      <c r="B4604" s="21" t="s">
+      <c r="B4604" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="C4604" s="22"/>
+      <c r="C4604" s="21"/>
     </row>
     <row r="4605" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4605" s="5" t="s">
@@ -17561,10 +17861,10 @@
     </row>
     <row r="4840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4840" s="13"/>
-      <c r="B4840" s="21" t="s">
+      <c r="B4840" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C4840" s="22"/>
+      <c r="C4840" s="21"/>
     </row>
     <row r="4841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4841" s="5" t="s">
@@ -17866,10 +18166,10 @@
     </row>
     <row r="4958" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4958" s="13"/>
-      <c r="B4958" s="21" t="s">
+      <c r="B4958" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="C4958" s="22"/>
+      <c r="C4958" s="21"/>
     </row>
     <row r="4959" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4959" s="5" t="s">
@@ -17989,10 +18289,10 @@
     </row>
     <row r="5017" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5017" s="13"/>
-      <c r="B5017" s="21" t="s">
+      <c r="B5017" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="C5017" s="22"/>
+      <c r="C5017" s="21"/>
     </row>
     <row r="5018" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5018" s="5" t="s">
@@ -18132,10 +18432,10 @@
     </row>
     <row r="5076" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5076" s="13"/>
-      <c r="B5076" s="21" t="s">
+      <c r="B5076" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="C5076" s="22"/>
+      <c r="C5076" s="21"/>
     </row>
     <row r="5077" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5077" s="5" t="s">
@@ -18275,10 +18575,10 @@
     </row>
     <row r="5135" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5135" s="13"/>
-      <c r="B5135" s="21" t="s">
+      <c r="B5135" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C5135" s="22"/>
+      <c r="C5135" s="21"/>
     </row>
     <row r="5136" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5136" s="5" t="s">
@@ -18369,7 +18669,7 @@
       <c r="A5145" s="3">
         <v>4.2</v>
       </c>
-      <c r="B5145" s="20" t="s">
+      <c r="B5145" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C5145" s="2" t="s">
@@ -18378,7 +18678,7 @@
     </row>
     <row r="5146" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5146" s="3"/>
-      <c r="B5146" s="20"/>
+      <c r="B5146" s="22"/>
       <c r="C5146" s="2"/>
     </row>
     <row r="5147" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18441,10 +18741,10 @@
     </row>
     <row r="5194" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5194" s="13"/>
-      <c r="B5194" s="21" t="s">
+      <c r="B5194" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="C5194" s="22"/>
+      <c r="C5194" s="21"/>
     </row>
     <row r="5195" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5195" s="5" t="s">
@@ -18586,10 +18886,10 @@
     </row>
     <row r="5253" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5253" s="13"/>
-      <c r="B5253" s="21" t="s">
+      <c r="B5253" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="C5253" s="22"/>
+      <c r="C5253" s="21"/>
     </row>
     <row r="5254" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5254" s="5" t="s">
@@ -18682,7 +18982,7 @@
       <c r="A5263" s="3">
         <v>4.2</v>
       </c>
-      <c r="B5263" s="20" t="s">
+      <c r="B5263" s="22" t="s">
         <v>137</v>
       </c>
       <c r="C5263" s="2" t="s">
@@ -18691,7 +18991,7 @@
     </row>
     <row r="5264" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5264" s="3"/>
-      <c r="B5264" s="20"/>
+      <c r="B5264" s="22"/>
       <c r="C5264" s="2"/>
     </row>
     <row r="5265" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18810,7 +19110,7 @@
       <c r="A5320" s="3">
         <v>3.2</v>
       </c>
-      <c r="B5320" s="20" t="s">
+      <c r="B5320" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C5320" s="2" t="s">
@@ -18819,7 +19119,7 @@
     </row>
     <row r="5321" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5321" s="3"/>
-      <c r="B5321" s="20"/>
+      <c r="B5321" s="22"/>
       <c r="C5321" s="2"/>
     </row>
     <row r="5322" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18862,10 +19162,10 @@
     </row>
     <row r="5371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5371" s="13"/>
-      <c r="B5371" s="21" t="s">
+      <c r="B5371" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="C5371" s="22"/>
+      <c r="C5371" s="21"/>
     </row>
     <row r="5372" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5372" s="5" t="s">
@@ -19677,10 +19977,10 @@
     </row>
     <row r="5784" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5784" s="13"/>
-      <c r="B5784" s="21" t="s">
+      <c r="B5784" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C5784" s="22"/>
+      <c r="C5784" s="21"/>
     </row>
     <row r="5785" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5785" s="5" t="s">
@@ -19802,10 +20102,10 @@
     </row>
     <row r="5843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5843" s="13"/>
-      <c r="B5843" s="21" t="s">
+      <c r="B5843" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C5843" s="22"/>
+      <c r="C5843" s="21"/>
     </row>
     <row r="5844" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5844" s="5" t="s">
@@ -20317,10 +20617,10 @@
     </row>
     <row r="6079" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6079" s="13"/>
-      <c r="B6079" s="21" t="s">
+      <c r="B6079" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="C6079" s="22"/>
+      <c r="C6079" s="21"/>
     </row>
     <row r="6080" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6080" s="5" t="s">
@@ -20411,7 +20711,7 @@
       <c r="A6089" s="3">
         <v>4.2</v>
       </c>
-      <c r="B6089" s="20" t="s">
+      <c r="B6089" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C6089" s="2" t="s">
@@ -20420,7 +20720,7 @@
     </row>
     <row r="6090" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6090" s="3"/>
-      <c r="B6090" s="20"/>
+      <c r="B6090" s="22"/>
       <c r="C6090" s="2"/>
     </row>
     <row r="6091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -20568,10 +20868,10 @@
     </row>
     <row r="6197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6197" s="13"/>
-      <c r="B6197" s="21" t="s">
+      <c r="B6197" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="C6197" s="22"/>
+      <c r="C6197" s="21"/>
     </row>
     <row r="6198" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6198" s="5" t="s">
@@ -20865,10 +21165,10 @@
     </row>
     <row r="6315" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6315" s="13"/>
-      <c r="B6315" s="21" t="s">
+      <c r="B6315" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="C6315" s="22"/>
+      <c r="C6315" s="21"/>
     </row>
     <row r="6316" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6316" s="5" t="s">
@@ -20937,14 +21237,14 @@
         <v>3.1</v>
       </c>
       <c r="B6322" s="7"/>
-      <c r="C6322" s="20" t="s">
+      <c r="C6322" s="22" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="6323" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6323" s="3"/>
       <c r="B6323" s="7"/>
-      <c r="C6323" s="20"/>
+      <c r="C6323" s="22"/>
     </row>
     <row r="6324" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6324" s="3">
@@ -20995,10 +21295,10 @@
     </row>
     <row r="6374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6374" s="13"/>
-      <c r="B6374" s="21" t="s">
+      <c r="B6374" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="C6374" s="22"/>
+      <c r="C6374" s="21"/>
     </row>
     <row r="6375" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6375" s="5" t="s">
@@ -21900,10 +22200,10 @@
     </row>
     <row r="6728" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6728" s="13"/>
-      <c r="B6728" s="21" t="s">
+      <c r="B6728" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C6728" s="22"/>
+      <c r="C6728" s="21"/>
     </row>
     <row r="6729" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6729" s="5" t="s">
@@ -22025,10 +22325,10 @@
     </row>
     <row r="6787" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6787" s="13"/>
-      <c r="B6787" s="21" t="s">
+      <c r="B6787" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="C6787" s="22"/>
+      <c r="C6787" s="21"/>
     </row>
     <row r="6788" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6788" s="5" t="s">
@@ -22205,10 +22505,10 @@
     </row>
     <row r="6846" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6846" s="13"/>
-      <c r="B6846" s="21" t="s">
+      <c r="B6846" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="C6846" s="22"/>
+      <c r="C6846" s="21"/>
     </row>
     <row r="6847" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6847" s="5" t="s">
@@ -22328,10 +22628,10 @@
     </row>
     <row r="6905" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6905" s="13"/>
-      <c r="B6905" s="21" t="s">
+      <c r="B6905" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="C6905" s="22"/>
+      <c r="C6905" s="21"/>
     </row>
     <row r="6906" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6906" s="5" t="s">
@@ -22471,10 +22771,10 @@
     </row>
     <row r="6964" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6964" s="13"/>
-      <c r="B6964" s="21" t="s">
+      <c r="B6964" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="C6964" s="22"/>
+      <c r="C6964" s="21"/>
     </row>
     <row r="6965" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6965" s="5" t="s">
@@ -22614,10 +22914,10 @@
     </row>
     <row r="7023" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7023" s="13"/>
-      <c r="B7023" s="21" t="s">
+      <c r="B7023" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="C7023" s="22"/>
+      <c r="C7023" s="21"/>
     </row>
     <row r="7024" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7024" s="5" t="s">
@@ -22708,7 +23008,7 @@
       <c r="A7033" s="3">
         <v>4.2</v>
       </c>
-      <c r="B7033" s="20" t="s">
+      <c r="B7033" s="22" t="s">
         <v>88</v>
       </c>
       <c r="C7033" s="2" t="s">
@@ -22717,7 +23017,7 @@
     </row>
     <row r="7034" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7034" s="3"/>
-      <c r="B7034" s="20"/>
+      <c r="B7034" s="22"/>
       <c r="C7034" s="2"/>
     </row>
     <row r="7035" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -22780,10 +23080,10 @@
     </row>
     <row r="7082" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7082" s="13"/>
-      <c r="B7082" s="21" t="s">
+      <c r="B7082" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="C7082" s="22"/>
+      <c r="C7082" s="21"/>
     </row>
     <row r="7083" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7083" s="5" t="s">
@@ -22925,10 +23225,10 @@
     </row>
     <row r="7141" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7141" s="13"/>
-      <c r="B7141" s="21" t="s">
+      <c r="B7141" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="C7141" s="22"/>
+      <c r="C7141" s="21"/>
     </row>
     <row r="7142" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7142" s="5" t="s">
@@ -23021,7 +23321,7 @@
       <c r="A7151" s="3">
         <v>4.2</v>
       </c>
-      <c r="B7151" s="20" t="s">
+      <c r="B7151" s="22" t="s">
         <v>137</v>
       </c>
       <c r="C7151" s="2" t="s">
@@ -23030,7 +23330,7 @@
     </row>
     <row r="7152" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7152" s="3"/>
-      <c r="B7152" s="20"/>
+      <c r="B7152" s="22"/>
       <c r="C7152" s="2"/>
     </row>
     <row r="7153" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -23058,13 +23358,279 @@
       <c r="B7155" s="9"/>
       <c r="C7155" s="8"/>
     </row>
+    <row r="7199" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7199" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="B7199" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7199" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7200" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7200" s="13"/>
+      <c r="B7200" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="C7200" s="21"/>
+    </row>
+    <row r="7201" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7201" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7201" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7201" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7202" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7202" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7202" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7202" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7203" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7203" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B7203" s="7"/>
+      <c r="C7203" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7204" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7204" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B7204" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7204" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7205" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7205" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B7205" s="7"/>
+      <c r="C7205" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7206" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7206" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7206" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7206" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="7207" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7207" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B7207" s="7"/>
+      <c r="C7207" s="2"/>
+    </row>
+    <row r="7208" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7208" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B7208" s="7"/>
+      <c r="C7208" s="2"/>
+    </row>
+    <row r="7209" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7209" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B7209" s="7"/>
+      <c r="C7209" s="2"/>
+    </row>
+    <row r="7210" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7210" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B7210" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7210" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="7211" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7211" s="3"/>
+      <c r="B7211" s="22"/>
+      <c r="C7211" s="2"/>
+    </row>
+    <row r="7212" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7212" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B7212" s="7"/>
+      <c r="C7212" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7213" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7213" s="3"/>
+      <c r="B7213" s="7"/>
+      <c r="C7213" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="7214" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7214" s="3"/>
+      <c r="B7214" s="7"/>
+      <c r="C7214" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="7215" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7215" s="3"/>
+      <c r="B7215" s="7"/>
+      <c r="C7215" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="7216" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7216" s="3"/>
+      <c r="B7216" s="7"/>
+      <c r="C7216" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="7217" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7217" s="3"/>
+      <c r="B7217" s="7"/>
+      <c r="C7217" s="2" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="7218" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7218" s="3"/>
+      <c r="B7218" s="7"/>
+      <c r="C7218" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="7219" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7219" s="3"/>
+      <c r="B7219" s="7"/>
+      <c r="C7219" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="7220" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7220" s="3"/>
+      <c r="B7220" s="7"/>
+      <c r="C7220" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="7221" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7221" s="3"/>
+      <c r="B7221" s="7"/>
+      <c r="C7221" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="7222" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7222" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B7222" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7222" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7223" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7223" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7223" s="9"/>
+      <c r="C7223" s="8"/>
+    </row>
   </sheetData>
-  <mergeCells count="83">
-    <mergeCell ref="B1595:C1595"/>
-    <mergeCell ref="B1548:B1549"/>
-    <mergeCell ref="B1551:B1552"/>
-    <mergeCell ref="B3365:C3365"/>
-    <mergeCell ref="B3375:B3376"/>
+  <mergeCells count="85">
+    <mergeCell ref="B7200:C7200"/>
+    <mergeCell ref="B7210:B7211"/>
+    <mergeCell ref="B7151:B7152"/>
+    <mergeCell ref="B7141:C7141"/>
+    <mergeCell ref="B6787:C6787"/>
+    <mergeCell ref="B6846:C6846"/>
+    <mergeCell ref="B6905:C6905"/>
+    <mergeCell ref="B6964:C6964"/>
+    <mergeCell ref="B7023:C7023"/>
+    <mergeCell ref="B7033:B7034"/>
+    <mergeCell ref="B7082:C7082"/>
+    <mergeCell ref="B5371:C5371"/>
+    <mergeCell ref="B5784:C5784"/>
+    <mergeCell ref="B5843:C5843"/>
+    <mergeCell ref="B6079:C6079"/>
+    <mergeCell ref="B6089:B6090"/>
+    <mergeCell ref="B5320:B5321"/>
+    <mergeCell ref="B4486:C4486"/>
+    <mergeCell ref="B4604:C4604"/>
+    <mergeCell ref="B4840:C4840"/>
+    <mergeCell ref="B4958:C4958"/>
+    <mergeCell ref="B5017:C5017"/>
+    <mergeCell ref="B5076:C5076"/>
+    <mergeCell ref="B5135:C5135"/>
+    <mergeCell ref="B5145:B5146"/>
+    <mergeCell ref="B5194:C5194"/>
+    <mergeCell ref="B5253:C5253"/>
+    <mergeCell ref="B5263:B5264"/>
+    <mergeCell ref="B4427:C4427"/>
+    <mergeCell ref="B2952:C2952"/>
+    <mergeCell ref="B3011:C3011"/>
+    <mergeCell ref="B3070:C3070"/>
+    <mergeCell ref="B3129:C3129"/>
+    <mergeCell ref="B3188:C3188"/>
+    <mergeCell ref="B3247:C3247"/>
+    <mergeCell ref="B3257:B3258"/>
+    <mergeCell ref="B3306:C3306"/>
+    <mergeCell ref="B3896:C3896"/>
+    <mergeCell ref="B3955:C3955"/>
+    <mergeCell ref="B4191:C4191"/>
+    <mergeCell ref="B4201:B4202"/>
+    <mergeCell ref="B4309:C4309"/>
+    <mergeCell ref="B4368:C4368"/>
+    <mergeCell ref="B120:C120"/>
+    <mergeCell ref="B179:C179"/>
+    <mergeCell ref="B425:B426"/>
+    <mergeCell ref="B533:C533"/>
+    <mergeCell ref="B651:C651"/>
+    <mergeCell ref="B710:C710"/>
+    <mergeCell ref="B356:C356"/>
+    <mergeCell ref="B6197:C6197"/>
+    <mergeCell ref="B6315:C6315"/>
+    <mergeCell ref="C6322:C6323"/>
+    <mergeCell ref="B1064:C1064"/>
+    <mergeCell ref="B1123:C1123"/>
+    <mergeCell ref="B1182:C1182"/>
+    <mergeCell ref="B1241:C1241"/>
+    <mergeCell ref="B1369:B1370"/>
+    <mergeCell ref="B1359:C1359"/>
+    <mergeCell ref="B1300:C1300"/>
+    <mergeCell ref="B1418:C1418"/>
+    <mergeCell ref="B1487:B1488"/>
+    <mergeCell ref="B828:C828"/>
+    <mergeCell ref="B1536:C1536"/>
     <mergeCell ref="B6374:C6374"/>
     <mergeCell ref="B6728:C6728"/>
     <mergeCell ref="B1831:C1831"/>
@@ -23081,68 +23647,11 @@
     <mergeCell ref="B3439:B3440"/>
     <mergeCell ref="B3483:C3483"/>
     <mergeCell ref="C3492:C3493"/>
-    <mergeCell ref="B710:C710"/>
-    <mergeCell ref="B356:C356"/>
-    <mergeCell ref="B6197:C6197"/>
-    <mergeCell ref="B6315:C6315"/>
-    <mergeCell ref="C6322:C6323"/>
-    <mergeCell ref="B1064:C1064"/>
-    <mergeCell ref="B1123:C1123"/>
-    <mergeCell ref="B1182:C1182"/>
-    <mergeCell ref="B1241:C1241"/>
-    <mergeCell ref="B1369:B1370"/>
-    <mergeCell ref="B1359:C1359"/>
-    <mergeCell ref="B1300:C1300"/>
-    <mergeCell ref="B1418:C1418"/>
-    <mergeCell ref="B1487:B1488"/>
-    <mergeCell ref="B828:C828"/>
-    <mergeCell ref="B1536:C1536"/>
-    <mergeCell ref="B120:C120"/>
-    <mergeCell ref="B179:C179"/>
-    <mergeCell ref="B425:B426"/>
-    <mergeCell ref="B533:C533"/>
-    <mergeCell ref="B651:C651"/>
-    <mergeCell ref="B4427:C4427"/>
-    <mergeCell ref="B2952:C2952"/>
-    <mergeCell ref="B3011:C3011"/>
-    <mergeCell ref="B3070:C3070"/>
-    <mergeCell ref="B3129:C3129"/>
-    <mergeCell ref="B3188:C3188"/>
-    <mergeCell ref="B3247:C3247"/>
-    <mergeCell ref="B3257:B3258"/>
-    <mergeCell ref="B3306:C3306"/>
-    <mergeCell ref="B3896:C3896"/>
-    <mergeCell ref="B3955:C3955"/>
-    <mergeCell ref="B4191:C4191"/>
-    <mergeCell ref="B4201:B4202"/>
-    <mergeCell ref="B4309:C4309"/>
-    <mergeCell ref="B4368:C4368"/>
-    <mergeCell ref="B5320:B5321"/>
-    <mergeCell ref="B4486:C4486"/>
-    <mergeCell ref="B4604:C4604"/>
-    <mergeCell ref="B4840:C4840"/>
-    <mergeCell ref="B4958:C4958"/>
-    <mergeCell ref="B5017:C5017"/>
-    <mergeCell ref="B5076:C5076"/>
-    <mergeCell ref="B5135:C5135"/>
-    <mergeCell ref="B5145:B5146"/>
-    <mergeCell ref="B5194:C5194"/>
-    <mergeCell ref="B5253:C5253"/>
-    <mergeCell ref="B5263:B5264"/>
-    <mergeCell ref="B5371:C5371"/>
-    <mergeCell ref="B5784:C5784"/>
-    <mergeCell ref="B5843:C5843"/>
-    <mergeCell ref="B6079:C6079"/>
-    <mergeCell ref="B6089:B6090"/>
-    <mergeCell ref="B7151:B7152"/>
-    <mergeCell ref="B7141:C7141"/>
-    <mergeCell ref="B6787:C6787"/>
-    <mergeCell ref="B6846:C6846"/>
-    <mergeCell ref="B6905:C6905"/>
-    <mergeCell ref="B6964:C6964"/>
-    <mergeCell ref="B7023:C7023"/>
-    <mergeCell ref="B7033:B7034"/>
-    <mergeCell ref="B7082:C7082"/>
+    <mergeCell ref="B1595:C1595"/>
+    <mergeCell ref="B1548:B1549"/>
+    <mergeCell ref="B1551:B1552"/>
+    <mergeCell ref="B3365:C3365"/>
+    <mergeCell ref="B3375:B3376"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup scale="79" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
SPC-700 instructions up to 9F.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7AE86F-FDF1-4876-80A0-690923420559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1385263-710F-42A8-91EC-37991203BF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3686" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3704" uniqueCount="407">
   <si>
     <t>Implied</t>
   </si>
@@ -7822,6 +7822,223 @@
   </si>
   <si>
     <t>If DivYa &amp; $20000: DivYa ^= $20001.</t>
+  </si>
+  <si>
+    <t>XCN (9F)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &gt;&gt; 7) | (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;&lt; 1).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &gt;&gt; 7) | (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;&lt; 1). </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; $80), </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = !</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -8400,7 +8617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C9380"/>
+  <dimension ref="A1:C9396"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -31212,6 +31429,137 @@
       </c>
       <c r="B9380" s="9"/>
       <c r="C9380" s="8"/>
+    </row>
+    <row r="9382" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9382" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="B9382" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9382" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9383" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9383" s="13"/>
+      <c r="B9383" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9383" s="18"/>
+    </row>
+    <row r="9384" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9384" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9384" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9384" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9385" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9385" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9385" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9385" s="23" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9386" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9386" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B9386" s="7"/>
+      <c r="C9386" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9387" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9387" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B9387" s="7"/>
+      <c r="C9387" s="2"/>
+    </row>
+    <row r="9388" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9388" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B9388" s="7"/>
+      <c r="C9388" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="9389" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9389" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9389" s="7"/>
+      <c r="C9389" s="2"/>
+    </row>
+    <row r="9390" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9390" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B9390" s="7"/>
+      <c r="C9390" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="9391" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9391" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B9391" s="7"/>
+      <c r="C9391" s="2"/>
+    </row>
+    <row r="9392" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9392" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B9392" s="7"/>
+      <c r="C9392" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="9393" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9393" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B9393" s="7"/>
+      <c r="C9393" s="2"/>
+    </row>
+    <row r="9394" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9394" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9394" s="7"/>
+      <c r="C9394" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="9395" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9395" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B9395" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9395" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9396" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9396" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9396" s="9"/>
+      <c r="C9396" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="107">

</xml_diff>

<commit_message>
Big major comment change.
</commit_message>
<xml_diff>
--- a/Research/Instructions/SPC-700 Instructions SNES.xlsx
+++ b/Research/Instructions/SPC-700 Instructions SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D9CBFA-9462-46D4-97FC-BF20AF5B0C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D2C45C-7AC4-4466-B214-DD17A5E88B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$11210</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$11553</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4433" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4564" uniqueCount="483">
   <si>
     <t>Implied</t>
   </si>
@@ -8995,6 +8995,86 @@
       </rPr>
       <t>.</t>
     </r>
+  </si>
+  <si>
+    <t>DI (C0)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp; ~$04).</t>
+    </r>
+  </si>
+  <si>
+    <t>TCALL12 (C1)</t>
+  </si>
+  <si>
+    <t>Read $FFC6</t>
+  </si>
+  <si>
+    <t>Read $FFC7</t>
+  </si>
+  <si>
+    <t>SET1 (A2)</t>
+  </si>
+  <si>
+    <t>Operand = (Operand &amp; ~$20) | $20.</t>
+  </si>
+  <si>
+    <t>SET1 (C2)</t>
+  </si>
+  <si>
+    <t>Operand = (Operand &amp; ~$40) | $40.</t>
+  </si>
+  <si>
+    <t>BBS6 (C3)</t>
+  </si>
+  <si>
+    <t>Set Jump to (Operand &amp; (1 &lt;&lt; 6)) == (1 &lt;&lt; 6).</t>
+  </si>
+  <si>
+    <t>MOV (C4)</t>
+  </si>
+  <si>
+    <t>Direct Page d (Write)</t>
   </si>
 </sst>
 </file>
@@ -9576,7 +9656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C11164"/>
+  <dimension ref="A1:C11518"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="19" customWidth="1"/>
@@ -32806,21 +32886,21 @@
     </row>
     <row r="9559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9559" s="10" t="s">
-        <v>400</v>
+        <v>475</v>
       </c>
       <c r="B9559" s="11" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="C9559" s="12" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9560" s="13"/>
-      <c r="B9560" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C9560" s="18"/>
+      <c r="B9560" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9560" s="23"/>
     </row>
     <row r="9561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9561" s="5" t="s">
@@ -32890,15 +32970,19 @@
       </c>
       <c r="B9567" s="7"/>
       <c r="C9567" s="2" t="s">
-        <v>401</v>
+        <v>476</v>
       </c>
     </row>
     <row r="9568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9568" s="3">
         <v>3.2</v>
       </c>
-      <c r="B9568" s="7"/>
-      <c r="C9568" s="2"/>
+      <c r="B9568" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9568" s="2" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="9569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9569" s="3">
@@ -32915,90 +32999,31 @@
         <v>47</v>
       </c>
       <c r="C9570" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9571" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9571" s="3">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B9571" s="7"/>
-      <c r="C9571" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9572" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9572" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B9572" s="7"/>
-      <c r="C9572" s="2"/>
-    </row>
-    <row r="9573" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9573" s="3">
-        <v>6.1</v>
-      </c>
-      <c r="B9573" s="7"/>
-      <c r="C9573" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="9574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9574" s="3"/>
-      <c r="B9574" s="7"/>
-      <c r="C9574" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9575" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="B9575" s="7"/>
-      <c r="C9575" s="2"/>
-    </row>
-    <row r="9576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9576" s="3">
-        <v>7.1</v>
-      </c>
-      <c r="B9576" s="7"/>
-      <c r="C9576" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9577" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9577" s="3">
-        <v>7.2</v>
-      </c>
-      <c r="B9577" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9577" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9578" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9578" s="16" t="s">
+      <c r="A9571" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9578" s="9"/>
-      <c r="C9578" s="8"/>
+      <c r="B9571" s="9"/>
+      <c r="C9571" s="8"/>
     </row>
     <row r="9618" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9618" s="10" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B9618" s="11" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="C9618" s="12" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9619" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9619" s="13"/>
       <c r="B9619" s="17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C9619" s="18"/>
     </row>
@@ -33070,91 +33095,115 @@
       </c>
       <c r="B9626" s="7"/>
       <c r="C9626" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9627" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9627" s="3"/>
+      <c r="A9627" s="3">
+        <v>3.2</v>
+      </c>
       <c r="B9627" s="7"/>
-      <c r="C9627" s="2" t="s">
-        <v>404</v>
-      </c>
+      <c r="C9627" s="2"/>
     </row>
     <row r="9628" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9628" s="3"/>
+      <c r="A9628" s="3">
+        <v>4.0999999999999996</v>
+      </c>
       <c r="B9628" s="7"/>
-      <c r="C9628" s="2" t="s">
-        <v>303</v>
-      </c>
+      <c r="C9628" s="2"/>
     </row>
     <row r="9629" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9629" s="3"/>
-      <c r="B9629" s="7"/>
+      <c r="A9629" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B9629" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C9629" s="2" t="s">
-        <v>334</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9630" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9630" s="3"/>
+      <c r="A9630" s="3">
+        <v>5.0999999999999996</v>
+      </c>
       <c r="B9630" s="7"/>
       <c r="C9630" s="2" t="s">
-        <v>405</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9631" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9631" s="3"/>
+      <c r="A9631" s="3">
+        <v>5.2</v>
+      </c>
       <c r="B9631" s="7"/>
-      <c r="C9631" s="2" t="s">
-        <v>406</v>
-      </c>
+      <c r="C9631" s="2"/>
     </row>
     <row r="9632" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9632" s="3"/>
+      <c r="A9632" s="3">
+        <v>6.1</v>
+      </c>
       <c r="B9632" s="7"/>
       <c r="C9632" s="2" t="s">
-        <v>308</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9633" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9633" s="3"/>
       <c r="B9633" s="7"/>
       <c r="C9633" s="2" t="s">
-        <v>304</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9634" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9634" s="3">
-        <v>3.2</v>
-      </c>
-      <c r="B9634" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9634" s="2" t="s">
-        <v>5</v>
-      </c>
+        <v>6.2</v>
+      </c>
+      <c r="B9634" s="7"/>
+      <c r="C9634" s="2"/>
     </row>
     <row r="9635" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9635" s="16" t="s">
+      <c r="A9635" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B9635" s="7"/>
+      <c r="C9635" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9636" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9636" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B9636" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9636" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9637" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9637" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9635" s="9"/>
-      <c r="C9635" s="8"/>
+      <c r="B9637" s="9"/>
+      <c r="C9637" s="8"/>
     </row>
     <row r="9677" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9677" s="10" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B9677" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C9677" s="12" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9678" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9678" s="13"/>
       <c r="B9678" s="17" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C9678" s="18"/>
     </row>
@@ -33193,22 +33242,28 @@
       <c r="A9682" s="3">
         <v>1.2</v>
       </c>
-      <c r="B9682" s="7"/>
-      <c r="C9682" s="2"/>
+      <c r="B9682" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9682" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="9683" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9683" s="3">
         <v>2.1</v>
       </c>
       <c r="B9683" s="7"/>
-      <c r="C9683" s="2"/>
+      <c r="C9683" s="2" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="9684" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9684" s="3">
         <v>2.2000000000000002</v>
       </c>
       <c r="B9684" s="7" t="s">
-        <v>410</v>
+        <v>7</v>
       </c>
       <c r="C9684" s="2" t="s">
         <v>6</v>
@@ -33292,21 +33347,21 @@
     </row>
     <row r="9736" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9736" s="10" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B9736" s="11" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C9736" s="12" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9737" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9737" s="13"/>
-      <c r="B9737" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="C9737" s="23"/>
+      <c r="B9737" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9737" s="18"/>
     </row>
     <row r="9738" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9738" s="5" t="s">
@@ -33343,28 +33398,26 @@
       <c r="A9741" s="3">
         <v>1.2</v>
       </c>
-      <c r="B9741" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9741" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="B9741" s="7"/>
+      <c r="C9741" s="2"/>
     </row>
     <row r="9742" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9742" s="3">
         <v>2.1</v>
       </c>
       <c r="B9742" s="7"/>
-      <c r="C9742" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="C9742" s="2"/>
     </row>
     <row r="9743" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9743" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B9743" s="7"/>
-      <c r="C9743" s="2"/>
+      <c r="B9743" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="C9743" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="9744" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9744" s="3">
@@ -33372,143 +33425,82 @@
       </c>
       <c r="B9744" s="7"/>
       <c r="C9744" s="2" t="s">
-        <v>411</v>
+        <v>403</v>
       </c>
     </row>
     <row r="9745" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9745" s="3">
-        <v>3.2</v>
-      </c>
-      <c r="B9745" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="A9745" s="3"/>
+      <c r="B9745" s="7"/>
       <c r="C9745" s="2" t="s">
-        <v>65</v>
+        <v>404</v>
       </c>
     </row>
     <row r="9746" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9746" s="3">
-        <v>4.0999999999999996</v>
-      </c>
+      <c r="A9746" s="3"/>
       <c r="B9746" s="7"/>
-      <c r="C9746" s="2"/>
+      <c r="C9746" s="2" t="s">
+        <v>303</v>
+      </c>
     </row>
     <row r="9747" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9747" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B9747" s="24" t="s">
-        <v>412</v>
-      </c>
+      <c r="A9747" s="3"/>
+      <c r="B9747" s="7"/>
       <c r="C9747" s="2" t="s">
-        <v>20</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9748" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9748" s="3"/>
-      <c r="B9748" s="24"/>
-      <c r="C9748" s="2"/>
+      <c r="B9748" s="7"/>
+      <c r="C9748" s="2" t="s">
+        <v>405</v>
+      </c>
     </row>
     <row r="9749" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9749" s="3">
-        <v>5.0999999999999996</v>
-      </c>
+      <c r="A9749" s="3"/>
       <c r="B9749" s="7"/>
-      <c r="C9749" s="2"/>
+      <c r="C9749" s="2" t="s">
+        <v>406</v>
+      </c>
     </row>
     <row r="9750" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9750" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B9750" s="7" t="s">
-        <v>42</v>
-      </c>
+      <c r="A9750" s="3"/>
+      <c r="B9750" s="7"/>
       <c r="C9750" s="2" t="s">
-        <v>6</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9751" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9751" s="3">
-        <v>6.1</v>
-      </c>
+      <c r="A9751" s="3"/>
       <c r="B9751" s="7"/>
       <c r="C9751" s="2" t="s">
-        <v>403</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9752" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9752" s="3"/>
-      <c r="B9752" s="7"/>
+      <c r="A9752" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B9752" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C9752" s="2" t="s">
-        <v>404</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9753" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9753" s="3"/>
-      <c r="B9753" s="7"/>
-      <c r="C9753" s="2" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="9754" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9754" s="3"/>
-      <c r="B9754" s="7"/>
-      <c r="C9754" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="9755" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9755" s="3"/>
-      <c r="B9755" s="7"/>
-      <c r="C9755" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="9756" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9756" s="3"/>
-      <c r="B9756" s="7"/>
-      <c r="C9756" s="2" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="9757" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9757" s="3"/>
-      <c r="B9757" s="7"/>
-      <c r="C9757" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="9758" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9758" s="3"/>
-      <c r="B9758" s="7"/>
-      <c r="C9758" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="9759" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9759" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="B9759" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9759" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9760" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9760" s="16" t="s">
+      <c r="A9753" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9760" s="9"/>
-      <c r="C9760" s="8"/>
+      <c r="B9753" s="9"/>
+      <c r="C9753" s="8"/>
     </row>
     <row r="9795" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9795" s="10" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="B9795" s="11" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C9795" s="12" t="s">
         <v>4</v>
@@ -33516,10 +33508,10 @@
     </row>
     <row r="9796" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9796" s="13"/>
-      <c r="B9796" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9796" s="18"/>
+      <c r="B9796" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C9796" s="23"/>
     </row>
     <row r="9797" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9797" s="5" t="s">
@@ -33569,93 +33561,170 @@
       </c>
       <c r="B9801" s="7"/>
       <c r="C9801" s="2" t="s">
-        <v>418</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9802" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9802" s="3"/>
+      <c r="A9802" s="3">
+        <v>2.2000000000000002</v>
+      </c>
       <c r="B9802" s="7"/>
-      <c r="C9802" s="2" t="s">
-        <v>404</v>
-      </c>
+      <c r="C9802" s="2"/>
     </row>
     <row r="9803" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9803" s="3"/>
+      <c r="A9803" s="3">
+        <v>3.1</v>
+      </c>
       <c r="B9803" s="7"/>
       <c r="C9803" s="2" t="s">
-        <v>303</v>
+        <v>411</v>
       </c>
     </row>
     <row r="9804" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9804" s="3"/>
-      <c r="B9804" s="7"/>
+      <c r="A9804" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B9804" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="C9804" s="2" t="s">
-        <v>334</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9805" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9805" s="3"/>
+      <c r="A9805" s="3">
+        <v>4.0999999999999996</v>
+      </c>
       <c r="B9805" s="7"/>
-      <c r="C9805" s="2" t="s">
-        <v>405</v>
-      </c>
+      <c r="C9805" s="2"/>
     </row>
     <row r="9806" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9806" s="3"/>
-      <c r="B9806" s="2"/>
+      <c r="A9806" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B9806" s="24" t="s">
+        <v>412</v>
+      </c>
       <c r="C9806" s="2" t="s">
-        <v>406</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9807" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9807" s="3"/>
-      <c r="B9807" s="2"/>
-      <c r="C9807" s="2" t="s">
-        <v>308</v>
-      </c>
+      <c r="B9807" s="24"/>
+      <c r="C9807" s="2"/>
     </row>
     <row r="9808" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9808" s="3"/>
+      <c r="A9808" s="3">
+        <v>5.0999999999999996</v>
+      </c>
       <c r="B9808" s="7"/>
-      <c r="C9808" s="2" t="s">
-        <v>304</v>
-      </c>
+      <c r="C9808" s="2"/>
     </row>
     <row r="9809" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9809" s="3">
-        <v>2.2000000000000002</v>
+        <v>5.2</v>
       </c>
       <c r="B9809" s="7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C9809" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9810" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9810" s="16" t="s">
+      <c r="A9810" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B9810" s="7"/>
+      <c r="C9810" s="2" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="9811" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9811" s="3"/>
+      <c r="B9811" s="7"/>
+      <c r="C9811" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="9812" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9812" s="3"/>
+      <c r="B9812" s="7"/>
+      <c r="C9812" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="9813" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9813" s="3"/>
+      <c r="B9813" s="7"/>
+      <c r="C9813" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="9814" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9814" s="3"/>
+      <c r="B9814" s="7"/>
+      <c r="C9814" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="9815" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9815" s="3"/>
+      <c r="B9815" s="7"/>
+      <c r="C9815" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="9816" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9816" s="3"/>
+      <c r="B9816" s="7"/>
+      <c r="C9816" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="9817" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9817" s="3"/>
+      <c r="B9817" s="7"/>
+      <c r="C9817" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="9818" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9818" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B9818" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9818" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9819" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9819" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9810" s="9"/>
-      <c r="C9810" s="8"/>
+      <c r="B9819" s="9"/>
+      <c r="C9819" s="8"/>
     </row>
     <row r="9854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9854" s="10" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B9854" s="11" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C9854" s="12" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9855" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9855" s="13"/>
-      <c r="B9855" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="C9855" s="23"/>
+      <c r="B9855" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9855" s="18"/>
     </row>
     <row r="9856" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9856" s="5" t="s">
@@ -33705,158 +33774,82 @@
       </c>
       <c r="B9860" s="7"/>
       <c r="C9860" s="2" t="s">
-        <v>409</v>
+        <v>418</v>
       </c>
     </row>
     <row r="9861" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9861" s="3">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="B9861" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="A9861" s="3"/>
+      <c r="B9861" s="7"/>
       <c r="C9861" s="2" t="s">
-        <v>68</v>
+        <v>404</v>
       </c>
     </row>
     <row r="9862" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9862" s="3">
-        <v>3.1</v>
-      </c>
+      <c r="A9862" s="3"/>
       <c r="B9862" s="7"/>
-      <c r="C9862" s="2"/>
+      <c r="C9862" s="2" t="s">
+        <v>303</v>
+      </c>
     </row>
     <row r="9863" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9863" s="3">
-        <v>3.2</v>
-      </c>
-      <c r="B9863" s="7" t="s">
-        <v>47</v>
-      </c>
+      <c r="A9863" s="3"/>
+      <c r="B9863" s="7"/>
       <c r="C9863" s="2" t="s">
-        <v>6</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9864" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9864" s="3">
-        <v>4.0999999999999996</v>
-      </c>
+      <c r="A9864" s="3"/>
       <c r="B9864" s="7"/>
       <c r="C9864" s="2" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="9865" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9865" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B9865" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="A9865" s="3"/>
+      <c r="B9865" s="2"/>
       <c r="C9865" s="2" t="s">
-        <v>69</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9866" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9866" s="3">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B9866" s="7"/>
+      <c r="A9866" s="3"/>
+      <c r="B9866" s="2"/>
       <c r="C9866" s="2" t="s">
-        <v>420</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9867" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9867" s="3"/>
       <c r="B9867" s="7"/>
       <c r="C9867" s="2" t="s">
-        <v>421</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9868" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9868" s="3"/>
-      <c r="B9868" s="7"/>
+      <c r="A9868" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B9868" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C9868" s="2" t="s">
-        <v>303</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9869" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9869" s="3"/>
-      <c r="B9869" s="7"/>
-      <c r="C9869" s="2" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="9870" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9870" s="3"/>
-      <c r="B9870" s="7"/>
-      <c r="C9870" s="2" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="9871" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9871" s="3"/>
-      <c r="B9871" s="7"/>
-      <c r="C9871" s="2" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="9872" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9872" s="3"/>
-      <c r="B9872" s="7"/>
-      <c r="C9872" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="9873" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9873" s="3"/>
-      <c r="B9873" s="7"/>
-      <c r="C9873" s="2" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="9874" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9874" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B9874" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9874" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9875" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9875" s="3">
-        <v>6.1</v>
-      </c>
-      <c r="B9875" s="2"/>
-      <c r="C9875" s="2"/>
-    </row>
-    <row r="9876" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9876" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="B9876" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9876" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9877" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9877" s="16" t="s">
+      <c r="A9869" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9877" s="9"/>
-      <c r="C9877" s="8"/>
+      <c r="B9869" s="9"/>
+      <c r="C9869" s="8"/>
     </row>
     <row r="9913" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9913" s="10" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="B9913" s="11" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C9913" s="12" t="s">
         <v>16</v>
@@ -33864,10 +33857,10 @@
     </row>
     <row r="9914" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9914" s="13"/>
-      <c r="B9914" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9914" s="18"/>
+      <c r="B9914" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9914" s="23"/>
     </row>
     <row r="9915" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9915" s="5" t="s">
@@ -33908,7 +33901,7 @@
         <v>47</v>
       </c>
       <c r="C9918" s="2" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9919" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -33917,7 +33910,7 @@
       </c>
       <c r="B9919" s="7"/>
       <c r="C9919" s="2" t="s">
-        <v>25</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9920" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -33925,10 +33918,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B9920" s="7" t="s">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="C9920" s="2" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9921" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -33936,16 +33929,14 @@
         <v>3.1</v>
       </c>
       <c r="B9921" s="7"/>
-      <c r="C9921" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="C9921" s="2"/>
     </row>
     <row r="9922" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9922" s="3">
         <v>3.2</v>
       </c>
       <c r="B9922" s="7" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="C9922" s="2" t="s">
         <v>6</v>
@@ -33957,51 +33948,131 @@
       </c>
       <c r="B9923" s="7"/>
       <c r="C9923" s="2" t="s">
-        <v>73</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9924" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9924" s="3"/>
-      <c r="B9924" s="7"/>
+      <c r="A9924" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B9924" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="C9924" s="2" t="s">
-        <v>425</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9925" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9925" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B9925" s="7" t="s">
-        <v>47</v>
-      </c>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B9925" s="7"/>
       <c r="C9925" s="2" t="s">
-        <v>5</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9926" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9926" s="16" t="s">
+      <c r="A9926" s="3"/>
+      <c r="B9926" s="7"/>
+      <c r="C9926" s="2" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="9927" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9927" s="3"/>
+      <c r="B9927" s="7"/>
+      <c r="C9927" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="9928" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9928" s="3"/>
+      <c r="B9928" s="7"/>
+      <c r="C9928" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="9929" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9929" s="3"/>
+      <c r="B9929" s="7"/>
+      <c r="C9929" s="2" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="9930" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9930" s="3"/>
+      <c r="B9930" s="7"/>
+      <c r="C9930" s="2" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9931" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9931" s="3"/>
+      <c r="B9931" s="7"/>
+      <c r="C9931" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="9932" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9932" s="3"/>
+      <c r="B9932" s="7"/>
+      <c r="C9932" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="9933" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9933" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B9933" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9933" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9934" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9934" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B9934" s="2"/>
+      <c r="C9934" s="2"/>
+    </row>
+    <row r="9935" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9935" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B9935" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9935" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9936" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9936" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9926" s="9"/>
-      <c r="C9926" s="8"/>
+      <c r="B9936" s="9"/>
+      <c r="C9936" s="8"/>
     </row>
     <row r="9972" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9972" s="10" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B9972" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C9972" s="12" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9973" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9973" s="13"/>
-      <c r="B9973" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="C9973" s="23"/>
+      <c r="B9973" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9973" s="18"/>
     </row>
     <row r="9974" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9974" s="5" t="s">
@@ -34042,7 +34113,7 @@
         <v>47</v>
       </c>
       <c r="C9977" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9978" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34051,7 +34122,7 @@
       </c>
       <c r="B9978" s="7"/>
       <c r="C9978" s="2" t="s">
-        <v>409</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9979" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34059,10 +34130,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B9979" s="7" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="C9979" s="2" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9980" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34071,7 +34142,7 @@
       </c>
       <c r="B9980" s="7"/>
       <c r="C9980" s="2" t="s">
-        <v>427</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9981" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34079,10 +34150,10 @@
         <v>3.2</v>
       </c>
       <c r="B9981" s="7" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="C9981" s="2" t="s">
-        <v>55</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9982" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34090,41 +34161,50 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B9982" s="7"/>
-      <c r="C9982" s="2"/>
+      <c r="C9982" s="2" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="9983" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9983" s="3">
+      <c r="A9983" s="3"/>
+      <c r="B9983" s="7"/>
+      <c r="C9983" s="2" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="9984" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9984" s="3">
         <v>4.2</v>
       </c>
-      <c r="B9983" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9983" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9984" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9984" s="16" t="s">
+      <c r="B9984" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9984" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9985" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9985" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9984" s="9"/>
-      <c r="C9984" s="8"/>
+      <c r="B9985" s="9"/>
+      <c r="C9985" s="8"/>
     </row>
     <row r="10031" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10031" s="10" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B10031" s="11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C10031" s="12" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10032" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10032" s="13"/>
       <c r="B10032" s="22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C10032" s="23"/>
     </row>
@@ -34167,7 +34247,7 @@
         <v>47</v>
       </c>
       <c r="C10036" s="2" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10037" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34176,7 +34256,7 @@
       </c>
       <c r="B10037" s="7"/>
       <c r="C10037" s="2" t="s">
-        <v>25</v>
+        <v>409</v>
       </c>
     </row>
     <row r="10038" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34184,10 +34264,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B10038" s="7" t="s">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="C10038" s="2" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10039" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34196,7 +34276,7 @@
       </c>
       <c r="B10039" s="7"/>
       <c r="C10039" s="2" t="s">
-        <v>25</v>
+        <v>427</v>
       </c>
     </row>
     <row r="10040" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34204,10 +34284,10 @@
         <v>3.2</v>
       </c>
       <c r="B10040" s="7" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="C10040" s="2" t="s">
-        <v>6</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10041" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34215,63 +34295,43 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B10041" s="7"/>
-      <c r="C10041" s="2" t="s">
-        <v>427</v>
-      </c>
+      <c r="C10041" s="2"/>
     </row>
     <row r="10042" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10042" s="3">
         <v>4.2</v>
       </c>
       <c r="B10042" s="7" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C10042" s="2" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10043" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10043" s="3">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B10043" s="7"/>
-      <c r="C10043" s="2"/>
-    </row>
-    <row r="10044" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10044" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B10044" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10044" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10045" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10045" s="16" t="s">
+      <c r="A10043" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10045" s="9"/>
-      <c r="C10045" s="8"/>
+      <c r="B10043" s="9"/>
+      <c r="C10043" s="8"/>
     </row>
     <row r="10090" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10090" s="10" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B10090" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10090" s="12" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10091" s="13"/>
-      <c r="B10091" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10091" s="18"/>
+      <c r="B10091" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10091" s="23"/>
     </row>
     <row r="10092" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10092" s="5" t="s">
@@ -34312,7 +34372,7 @@
         <v>47</v>
       </c>
       <c r="C10095" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10096" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34321,7 +34381,7 @@
       </c>
       <c r="B10096" s="7"/>
       <c r="C10096" s="2" t="s">
-        <v>430</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10097" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34332,31 +34392,89 @@
         <v>47</v>
       </c>
       <c r="C10097" s="2" t="s">
-        <v>5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10098" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10098" s="16" t="s">
+      <c r="A10098" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B10098" s="7"/>
+      <c r="C10098" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10099" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10099" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B10099" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10099" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10100" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10100" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10100" s="7"/>
+      <c r="C10100" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="10101" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10101" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B10101" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10101" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10102" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10102" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10102" s="7"/>
+      <c r="C10102" s="2"/>
+    </row>
+    <row r="10103" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10103" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B10103" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10103" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10104" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10104" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10098" s="9"/>
-      <c r="C10098" s="8"/>
+      <c r="B10104" s="9"/>
+      <c r="C10104" s="8"/>
     </row>
     <row r="10149" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10149" s="10" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B10149" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10149" s="12" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10150" s="13"/>
       <c r="B10150" s="17" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="C10150" s="18"/>
     </row>
@@ -34399,7 +34517,7 @@
         <v>47</v>
       </c>
       <c r="C10154" s="2" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10155" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34407,63 +34525,31 @@
         <v>2.1</v>
       </c>
       <c r="B10155" s="7"/>
-      <c r="C10155" s="2"/>
+      <c r="C10155" s="2" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="10156" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10156" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10156" s="7"/>
-      <c r="C10156" s="2"/>
+      <c r="B10156" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10156" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="10157" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10157" s="3">
-        <v>3.1</v>
-      </c>
-      <c r="B10157" s="7"/>
-      <c r="C10157" s="2" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="10158" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10158" s="3">
-        <v>3.2</v>
-      </c>
-      <c r="B10158" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="C10158" s="2" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="10159" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10159" s="3">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="B10159" s="7"/>
-      <c r="C10159" s="2"/>
-    </row>
-    <row r="10160" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10160" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B10160" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10160" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10161" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10161" s="16" t="s">
+      <c r="A10157" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10161" s="9"/>
-      <c r="C10161" s="8"/>
+      <c r="B10157" s="9"/>
+      <c r="C10157" s="8"/>
     </row>
     <row r="10208" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10208" s="25" t="s">
-        <v>433</v>
+      <c r="A10208" s="10" t="s">
+        <v>431</v>
       </c>
       <c r="B10208" s="11" t="s">
         <v>13</v>
@@ -34474,10 +34560,10 @@
     </row>
     <row r="10209" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10209" s="13"/>
-      <c r="B10209" s="22" t="s">
-        <v>434</v>
-      </c>
-      <c r="C10209" s="23"/>
+      <c r="B10209" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10209" s="18"/>
     </row>
     <row r="10210" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10210" s="5" t="s">
@@ -34526,9 +34612,7 @@
         <v>2.1</v>
       </c>
       <c r="B10214" s="7"/>
-      <c r="C10214" s="2" t="s">
-        <v>436</v>
-      </c>
+      <c r="C10214" s="2"/>
     </row>
     <row r="10215" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10215" s="3">
@@ -34542,17 +34626,19 @@
         <v>3.1</v>
       </c>
       <c r="B10216" s="7"/>
-      <c r="C10216" s="2"/>
+      <c r="C10216" s="2" t="s">
+        <v>281</v>
+      </c>
     </row>
     <row r="10217" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10217" s="3">
         <v>3.2</v>
       </c>
       <c r="B10217" s="7" t="s">
-        <v>23</v>
+        <v>284</v>
       </c>
       <c r="C10217" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
     </row>
     <row r="10218" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34560,9 +34646,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B10218" s="7"/>
-      <c r="C10218" s="2" t="s">
-        <v>435</v>
-      </c>
+      <c r="C10218" s="2"/>
     </row>
     <row r="10219" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10219" s="3">
@@ -34583,22 +34667,22 @@
       <c r="C10220" s="8"/>
     </row>
     <row r="10267" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10267" s="10" t="s">
-        <v>438</v>
+      <c r="A10267" s="25" t="s">
+        <v>433</v>
       </c>
       <c r="B10267" s="11" t="s">
-        <v>101</v>
+        <v>13</v>
       </c>
       <c r="C10267" s="12" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10268" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10268" s="13"/>
-      <c r="B10268" s="17" t="s">
-        <v>172</v>
-      </c>
-      <c r="C10268" s="18"/>
+      <c r="B10268" s="22" t="s">
+        <v>434</v>
+      </c>
+      <c r="C10268" s="23"/>
     </row>
     <row r="10269" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10269" s="5" t="s">
@@ -34628,7 +34712,7 @@
       </c>
       <c r="B10271" s="7"/>
       <c r="C10271" s="2" t="s">
-        <v>439</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10272" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34639,7 +34723,7 @@
         <v>47</v>
       </c>
       <c r="C10272" s="2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10273" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34648,7 +34732,7 @@
       </c>
       <c r="B10273" s="7"/>
       <c r="C10273" s="2" t="s">
-        <v>93</v>
+        <v>436</v>
       </c>
     </row>
     <row r="10274" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34663,66 +34747,61 @@
         <v>3.1</v>
       </c>
       <c r="B10275" s="7"/>
-      <c r="C10275" s="2" t="s">
-        <v>145</v>
-      </c>
+      <c r="C10275" s="2"/>
     </row>
     <row r="10276" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10276" s="3"/>
-      <c r="B10276" s="7"/>
+      <c r="A10276" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B10276" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="C10276" s="2" t="s">
-        <v>58</v>
+        <v>437</v>
       </c>
     </row>
     <row r="10277" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10277" s="3">
-        <v>3.2</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="B10277" s="7"/>
-      <c r="C10277" s="2"/>
+      <c r="C10277" s="2" t="s">
+        <v>435</v>
+      </c>
     </row>
     <row r="10278" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10278" s="3">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="B10278" s="7"/>
+        <v>4.2</v>
+      </c>
+      <c r="B10278" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C10278" s="2" t="s">
-        <v>59</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10279" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10279" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B10279" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10279" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10280" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10280" s="16" t="s">
+      <c r="A10279" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10280" s="9"/>
-      <c r="C10280" s="8"/>
+      <c r="B10279" s="9"/>
+      <c r="C10279" s="8"/>
     </row>
     <row r="10326" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10326" s="10" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B10326" s="11" t="s">
-        <v>9</v>
+        <v>101</v>
       </c>
       <c r="C10326" s="12" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10327" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10327" s="13"/>
       <c r="B10327" s="17" t="s">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="C10327" s="18"/>
     </row>
@@ -34754,7 +34833,7 @@
       </c>
       <c r="B10330" s="7"/>
       <c r="C10330" s="2" t="s">
-        <v>25</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10331" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34773,7 +34852,9 @@
         <v>2.1</v>
       </c>
       <c r="B10332" s="7"/>
-      <c r="C10332" s="2"/>
+      <c r="C10332" s="2" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="10333" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10333" s="3">
@@ -34787,131 +34868,68 @@
         <v>3.1</v>
       </c>
       <c r="B10334" s="7"/>
-      <c r="C10334" s="2"/>
+      <c r="C10334" s="2" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="10335" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10335" s="3">
-        <v>3.2</v>
-      </c>
-      <c r="B10335" s="7" t="s">
-        <v>82</v>
-      </c>
+      <c r="A10335" s="3"/>
+      <c r="B10335" s="7"/>
       <c r="C10335" s="2" t="s">
-        <v>18</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10336" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10336" s="3">
-        <v>4.0999999999999996</v>
+        <v>3.2</v>
       </c>
       <c r="B10336" s="7"/>
       <c r="C10336" s="2"/>
     </row>
     <row r="10337" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10337" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B10337" s="7" t="s">
-        <v>83</v>
-      </c>
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10337" s="7"/>
       <c r="C10337" s="2" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10338" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10338" s="3">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B10338" s="7"/>
+        <v>4.2</v>
+      </c>
+      <c r="B10338" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C10338" s="2" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10339" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10339" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B10339" s="7"/>
-      <c r="C10339" s="2"/>
-    </row>
-    <row r="10340" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10340" s="3">
-        <v>6.1</v>
-      </c>
-      <c r="B10340" s="7"/>
-      <c r="C10340" s="2"/>
-    </row>
-    <row r="10341" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10341" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="B10341" s="7" t="s">
-        <v>441</v>
-      </c>
-      <c r="C10341" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10342" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10342" s="3">
-        <v>7.1</v>
-      </c>
-      <c r="B10342" s="7"/>
-      <c r="C10342" s="2"/>
-    </row>
-    <row r="10343" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10343" s="3">
-        <v>7.2</v>
-      </c>
-      <c r="B10343" s="7" t="s">
-        <v>442</v>
-      </c>
-      <c r="C10343" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10344" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10344" s="3">
-        <v>8.1</v>
-      </c>
-      <c r="B10344" s="7"/>
-      <c r="C10344" s="2"/>
-    </row>
-    <row r="10345" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10345" s="3">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="B10345" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10345" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10346" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10346" s="16" t="s">
+      <c r="A10339" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10346" s="9"/>
-      <c r="C10346" s="8"/>
+      <c r="B10339" s="9"/>
+      <c r="C10339" s="8"/>
     </row>
     <row r="10385" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10385" s="10" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="B10385" s="11" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C10385" s="12" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10386" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10386" s="13"/>
-      <c r="B10386" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="C10386" s="23"/>
+      <c r="B10386" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10386" s="18"/>
     </row>
     <row r="10387" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10387" s="5" t="s">
@@ -34960,39 +34978,31 @@
         <v>2.1</v>
       </c>
       <c r="B10391" s="7"/>
-      <c r="C10391" s="2" t="s">
-        <v>409</v>
-      </c>
+      <c r="C10391" s="2"/>
     </row>
     <row r="10392" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10392" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10392" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10392" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="B10392" s="7"/>
+      <c r="C10392" s="2"/>
     </row>
     <row r="10393" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10393" s="3">
         <v>3.1</v>
       </c>
       <c r="B10393" s="7"/>
-      <c r="C10393" s="2" t="s">
-        <v>444</v>
-      </c>
+      <c r="C10393" s="2"/>
     </row>
     <row r="10394" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10394" s="3">
         <v>3.2</v>
       </c>
       <c r="B10394" s="7" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="C10394" s="2" t="s">
-        <v>55</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10395" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -35007,36 +35017,106 @@
         <v>4.2</v>
       </c>
       <c r="B10396" s="7" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="C10396" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10397" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10397" s="16" t="s">
+      <c r="A10397" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10397" s="7"/>
+      <c r="C10397" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10398" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10398" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B10398" s="7"/>
+      <c r="C10398" s="2"/>
+    </row>
+    <row r="10399" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10399" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B10399" s="7"/>
+      <c r="C10399" s="2"/>
+    </row>
+    <row r="10400" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10400" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B10400" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="C10400" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10401" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10401" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B10401" s="7"/>
+      <c r="C10401" s="2"/>
+    </row>
+    <row r="10402" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10402" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B10402" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="C10402" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10403" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10403" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="B10403" s="7"/>
+      <c r="C10403" s="2"/>
+    </row>
+    <row r="10404" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10404" s="3">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B10404" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10404" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10405" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10405" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10397" s="9"/>
-      <c r="C10397" s="8"/>
+      <c r="B10405" s="9"/>
+      <c r="C10405" s="8"/>
     </row>
     <row r="10444" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10444" s="10" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B10444" s="11" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="C10444" s="12" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10445" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10445" s="13"/>
-      <c r="B10445" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10445" s="18"/>
+      <c r="B10445" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10445" s="23"/>
     </row>
     <row r="10446" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10446" s="5" t="s">
@@ -35106,15 +35186,19 @@
       </c>
       <c r="B10452" s="7"/>
       <c r="C10452" s="2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="10453" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10453" s="3">
         <v>3.2</v>
       </c>
-      <c r="B10453" s="7"/>
-      <c r="C10453" s="2"/>
+      <c r="B10453" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10453" s="2" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="10454" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10454" s="3">
@@ -35131,92 +35215,33 @@
         <v>47</v>
       </c>
       <c r="C10455" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10456" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10456" s="3">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B10456" s="7"/>
-      <c r="C10456" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10457" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10457" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B10457" s="7"/>
-      <c r="C10457" s="2"/>
-    </row>
-    <row r="10458" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10458" s="3">
-        <v>6.1</v>
-      </c>
-      <c r="B10458" s="7"/>
-      <c r="C10458" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="10459" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10459" s="3"/>
-      <c r="B10459" s="7"/>
-      <c r="C10459" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10460" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10460" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="B10460" s="7"/>
-      <c r="C10460" s="2"/>
-    </row>
-    <row r="10461" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10461" s="3">
-        <v>7.1</v>
-      </c>
-      <c r="B10461" s="7"/>
-      <c r="C10461" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10462" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10462" s="3">
-        <v>7.2</v>
-      </c>
-      <c r="B10462" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10462" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10463" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10463" s="16" t="s">
+      <c r="A10456" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10463" s="9"/>
-      <c r="C10463" s="8"/>
+      <c r="B10456" s="9"/>
+      <c r="C10456" s="8"/>
     </row>
     <row r="10503" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10503" s="10" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="B10503" s="11" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="C10503" s="12" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10504" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10504" s="13"/>
-      <c r="B10504" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="C10504" s="23"/>
+      <c r="B10504" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10504" s="18"/>
     </row>
     <row r="10505" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10505" s="5" t="s">
@@ -35266,15 +35291,19 @@
       </c>
       <c r="B10509" s="7"/>
       <c r="C10509" s="2" t="s">
-        <v>25</v>
+        <v>409</v>
       </c>
     </row>
     <row r="10510" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10510" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10510" s="7"/>
-      <c r="C10510" s="2"/>
+      <c r="B10510" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10510" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="10511" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10511" s="3">
@@ -35282,81 +35311,85 @@
       </c>
       <c r="B10511" s="7"/>
       <c r="C10511" s="2" t="s">
-        <v>411</v>
+        <v>446</v>
       </c>
     </row>
     <row r="10512" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10512" s="3">
         <v>3.2</v>
       </c>
-      <c r="B10512" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10512" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="B10512" s="7"/>
+      <c r="C10512" s="2"/>
     </row>
     <row r="10513" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10513" s="3">
         <v>4.0999999999999996</v>
       </c>
       <c r="B10513" s="7"/>
-      <c r="C10513" s="2" t="s">
-        <v>403</v>
-      </c>
+      <c r="C10513" s="2"/>
     </row>
     <row r="10514" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10514" s="3"/>
-      <c r="B10514" s="7"/>
+      <c r="A10514" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B10514" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C10514" s="2" t="s">
-        <v>404</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10515" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10515" s="3"/>
+      <c r="A10515" s="3">
+        <v>5.0999999999999996</v>
+      </c>
       <c r="B10515" s="7"/>
       <c r="C10515" s="2" t="s">
-        <v>303</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10516" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10516" s="3"/>
+      <c r="A10516" s="3">
+        <v>5.2</v>
+      </c>
       <c r="B10516" s="7"/>
-      <c r="C10516" s="2" t="s">
-        <v>334</v>
-      </c>
+      <c r="C10516" s="2"/>
     </row>
     <row r="10517" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10517" s="3"/>
+      <c r="A10517" s="3">
+        <v>6.1</v>
+      </c>
       <c r="B10517" s="7"/>
       <c r="C10517" s="2" t="s">
-        <v>405</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10518" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10518" s="3"/>
       <c r="B10518" s="7"/>
       <c r="C10518" s="2" t="s">
-        <v>406</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10519" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10519" s="3"/>
+      <c r="A10519" s="3">
+        <v>6.2</v>
+      </c>
       <c r="B10519" s="7"/>
-      <c r="C10519" s="2" t="s">
-        <v>308</v>
-      </c>
+      <c r="C10519" s="2"/>
     </row>
     <row r="10520" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10520" s="3"/>
+      <c r="A10520" s="3">
+        <v>7.1</v>
+      </c>
       <c r="B10520" s="7"/>
       <c r="C10520" s="2" t="s">
-        <v>304</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10521" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10521" s="3">
-        <v>4.2</v>
+        <v>7.2</v>
       </c>
       <c r="B10521" s="7" t="s">
         <v>47</v>
@@ -35374,19 +35407,19 @@
     </row>
     <row r="10562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10562" s="10" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B10562" s="11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C10562" s="12" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10563" s="13"/>
       <c r="B10563" s="22" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C10563" s="23"/>
     </row>
@@ -35429,7 +35462,7 @@
         <v>47</v>
       </c>
       <c r="C10567" s="2" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -35445,12 +35478,8 @@
       <c r="A10569" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10569" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10569" s="2" t="s">
-        <v>41</v>
-      </c>
+      <c r="B10569" s="7"/>
+      <c r="C10569" s="2"/>
     </row>
     <row r="10570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10570" s="3">
@@ -35458,15 +35487,19 @@
       </c>
       <c r="B10570" s="7"/>
       <c r="C10570" s="2" t="s">
-        <v>25</v>
+        <v>411</v>
       </c>
     </row>
     <row r="10571" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10571" s="3">
         <v>3.2</v>
       </c>
-      <c r="B10571" s="7"/>
-      <c r="C10571" s="2"/>
+      <c r="B10571" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10571" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="10572" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10572" s="3">
@@ -35474,99 +35507,79 @@
       </c>
       <c r="B10572" s="7"/>
       <c r="C10572" s="2" t="s">
-        <v>104</v>
+        <v>403</v>
       </c>
     </row>
     <row r="10573" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10573" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B10573" s="7" t="s">
-        <v>42</v>
-      </c>
+      <c r="A10573" s="3"/>
+      <c r="B10573" s="7"/>
       <c r="C10573" s="2" t="s">
-        <v>6</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10574" s="3">
-        <v>5.0999999999999996</v>
-      </c>
+      <c r="A10574" s="3"/>
       <c r="B10574" s="7"/>
       <c r="C10574" s="2" t="s">
-        <v>403</v>
+        <v>303</v>
       </c>
     </row>
     <row r="10575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10575" s="3"/>
       <c r="B10575" s="7"/>
       <c r="C10575" s="2" t="s">
-        <v>404</v>
+        <v>334</v>
       </c>
     </row>
     <row r="10576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10576" s="3"/>
       <c r="B10576" s="7"/>
       <c r="C10576" s="2" t="s">
-        <v>303</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10577" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10577" s="3"/>
       <c r="B10577" s="7"/>
       <c r="C10577" s="2" t="s">
-        <v>334</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10578" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10578" s="3"/>
       <c r="B10578" s="7"/>
       <c r="C10578" s="2" t="s">
-        <v>405</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10579" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10579" s="3"/>
       <c r="B10579" s="7"/>
       <c r="C10579" s="2" t="s">
-        <v>406</v>
+        <v>304</v>
       </c>
     </row>
     <row r="10580" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10580" s="3"/>
-      <c r="B10580" s="7"/>
+      <c r="A10580" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B10580" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C10580" s="2" t="s">
-        <v>308</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10581" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10581" s="3"/>
-      <c r="B10581" s="7"/>
-      <c r="C10581" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="10582" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10582" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B10582" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10582" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10583" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10583" s="16" t="s">
+      <c r="A10581" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10583" s="9"/>
-      <c r="C10583" s="8"/>
+      <c r="B10581" s="9"/>
+      <c r="C10581" s="8"/>
     </row>
     <row r="10621" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10621" s="10" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B10621" s="11" t="s">
         <v>11</v>
@@ -35578,7 +35591,7 @@
     <row r="10622" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10622" s="13"/>
       <c r="B10622" s="22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C10622" s="23"/>
     </row>
@@ -35666,7 +35679,7 @@
       </c>
       <c r="B10631" s="7"/>
       <c r="C10631" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10632" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -35758,19 +35771,19 @@
     </row>
     <row r="10680" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10680" s="10" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B10680" s="11" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C10680" s="12" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10681" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10681" s="13"/>
       <c r="B10681" s="22" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="C10681" s="23"/>
     </row>
@@ -35813,7 +35826,7 @@
         <v>47</v>
       </c>
       <c r="C10685" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10686" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -35829,8 +35842,12 @@
       <c r="A10687" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10687" s="7"/>
-      <c r="C10687" s="2"/>
+      <c r="B10687" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10687" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="10688" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10688" s="3">
@@ -35838,154 +35855,127 @@
       </c>
       <c r="B10688" s="7"/>
       <c r="C10688" s="2" t="s">
-        <v>413</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10689" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10689" s="3">
         <v>3.2</v>
       </c>
-      <c r="B10689" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10689" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="B10689" s="7"/>
+      <c r="C10689" s="2"/>
     </row>
     <row r="10690" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10690" s="3">
         <v>4.0999999999999996</v>
       </c>
       <c r="B10690" s="7"/>
-      <c r="C10690" s="2"/>
+      <c r="C10690" s="2" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="10691" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10691" s="3">
         <v>4.2</v>
       </c>
-      <c r="B10691" s="24" t="s">
-        <v>412</v>
+      <c r="B10691" s="7" t="s">
+        <v>42</v>
       </c>
       <c r="C10691" s="2" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10692" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10692" s="3"/>
-      <c r="B10692" s="24"/>
-      <c r="C10692" s="2"/>
+      <c r="A10692" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10692" s="7"/>
+      <c r="C10692" s="2" t="s">
+        <v>403</v>
+      </c>
     </row>
     <row r="10693" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10693" s="3">
-        <v>5.0999999999999996</v>
-      </c>
+      <c r="A10693" s="3"/>
       <c r="B10693" s="7"/>
       <c r="C10693" s="2" t="s">
-        <v>109</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10694" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10694" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B10694" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="A10694" s="3"/>
+      <c r="B10694" s="7"/>
       <c r="C10694" s="2" t="s">
-        <v>6</v>
+        <v>303</v>
       </c>
     </row>
     <row r="10695" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10695" s="3">
-        <v>6.1</v>
-      </c>
+      <c r="A10695" s="3"/>
       <c r="B10695" s="7"/>
       <c r="C10695" s="2" t="s">
-        <v>403</v>
+        <v>334</v>
       </c>
     </row>
     <row r="10696" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10696" s="3"/>
       <c r="B10696" s="7"/>
       <c r="C10696" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10697" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10697" s="3"/>
       <c r="B10697" s="7"/>
       <c r="C10697" s="2" t="s">
-        <v>303</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10698" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10698" s="3"/>
       <c r="B10698" s="7"/>
       <c r="C10698" s="2" t="s">
-        <v>334</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10699" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10699" s="3"/>
       <c r="B10699" s="7"/>
       <c r="C10699" s="2" t="s">
-        <v>405</v>
+        <v>304</v>
       </c>
     </row>
     <row r="10700" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10700" s="3"/>
-      <c r="B10700" s="7"/>
+      <c r="A10700" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B10700" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C10700" s="2" t="s">
-        <v>406</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10701" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10701" s="3"/>
-      <c r="B10701" s="7"/>
-      <c r="C10701" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="10702" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10702" s="3"/>
-      <c r="B10702" s="7"/>
-      <c r="C10702" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="10703" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10703" s="3">
-        <v>6.2</v>
-      </c>
-      <c r="B10703" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10703" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10704" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10704" s="16" t="s">
+      <c r="A10701" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10704" s="9"/>
-      <c r="C10704" s="8"/>
+      <c r="B10701" s="9"/>
+      <c r="C10701" s="8"/>
     </row>
     <row r="10739" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10739" s="10" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B10739" s="11" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C10739" s="12" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10740" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10740" s="13"/>
       <c r="B10740" s="22" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="C10740" s="23"/>
     </row>
@@ -36028,7 +36018,7 @@
         <v>47</v>
       </c>
       <c r="C10744" s="2" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10745" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36044,12 +36034,8 @@
       <c r="A10746" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10746" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10746" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="B10746" s="7"/>
+      <c r="C10746" s="2"/>
     </row>
     <row r="10747" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10747" s="3">
@@ -36057,7 +36043,7 @@
       </c>
       <c r="B10747" s="7"/>
       <c r="C10747" s="2" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="10748" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36068,7 +36054,7 @@
         <v>7</v>
       </c>
       <c r="C10748" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10749" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36076,110 +36062,135 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B10749" s="7"/>
-      <c r="C10749" s="2" t="s">
-        <v>420</v>
-      </c>
+      <c r="C10749" s="2"/>
     </row>
     <row r="10750" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10750" s="3"/>
-      <c r="B10750" s="2"/>
+      <c r="A10750" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B10750" s="24" t="s">
+        <v>412</v>
+      </c>
       <c r="C10750" s="2" t="s">
-        <v>421</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10751" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10751" s="3"/>
-      <c r="B10751" s="2"/>
-      <c r="C10751" s="2" t="s">
-        <v>303</v>
-      </c>
+      <c r="B10751" s="24"/>
+      <c r="C10751" s="2"/>
     </row>
     <row r="10752" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10752" s="3"/>
+      <c r="A10752" s="3">
+        <v>5.0999999999999996</v>
+      </c>
       <c r="B10752" s="7"/>
       <c r="C10752" s="2" t="s">
-        <v>334</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10753" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10753" s="3"/>
-      <c r="B10753" s="7"/>
+      <c r="A10753" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B10753" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="C10753" s="2" t="s">
-        <v>422</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10754" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10754" s="3"/>
+      <c r="A10754" s="3">
+        <v>6.1</v>
+      </c>
       <c r="B10754" s="7"/>
       <c r="C10754" s="2" t="s">
-        <v>423</v>
+        <v>403</v>
       </c>
     </row>
     <row r="10755" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10755" s="3"/>
       <c r="B10755" s="7"/>
       <c r="C10755" s="2" t="s">
-        <v>308</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10756" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10756" s="3"/>
       <c r="B10756" s="7"/>
       <c r="C10756" s="2" t="s">
-        <v>340</v>
+        <v>303</v>
       </c>
     </row>
     <row r="10757" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10757" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B10757" s="7" t="s">
-        <v>23</v>
-      </c>
+      <c r="A10757" s="3"/>
+      <c r="B10757" s="7"/>
       <c r="C10757" s="2" t="s">
-        <v>70</v>
+        <v>334</v>
       </c>
     </row>
     <row r="10758" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10758" s="3">
-        <v>5.0999999999999996</v>
-      </c>
+      <c r="A10758" s="3"/>
       <c r="B10758" s="7"/>
-      <c r="C10758" s="2"/>
+      <c r="C10758" s="2" t="s">
+        <v>405</v>
+      </c>
     </row>
     <row r="10759" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10759" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B10759" s="7" t="s">
-        <v>47</v>
-      </c>
+      <c r="A10759" s="3"/>
+      <c r="B10759" s="7"/>
       <c r="C10759" s="2" t="s">
-        <v>5</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10760" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10760" s="16" t="s">
+      <c r="A10760" s="3"/>
+      <c r="B10760" s="7"/>
+      <c r="C10760" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="10761" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10761" s="3"/>
+      <c r="B10761" s="7"/>
+      <c r="C10761" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="10762" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10762" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B10762" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10762" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10763" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10763" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10760" s="9"/>
-      <c r="C10760" s="8"/>
+      <c r="B10763" s="9"/>
+      <c r="C10763" s="8"/>
     </row>
     <row r="10798" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10798" s="10" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B10798" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C10798" s="12" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10799" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10799" s="13"/>
       <c r="B10799" s="22" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C10799" s="23"/>
     </row>
@@ -36222,7 +36233,7 @@
         <v>47</v>
       </c>
       <c r="C10803" s="2" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10804" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36230,17 +36241,19 @@
         <v>2.1</v>
       </c>
       <c r="B10804" s="7"/>
-      <c r="C10804" s="2"/>
+      <c r="C10804" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="10805" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10805" s="3">
         <v>2.2000000000000002</v>
       </c>
       <c r="B10805" s="7" t="s">
-        <v>414</v>
+        <v>47</v>
       </c>
       <c r="C10805" s="2" t="s">
-        <v>68</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10806" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36248,14 +36261,16 @@
         <v>3.1</v>
       </c>
       <c r="B10806" s="7"/>
-      <c r="C10806" s="2"/>
+      <c r="C10806" s="2" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="10807" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10807" s="3">
         <v>3.2</v>
       </c>
       <c r="B10807" s="7" t="s">
-        <v>410</v>
+        <v>7</v>
       </c>
       <c r="C10807" s="2" t="s">
         <v>69</v>
@@ -36323,60 +36338,55 @@
       <c r="A10816" s="3">
         <v>4.2</v>
       </c>
-      <c r="B10816" s="24" t="s">
-        <v>415</v>
+      <c r="B10816" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="C10816" s="2" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="10817" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10817" s="3"/>
-      <c r="B10817" s="24"/>
+      <c r="A10817" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10817" s="7"/>
       <c r="C10817" s="2"/>
     </row>
     <row r="10818" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10818" s="3">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B10818" s="7"/>
-      <c r="C10818" s="2"/>
+        <v>5.2</v>
+      </c>
+      <c r="B10818" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10818" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="10819" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10819" s="3">
-        <v>5.2</v>
-      </c>
-      <c r="B10819" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10819" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10820" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10820" s="16" t="s">
+      <c r="A10819" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10820" s="9"/>
-      <c r="C10820" s="8"/>
+      <c r="B10819" s="9"/>
+      <c r="C10819" s="8"/>
     </row>
     <row r="10857" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10857" s="10" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B10857" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C10857" s="12" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10858" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10858" s="13"/>
-      <c r="B10858" s="17" t="s">
-        <v>239</v>
-      </c>
-      <c r="C10858" s="18"/>
+      <c r="B10858" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10858" s="23"/>
     </row>
     <row r="10859" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10859" s="5" t="s">
@@ -36417,7 +36427,7 @@
         <v>47</v>
       </c>
       <c r="C10862" s="2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10863" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36425,19 +36435,17 @@
         <v>2.1</v>
       </c>
       <c r="B10863" s="7"/>
-      <c r="C10863" s="2" t="s">
-        <v>409</v>
-      </c>
+      <c r="C10863" s="2"/>
     </row>
     <row r="10864" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10864" s="3">
         <v>2.2000000000000002</v>
       </c>
       <c r="B10864" s="7" t="s">
-        <v>7</v>
+        <v>414</v>
       </c>
       <c r="C10864" s="2" t="s">
-        <v>455</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10865" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36451,62 +36459,115 @@
       <c r="A10866" s="3">
         <v>3.2</v>
       </c>
-      <c r="B10866" s="7"/>
-      <c r="C10866" s="2"/>
+      <c r="B10866" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="C10866" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="10867" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10867" s="3">
         <v>4.0999999999999996</v>
       </c>
       <c r="B10867" s="7"/>
-      <c r="C10867" s="2"/>
+      <c r="C10867" s="2" t="s">
+        <v>420</v>
+      </c>
     </row>
     <row r="10868" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10868" s="3">
-        <v>4.2</v>
-      </c>
-      <c r="B10868" s="24" t="s">
-        <v>412</v>
-      </c>
+      <c r="A10868" s="3"/>
+      <c r="B10868" s="2"/>
       <c r="C10868" s="2" t="s">
-        <v>454</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10869" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10869" s="3"/>
-      <c r="B10869" s="24"/>
-      <c r="C10869" s="2"/>
+      <c r="B10869" s="2"/>
+      <c r="C10869" s="2" t="s">
+        <v>303</v>
+      </c>
     </row>
     <row r="10870" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10870" s="3">
+      <c r="A10870" s="3"/>
+      <c r="B10870" s="7"/>
+      <c r="C10870" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="10871" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10871" s="3"/>
+      <c r="B10871" s="7"/>
+      <c r="C10871" s="2" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="10872" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10872" s="3"/>
+      <c r="B10872" s="7"/>
+      <c r="C10872" s="2" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="10873" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10873" s="3"/>
+      <c r="B10873" s="7"/>
+      <c r="C10873" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="10874" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10874" s="3"/>
+      <c r="B10874" s="7"/>
+      <c r="C10874" s="2" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="10875" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10875" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B10875" s="24" t="s">
+        <v>415</v>
+      </c>
+      <c r="C10875" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10876" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10876" s="3"/>
+      <c r="B10876" s="24"/>
+      <c r="C10876" s="2"/>
+    </row>
+    <row r="10877" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10877" s="3">
         <v>5.0999999999999996</v>
       </c>
-      <c r="B10870" s="2"/>
-      <c r="C10870" s="2" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="10871" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10871" s="3">
+      <c r="B10877" s="7"/>
+      <c r="C10877" s="2"/>
+    </row>
+    <row r="10878" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10878" s="3">
         <v>5.2</v>
       </c>
-      <c r="B10871" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10871" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10872" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10872" s="16" t="s">
+      <c r="B10878" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10878" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10879" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10879" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10872" s="9"/>
-      <c r="C10872" s="8"/>
+      <c r="B10879" s="9"/>
+      <c r="C10879" s="8"/>
     </row>
     <row r="10916" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10916" s="10" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="B10916" s="11" t="s">
         <v>11</v>
@@ -36517,10 +36578,10 @@
     </row>
     <row r="10917" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10917" s="13"/>
-      <c r="B10917" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="C10917" s="23"/>
+      <c r="B10917" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="C10917" s="18"/>
     </row>
     <row r="10918" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10918" s="5" t="s">
@@ -36570,98 +36631,101 @@
       </c>
       <c r="B10922" s="7"/>
       <c r="C10922" s="2" t="s">
-        <v>25</v>
+        <v>409</v>
       </c>
     </row>
     <row r="10923" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10923" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10923" s="7"/>
-      <c r="C10923" s="2"/>
+      <c r="B10923" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10923" s="2" t="s">
+        <v>455</v>
+      </c>
     </row>
     <row r="10924" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10924" s="3">
         <v>3.1</v>
       </c>
       <c r="B10924" s="7"/>
-      <c r="C10924" s="2" t="s">
-        <v>411</v>
-      </c>
+      <c r="C10924" s="2"/>
     </row>
     <row r="10925" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10925" s="3">
         <v>3.2</v>
       </c>
-      <c r="B10925" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10925" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="B10925" s="7"/>
+      <c r="C10925" s="2"/>
     </row>
     <row r="10926" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10926" s="3">
         <v>4.0999999999999996</v>
       </c>
       <c r="B10926" s="7"/>
-      <c r="C10926" s="2" t="s">
-        <v>427</v>
-      </c>
+      <c r="C10926" s="2"/>
     </row>
     <row r="10927" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10927" s="3">
         <v>4.2</v>
       </c>
-      <c r="B10927" s="2" t="s">
-        <v>23</v>
+      <c r="B10927" s="24" t="s">
+        <v>412</v>
       </c>
       <c r="C10927" s="2" t="s">
-        <v>55</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10928" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10928" s="3">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B10928" s="2"/>
+      <c r="A10928" s="3"/>
+      <c r="B10928" s="24"/>
       <c r="C10928" s="2"/>
     </row>
     <row r="10929" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10929" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10929" s="2"/>
+      <c r="C10929" s="2" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="10930" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10930" s="3">
         <v>5.2</v>
       </c>
-      <c r="B10929" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10929" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10930" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10930" s="16" t="s">
+      <c r="B10930" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10930" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10931" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10931" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10930" s="9"/>
-      <c r="C10930" s="8"/>
+      <c r="B10931" s="9"/>
+      <c r="C10931" s="8"/>
     </row>
     <row r="10975" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10975" s="10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B10975" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10975" s="12" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10976" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10976" s="13"/>
-      <c r="B10976" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="C10976" s="18"/>
+      <c r="B10976" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10976" s="23"/>
     </row>
     <row r="10977" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10977" s="5" t="s">
@@ -36702,7 +36766,7 @@
         <v>47</v>
       </c>
       <c r="C10980" s="2" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10981" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36711,30 +36775,84 @@
       </c>
       <c r="B10981" s="7"/>
       <c r="C10981" s="2" t="s">
-        <v>459</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10982" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10982" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B10982" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10982" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="B10982" s="7"/>
+      <c r="C10982" s="2"/>
     </row>
     <row r="10983" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10983" s="16" t="s">
+      <c r="A10983" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B10983" s="7"/>
+      <c r="C10983" s="2" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="10984" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10984" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B10984" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10984" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10985" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10985" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B10985" s="7"/>
+      <c r="C10985" s="2" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="10986" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10986" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B10986" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10986" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10987" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10987" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B10987" s="2"/>
+      <c r="C10987" s="2"/>
+    </row>
+    <row r="10988" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10988" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B10988" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10988" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10989" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10989" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B10983" s="9"/>
-      <c r="C10983" s="8"/>
+      <c r="B10989" s="9"/>
+      <c r="C10989" s="8"/>
     </row>
     <row r="11034" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11034" s="10" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B11034" s="11" t="s">
         <v>12</v>
@@ -36746,7 +36864,7 @@
     <row r="11035" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11035" s="13"/>
       <c r="B11035" s="17" t="s">
-        <v>0</v>
+        <v>136</v>
       </c>
       <c r="C11035" s="18"/>
     </row>
@@ -36785,8 +36903,12 @@
       <c r="A11039" s="3">
         <v>1.2</v>
       </c>
-      <c r="B11039" s="7"/>
-      <c r="C11039" s="2"/>
+      <c r="B11039" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11039" s="2" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="11040" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11040" s="3">
@@ -36794,7 +36916,7 @@
       </c>
       <c r="B11040" s="7"/>
       <c r="C11040" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="11041" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36817,10 +36939,10 @@
     </row>
     <row r="11093" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11093" s="10" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B11093" s="11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C11093" s="12" t="s">
         <v>8</v>
@@ -36877,70 +36999,33 @@
       </c>
       <c r="B11099" s="7"/>
       <c r="C11099" s="2" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
     </row>
     <row r="11100" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11100" s="3"/>
-      <c r="B11100" s="7"/>
+      <c r="A11100" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11100" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C11100" s="2" t="s">
-        <v>463</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11101" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11101" s="3">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="B11101" s="7"/>
-      <c r="C11101" s="2"/>
-    </row>
-    <row r="11102" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11102" s="3">
-        <v>3.1</v>
-      </c>
-      <c r="B11102" s="7"/>
-      <c r="C11102" s="2" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="11103" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11103" s="3"/>
-      <c r="B11103" s="7"/>
-      <c r="C11103" s="2" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="11104" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11104" s="3"/>
-      <c r="B11104" s="7"/>
-      <c r="C11104" s="2" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="11105" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11105" s="3">
-        <v>3.2</v>
-      </c>
-      <c r="B11105" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11105" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11106" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11106" s="16" t="s">
+      <c r="A11101" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B11106" s="9"/>
-      <c r="C11106" s="8"/>
+      <c r="B11101" s="9"/>
+      <c r="C11101" s="8"/>
     </row>
     <row r="11152" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11152" s="10" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="B11152" s="11" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C11152" s="12" t="s">
         <v>8</v>
@@ -36948,10 +37033,10 @@
     </row>
     <row r="11153" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11153" s="13"/>
-      <c r="B11153" s="22" t="s">
-        <v>468</v>
-      </c>
-      <c r="C11153" s="23"/>
+      <c r="B11153" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11153" s="18"/>
     </row>
     <row r="11154" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11154" s="5" t="s">
@@ -36988,12 +37073,8 @@
       <c r="A11157" s="3">
         <v>1.2</v>
       </c>
-      <c r="B11157" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11157" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="B11157" s="7"/>
+      <c r="C11157" s="2"/>
     </row>
     <row r="11158" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11158" s="3">
@@ -37001,83 +37082,921 @@
       </c>
       <c r="B11158" s="7"/>
       <c r="C11158" s="2" t="s">
-        <v>436</v>
+        <v>465</v>
       </c>
     </row>
     <row r="11159" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11159" s="3">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="B11159" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="A11159" s="3"/>
+      <c r="B11159" s="7"/>
       <c r="C11159" s="2" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
     </row>
     <row r="11160" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11160" s="3">
-        <v>3.1</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="B11160" s="7"/>
-      <c r="C11160" s="2" t="s">
-        <v>469</v>
-      </c>
+      <c r="C11160" s="2"/>
     </row>
     <row r="11161" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11161" s="3">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="B11161" s="7"/>
-      <c r="C11161" s="2"/>
+      <c r="C11161" s="2" t="s">
+        <v>466</v>
+      </c>
     </row>
     <row r="11162" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11162" s="3">
-        <v>4.0999999999999996</v>
-      </c>
+      <c r="A11162" s="3"/>
       <c r="B11162" s="7"/>
       <c r="C11162" s="2" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="11163" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11163" s="3"/>
+      <c r="B11163" s="7"/>
+      <c r="C11163" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="11164" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11164" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B11164" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11164" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11165" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11165" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11165" s="9"/>
+      <c r="C11165" s="8"/>
+    </row>
+    <row r="11211" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11211" s="10" t="s">
+        <v>467</v>
+      </c>
+      <c r="B11211" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11211" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11212" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11212" s="13"/>
+      <c r="B11212" s="22" t="s">
+        <v>468</v>
+      </c>
+      <c r="C11212" s="23"/>
+    </row>
+    <row r="11213" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11213" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11213" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11213" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11214" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11214" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11214" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11214" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11215" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11215" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11215" s="7"/>
+      <c r="C11215" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11216" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11216" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B11216" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11216" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11217" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11217" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B11217" s="7"/>
+      <c r="C11217" s="2" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="11218" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11218" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11218" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11218" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="11219" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11219" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B11219" s="7"/>
+      <c r="C11219" s="2" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="11220" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11220" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B11220" s="7"/>
+      <c r="C11220" s="2"/>
+    </row>
+    <row r="11221" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11221" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11221" s="7"/>
+      <c r="C11221" s="2" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="11163" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11163" s="3">
+    <row r="11222" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11222" s="3">
         <v>4.2</v>
       </c>
-      <c r="B11163" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11163" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11164" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11164" s="16" t="s">
+      <c r="B11222" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11222" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11223" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11223" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B11164" s="9"/>
-      <c r="C11164" s="8"/>
+      <c r="B11223" s="9"/>
+      <c r="C11223" s="8"/>
+    </row>
+    <row r="11270" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11270" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="B11270" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11270" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11271" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11271" s="13"/>
+      <c r="B11271" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11271" s="18"/>
+    </row>
+    <row r="11272" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11272" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11272" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11272" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11273" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11273" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11273" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11273" s="20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11274" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11274" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11274" s="7"/>
+      <c r="C11274" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11275" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11275" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B11275" s="7"/>
+      <c r="C11275" s="2"/>
+    </row>
+    <row r="11276" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11276" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B11276" s="7"/>
+      <c r="C11276" s="2"/>
+    </row>
+    <row r="11277" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11277" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11277" s="7"/>
+      <c r="C11277" s="2"/>
+    </row>
+    <row r="11278" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11278" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B11278" s="7"/>
+      <c r="C11278" s="2" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="11279" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11279" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B11279" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11279" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11280" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11280" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11280" s="9"/>
+      <c r="C11280" s="8"/>
+    </row>
+    <row r="11329" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11329" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="B11329" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11329" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11330" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11330" s="13"/>
+      <c r="B11330" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11330" s="18"/>
+    </row>
+    <row r="11331" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11331" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11331" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11331" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11332" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11332" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11332" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11332" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11333" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11333" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11333" s="7"/>
+      <c r="C11333" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11334" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11334" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B11334" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11334" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11335" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11335" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B11335" s="7"/>
+      <c r="C11335" s="2"/>
+    </row>
+    <row r="11336" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11336" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11336" s="7"/>
+      <c r="C11336" s="2"/>
+    </row>
+    <row r="11337" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11337" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B11337" s="7"/>
+      <c r="C11337" s="2"/>
+    </row>
+    <row r="11338" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11338" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B11338" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11338" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11339" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11339" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11339" s="7"/>
+      <c r="C11339" s="2"/>
+    </row>
+    <row r="11340" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11340" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B11340" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11340" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11341" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11341" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B11341" s="7"/>
+      <c r="C11341" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11342" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11342" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B11342" s="7"/>
+      <c r="C11342" s="2"/>
+    </row>
+    <row r="11343" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11343" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B11343" s="7"/>
+      <c r="C11343" s="2"/>
+    </row>
+    <row r="11344" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11344" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B11344" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="C11344" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11345" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11345" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B11345" s="7"/>
+      <c r="C11345" s="2"/>
+    </row>
+    <row r="11346" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11346" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B11346" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="C11346" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11347" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11347" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="B11347" s="7"/>
+      <c r="C11347" s="2"/>
+    </row>
+    <row r="11348" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11348" s="3">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="B11348" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11348" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11349" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11349" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11349" s="9"/>
+      <c r="C11349" s="8"/>
+    </row>
+    <row r="11388" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11388" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="B11388" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11388" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11389" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11389" s="13"/>
+      <c r="B11389" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11389" s="23"/>
+    </row>
+    <row r="11390" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11390" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11390" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11390" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11391" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11391" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11391" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11391" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11392" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11392" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11392" s="7"/>
+      <c r="C11392" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11393" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11393" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B11393" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11393" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11394" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11394" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B11394" s="7"/>
+      <c r="C11394" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="11395" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11395" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11395" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11395" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11396" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11396" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B11396" s="7"/>
+      <c r="C11396" s="2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="11397" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11397" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B11397" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11397" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11398" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11398" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11398" s="7"/>
+      <c r="C11398" s="2"/>
+    </row>
+    <row r="11399" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11399" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B11399" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11399" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11400" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11400" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11400" s="9"/>
+      <c r="C11400" s="8"/>
+    </row>
+    <row r="11447" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11447" s="10" t="s">
+        <v>479</v>
+      </c>
+      <c r="B11447" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11447" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11448" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11448" s="13"/>
+      <c r="B11448" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11448" s="18"/>
+    </row>
+    <row r="11449" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11449" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11449" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11449" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11450" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11450" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11450" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11450" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11451" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11451" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11451" s="7"/>
+      <c r="C11451" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11452" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11452" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B11452" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11452" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11453" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11453" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B11453" s="7"/>
+      <c r="C11453" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="11454" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11454" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11454" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11454" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11455" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11455" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B11455" s="7"/>
+      <c r="C11455" s="2" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="11456" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11456" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B11456" s="7"/>
+      <c r="C11456" s="2"/>
+    </row>
+    <row r="11457" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11457" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11457" s="7"/>
+      <c r="C11457" s="2"/>
+    </row>
+    <row r="11458" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11458" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B11458" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11458" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11459" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11459" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B11459" s="7"/>
+      <c r="C11459" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11460" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11460" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="B11460" s="7"/>
+      <c r="C11460" s="2"/>
+    </row>
+    <row r="11461" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11461" s="3">
+        <v>6.1</v>
+      </c>
+      <c r="B11461" s="7"/>
+      <c r="C11461" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11462" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11462" s="3"/>
+      <c r="B11462" s="7"/>
+      <c r="C11462" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11463" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11463" s="3">
+        <v>6.2</v>
+      </c>
+      <c r="B11463" s="7"/>
+      <c r="C11463" s="2"/>
+    </row>
+    <row r="11464" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11464" s="3">
+        <v>7.1</v>
+      </c>
+      <c r="B11464" s="7"/>
+      <c r="C11464" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11465" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11465" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="B11465" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11465" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11466" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11466" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11466" s="9"/>
+      <c r="C11466" s="8"/>
+    </row>
+    <row r="11506" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11506" s="10" t="s">
+        <v>481</v>
+      </c>
+      <c r="B11506" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11506" s="12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11507" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11507" s="13"/>
+      <c r="B11507" s="17" t="s">
+        <v>482</v>
+      </c>
+      <c r="C11507" s="18"/>
+    </row>
+    <row r="11508" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11508" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11508" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11508" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11509" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11509" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11509" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11509" s="21" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11510" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11510" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B11510" s="7"/>
+      <c r="C11510" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11511" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11511" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="B11511" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11511" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11512" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11512" s="3">
+        <v>2.1</v>
+      </c>
+      <c r="B11512" s="7"/>
+      <c r="C11512" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="11513" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11513" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B11513" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11513" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11514" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11514" s="3">
+        <v>3.1</v>
+      </c>
+      <c r="B11514" s="7"/>
+      <c r="C11514" s="2"/>
+    </row>
+    <row r="11515" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11515" s="3">
+        <v>3.2</v>
+      </c>
+      <c r="B11515" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11515" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="11516" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11516" s="3">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B11516" s="7"/>
+      <c r="C11516" s="2"/>
+    </row>
+    <row r="11517" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11517" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="B11517" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11517" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11518" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11518" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11518" s="9"/>
+      <c r="C11518" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="125">
-    <mergeCell ref="B11153:C11153"/>
-    <mergeCell ref="B10740:C10740"/>
+  <mergeCells count="127">
+    <mergeCell ref="B11212:C11212"/>
+    <mergeCell ref="B9560:C9560"/>
+    <mergeCell ref="B11389:C11389"/>
     <mergeCell ref="B10799:C10799"/>
-    <mergeCell ref="B10816:B10817"/>
-    <mergeCell ref="B10868:B10869"/>
-    <mergeCell ref="B10917:C10917"/>
-    <mergeCell ref="B10209:C10209"/>
-    <mergeCell ref="B10386:C10386"/>
-    <mergeCell ref="B10504:C10504"/>
+    <mergeCell ref="B10858:C10858"/>
+    <mergeCell ref="B10875:B10876"/>
+    <mergeCell ref="B10927:B10928"/>
+    <mergeCell ref="B10976:C10976"/>
+    <mergeCell ref="B10268:C10268"/>
+    <mergeCell ref="B10445:C10445"/>
     <mergeCell ref="B10563:C10563"/>
     <mergeCell ref="B10622:C10622"/>
     <mergeCell ref="B10681:C10681"/>
-    <mergeCell ref="B10691:B10692"/>
-    <mergeCell ref="B9747:B9748"/>
-    <mergeCell ref="B9737:C9737"/>
-    <mergeCell ref="B9855:C9855"/>
-    <mergeCell ref="B9973:C9973"/>
+    <mergeCell ref="B10740:C10740"/>
+    <mergeCell ref="B10750:B10751"/>
+    <mergeCell ref="B9806:B9807"/>
+    <mergeCell ref="B9796:C9796"/>
+    <mergeCell ref="B9914:C9914"/>
     <mergeCell ref="B10032:C10032"/>
+    <mergeCell ref="B10091:C10091"/>
     <mergeCell ref="B9098:B9099"/>
     <mergeCell ref="B9147:C9147"/>
     <mergeCell ref="B8921:B8922"/>

</xml_diff>